<commit_message>
built some scenario input files
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229FFDA1-3331-4511-8F39-78EE870C31CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A1E0DA-C7BB-4CD5-805C-A5F35B6BEF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
+    <sheet name="S2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="36">
   <si>
     <t>Tech</t>
   </si>
@@ -129,6 +130,21 @@
   </si>
   <si>
     <t>2025 source</t>
+  </si>
+  <si>
+    <t>R&amp;D Impact</t>
+  </si>
+  <si>
+    <t>Pilot &amp; Demonstrations Impact</t>
+  </si>
+  <si>
+    <t>Reduction in costs</t>
+  </si>
+  <si>
+    <t>Hubs</t>
+  </si>
+  <si>
+    <t>Number of years of acceleration for cost decreases</t>
   </si>
 </sst>
 </file>
@@ -187,12 +203,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -658,11 +675,11 @@
         <v>2030</v>
       </c>
       <c r="B3">
-        <f>B$13*EXP(B$14*($A3-$A$2))</f>
+        <f t="shared" ref="B3:C6" si="0">B$13*EXP(B$14*($A3-$A$2))</f>
         <v>380.16957864810638</v>
       </c>
       <c r="C3">
-        <f>C$13*EXP(C$14*($A3-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>178.15121510639958</v>
       </c>
       <c r="D3">
@@ -676,19 +693,19 @@
         <v>212</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G7" si="0">F3/6.1/1000*44/12</f>
+        <f t="shared" ref="G3:G7" si="1">F3/6.1/1000*44/12</f>
         <v>0.12743169398907103</v>
       </c>
       <c r="I3">
-        <f>I$13*EXP(I$14*($A3-$A$2))</f>
+        <f t="shared" ref="I3:K6" si="2">I$13*EXP(I$14*($A3-$A$2))</f>
         <v>20.149627171231938</v>
       </c>
       <c r="J3">
-        <f>J$13*EXP(J$14*($A3-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>27.801038275533536</v>
       </c>
       <c r="K3">
-        <f>K$13*EXP(K$14*($A3-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>34.63261353326736</v>
       </c>
     </row>
@@ -697,11 +714,11 @@
         <v>2035</v>
       </c>
       <c r="B4">
-        <f>B$13*EXP(B$14*($A4-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>324.05584872080431</v>
       </c>
       <c r="C4">
-        <f>C$13*EXP(C$14*($A4-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>151.85576767409884</v>
       </c>
       <c r="D4">
@@ -717,19 +734,19 @@
         <v>193.72413793103445</v>
       </c>
       <c r="G4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1164462031279442</v>
       </c>
       <c r="I4">
-        <f>I$13*EXP(I$14*($A4-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>30.074627788122108</v>
       </c>
       <c r="J4">
-        <f>J$13*EXP(J$14*($A4-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>57.251683644272632</v>
       </c>
       <c r="K4">
-        <f>K$13*EXP(K$14*($A4-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>88.845771862566906</v>
       </c>
     </row>
@@ -738,11 +755,11 @@
         <v>2040</v>
       </c>
       <c r="B5">
-        <f>B$13*EXP(B$14*($A5-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>276.22460866960239</v>
       </c>
       <c r="C5">
-        <f>C$13*EXP(C$14*($A5-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>129.4415767084011</v>
       </c>
       <c r="D5">
@@ -758,19 +775,19 @@
         <v>177.02378121284181</v>
       </c>
       <c r="G5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.10640773734105245</v>
       </c>
       <c r="I5">
-        <f>I$13*EXP(I$14*($A5-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>44.888336092165353</v>
       </c>
       <c r="J5">
-        <f>J$13*EXP(J$14*($A5-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>117.90046283949337</v>
       </c>
       <c r="K5">
-        <f>K$13*EXP(K$14*($A5-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>227.9230578504532</v>
       </c>
     </row>
@@ -779,11 +796,11 @@
         <v>2045</v>
       </c>
       <c r="B6">
-        <f>B$13*EXP(B$14*($A6-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>235.45334773578654</v>
       </c>
       <c r="C6">
-        <f>C$13*EXP(C$14*($A6-$A$2))</f>
+        <f t="shared" si="0"/>
         <v>110.33576160712865</v>
       </c>
       <c r="D6">
@@ -799,19 +816,19 @@
         <v>161.7631104186313</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.7234656535789318E-2</v>
       </c>
       <c r="I6">
-        <f>I$13*EXP(I$14*($A6-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>66.998758266228606</v>
       </c>
       <c r="J6">
-        <f>J$13*EXP(J$14*($A6-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>242.79668741510181</v>
       </c>
       <c r="K6">
-        <f>K$13*EXP(K$14*($A6-$A$2))</f>
+        <f t="shared" si="2"/>
         <v>584.70897613742852</v>
       </c>
     </row>
@@ -838,7 +855,7 @@
         <v>147.8180146928872</v>
       </c>
       <c r="G7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8.8852358558566089E-2</v>
       </c>
       <c r="I7">
@@ -966,23 +983,23 @@
         <v>264.99999999999994</v>
       </c>
       <c r="E13">
-        <f t="shared" ref="D13:F13" si="1">EXP(LN(E2)-E14*0)</f>
+        <f t="shared" ref="E13:F13" si="3">EXP(LN(E2)-E14*0)</f>
         <v>139.99999999999994</v>
       </c>
       <c r="F13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>231.99999999999997</v>
       </c>
       <c r="I13">
-        <f t="shared" ref="I13" si="2">EXP(LN(I2)-I14*0)</f>
+        <f t="shared" ref="I13" si="4">EXP(LN(I2)-I14*0)</f>
         <v>13.5</v>
       </c>
       <c r="J13">
-        <f t="shared" ref="J13" si="3">EXP(LN(J2)-J14*0)</f>
+        <f t="shared" ref="J13" si="5">EXP(LN(J2)-J14*0)</f>
         <v>13.5</v>
       </c>
       <c r="K13">
-        <f t="shared" ref="K13" si="4">EXP(LN(K2)-K14*0)</f>
+        <f t="shared" ref="K13" si="6">EXP(LN(K2)-K14*0)</f>
         <v>13.5</v>
       </c>
     </row>
@@ -1015,11 +1032,11 @@
         <v>8.0099220021748324E-2</v>
       </c>
       <c r="J14">
-        <f t="shared" ref="J14:K14" si="5">(LN(J2)-LN(J7))/($A2-$A7)</f>
+        <f t="shared" ref="J14:K14" si="7">(LN(J2)-LN(J7))/($A2-$A7)</f>
         <v>0.1444767365191123</v>
       </c>
       <c r="K14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.18842122806583672</v>
       </c>
     </row>
@@ -1107,4 +1124,717 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23D47325-8713-4C29-9B32-6AF71A8D6F7B}">
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2">
+        <f>(1-B14)*(1-B22)*B$10*EXP(B$11*($A2-$A$2+B30))</f>
+        <v>301.2481276002236</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:F2" si="0">(1-C14)*(1-C22)*C$10*EXP(C$11*($A2-$A$2+C30))</f>
+        <v>141.16784454808683</v>
+      </c>
+      <c r="D2">
+        <f t="shared" si="0"/>
+        <v>190.79999999999998</v>
+      </c>
+      <c r="E2">
+        <f t="shared" si="0"/>
+        <v>100.79999999999997</v>
+      </c>
+      <c r="F2">
+        <f t="shared" si="0"/>
+        <v>167.04</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2030</v>
+      </c>
+      <c r="B3">
+        <f t="shared" ref="B3:F7" si="1">(1-B15)*(1-B23)*B$10*EXP(B$11*($A3-$A$2+B31))</f>
+        <v>256.78334918903136</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="1"/>
+        <v>120.33121071862676</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="1"/>
+        <v>159.98701142068063</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="1"/>
+        <v>90.792618901746735</v>
+      </c>
+      <c r="F3">
+        <f t="shared" si="1"/>
+        <v>152.63999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2035</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="1"/>
+        <v>218.88165395749689</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="1"/>
+        <v>102.57010241506018</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="1"/>
+        <v>134.15012486017295</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>81.778766339660933</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>139.48137931034481</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2040</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="1"/>
+        <v>186.57431874175384</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="1"/>
+        <v>87.43056640588911</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
+        <v>112.48573143653158</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>73.659805223530071</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>127.45712247324612</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2045</v>
+      </c>
+      <c r="B6">
+        <f t="shared" si="1"/>
+        <v>159.03560570091938</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="1"/>
+        <v>74.52565379258327</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="1"/>
+        <v>94.319999999999965</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>66.346891111476808</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>116.46943950141454</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2050</v>
+      </c>
+      <c r="B7">
+        <f t="shared" si="1"/>
+        <v>135.56165742010066</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="1"/>
+        <v>63.525530046639084</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="1"/>
+        <v>79.087918853242101</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>59.760000000000026</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>106.42897057887879</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <f>'Baseline Parameters'!B13</f>
+        <v>446.00000000000006</v>
+      </c>
+      <c r="C10">
+        <f>'Baseline Parameters'!C13</f>
+        <v>208.99999999999997</v>
+      </c>
+      <c r="D10">
+        <f>'Baseline Parameters'!D13</f>
+        <v>264.99999999999994</v>
+      </c>
+      <c r="E10">
+        <f>'Baseline Parameters'!E13</f>
+        <v>139.99999999999994</v>
+      </c>
+      <c r="F10">
+        <f>'Baseline Parameters'!F13</f>
+        <v>231.99999999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <f>'Baseline Parameters'!B14</f>
+        <v>-3.1940307848710853E-2</v>
+      </c>
+      <c r="C11">
+        <f>'Baseline Parameters'!C14</f>
+        <v>-3.1940307848710853E-2</v>
+      </c>
+      <c r="D11">
+        <f>'Baseline Parameters'!D14</f>
+        <v>-3.5226625139253544E-2</v>
+      </c>
+      <c r="E11">
+        <f>'Baseline Parameters'!E14</f>
+        <v>-2.0912072592508223E-2</v>
+      </c>
+      <c r="F11">
+        <f>'Baseline Parameters'!F14</f>
+        <v>-1.8030219398859515E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2025</v>
+      </c>
+      <c r="B14" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2030</v>
+      </c>
+      <c r="B15" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2035</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2040</v>
+      </c>
+      <c r="B17" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2045</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2050</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2025</v>
+      </c>
+      <c r="B22" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="G22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2030</v>
+      </c>
+      <c r="B23" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="F23" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="G23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2035</v>
+      </c>
+      <c r="B24" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="G24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2040</v>
+      </c>
+      <c r="B25" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="G25" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2045</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="G26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2050</v>
+      </c>
+      <c r="B27" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="C27" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="F27" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="G27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
+        <v>2</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>28</v>
+      </c>
+      <c r="G29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>2025</v>
+      </c>
+      <c r="B30" s="5">
+        <v>2</v>
+      </c>
+      <c r="C30" s="5">
+        <v>2</v>
+      </c>
+      <c r="D30" s="5">
+        <v>0</v>
+      </c>
+      <c r="E30" s="5">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5">
+        <v>0</v>
+      </c>
+      <c r="G30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>2030</v>
+      </c>
+      <c r="B31" s="5">
+        <v>2</v>
+      </c>
+      <c r="C31" s="5">
+        <v>2</v>
+      </c>
+      <c r="D31" s="5">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5">
+        <v>0</v>
+      </c>
+      <c r="G31" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>2035</v>
+      </c>
+      <c r="B32" s="5">
+        <v>2</v>
+      </c>
+      <c r="C32" s="5">
+        <v>2</v>
+      </c>
+      <c r="D32" s="5">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0</v>
+      </c>
+      <c r="G32" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>2040</v>
+      </c>
+      <c r="B33" s="5">
+        <v>2</v>
+      </c>
+      <c r="C33" s="5">
+        <v>2</v>
+      </c>
+      <c r="D33" s="5">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5">
+        <v>0</v>
+      </c>
+      <c r="F33" s="5">
+        <v>0</v>
+      </c>
+      <c r="G33" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>2045</v>
+      </c>
+      <c r="B34" s="5">
+        <v>2</v>
+      </c>
+      <c r="C34" s="5">
+        <v>2</v>
+      </c>
+      <c r="D34" s="5">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5">
+        <v>0</v>
+      </c>
+      <c r="F34" s="5">
+        <v>0</v>
+      </c>
+      <c r="G34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>2050</v>
+      </c>
+      <c r="B35" s="5">
+        <v>2</v>
+      </c>
+      <c r="C35" s="5">
+        <v>2</v>
+      </c>
+      <c r="D35" s="5">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5">
+        <v>0</v>
+      </c>
+      <c r="F35" s="5">
+        <v>0</v>
+      </c>
+      <c r="G35" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
7 new scenarios: excess; separating itc from procurement
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54F64265-0CEC-4CE5-AED3-93C03D151F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DC7337-26BC-47E3-8F6B-2B4E98E87F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="345" yWindow="495" windowWidth="16710" windowHeight="13710" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="37">
   <si>
     <t>Tech</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Number of years of acceleration for cost decreases</t>
+  </si>
+  <si>
+    <t>Very High</t>
   </si>
 </sst>
 </file>
@@ -3322,7 +3325,7 @@
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3353,8 +3356,11 @@
       <c r="K1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -3387,8 +3393,11 @@
       <c r="K2">
         <v>13.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2030</v>
       </c>
@@ -3415,7 +3424,7 @@
         <v>0.12743169398907103</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:K6" si="2">I$13*EXP(I$14*($A3-$A$2))</f>
+        <f t="shared" ref="I3:L6" si="2">I$13*EXP(I$14*($A3-$A$2))</f>
         <v>20.149627171231938</v>
       </c>
       <c r="J3">
@@ -3426,8 +3435,12 @@
         <f t="shared" si="2"/>
         <v>34.63261353326736</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <f t="shared" si="2"/>
+        <v>38.046022739216987</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2035</v>
       </c>
@@ -3467,8 +3480,12 @@
         <f t="shared" si="2"/>
         <v>88.845771862566906</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <f t="shared" si="2"/>
+        <v>107.22221083503824</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2040</v>
       </c>
@@ -3508,8 +3525,12 @@
         <f t="shared" si="2"/>
         <v>227.9230578504532</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <f t="shared" si="2"/>
+        <v>302.17619789473957</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2045</v>
       </c>
@@ -3549,8 +3570,12 @@
         <f t="shared" si="2"/>
         <v>584.70897613742852</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <f t="shared" si="2"/>
+        <v>851.60018491506594</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2050</v>
       </c>
@@ -3585,8 +3610,11 @@
       <c r="K7">
         <v>1500</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -3614,8 +3642,11 @@
       <c r="K8" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -3635,7 +3666,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -3652,7 +3683,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -3684,7 +3715,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -3717,11 +3748,15 @@
         <v>13.5</v>
       </c>
       <c r="K13">
-        <f t="shared" ref="K13" si="6">EXP(LN(K2)-K14*0)</f>
+        <f t="shared" ref="K13:L13" si="6">EXP(LN(K2)-K14*0)</f>
         <v>13.5</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <f t="shared" si="6"/>
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -3756,6 +3791,10 @@
       <c r="K14">
         <f t="shared" si="7"/>
         <v>0.18842122806583672</v>
+      </c>
+      <c r="L14">
+        <f t="shared" ref="L14" si="8">(LN(L2)-LN(L7))/($A2-$A7)</f>
+        <v>0.20722137323566614</v>
       </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
config files for verify 2025 scenario
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DC7337-26BC-47E3-8F6B-2B4E98E87F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72670DB3-492D-4E4A-9735-0B2F85F86583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="495" windowWidth="16710" windowHeight="13710" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="S2" sheetId="2" r:id="rId2"/>
+    <sheet name="verify-2025" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="37">
   <si>
     <t>Tech</t>
   </si>
@@ -4595,4 +4596,557 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16D7DDB-ECAA-4988-BB02-23E7116C40BF}">
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2">
+        <v>446</v>
+      </c>
+      <c r="C2">
+        <v>209</v>
+      </c>
+      <c r="D2">
+        <f>D$13*EXP(D$14*($A2-$A$3))</f>
+        <v>316.03815554156989</v>
+      </c>
+      <c r="E2">
+        <v>140</v>
+      </c>
+      <c r="F2">
+        <v>169</v>
+      </c>
+      <c r="G2">
+        <f>F2/6.1/1000*44/12</f>
+        <v>0.10158469945355192</v>
+      </c>
+      <c r="I2">
+        <v>13.5</v>
+      </c>
+      <c r="J2">
+        <v>13.5</v>
+      </c>
+      <c r="K2">
+        <v>13.5</v>
+      </c>
+      <c r="L2">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2030</v>
+      </c>
+      <c r="B3">
+        <f t="shared" ref="B3:C6" si="0">B$13*EXP(B$14*($A3-$A$2))</f>
+        <v>380.16957864810638</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="0"/>
+        <v>178.15121510639958</v>
+      </c>
+      <c r="D3">
+        <v>265</v>
+      </c>
+      <c r="E3">
+        <f>E$13*EXP(E$14*($A3-$A$2))</f>
+        <v>126.10085958575935</v>
+      </c>
+      <c r="F3">
+        <v>153</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G7" si="1">F3/6.1/1000*44/12</f>
+        <v>9.1967213114754101E-2</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:L6" si="2">I$13*EXP(I$14*($A3-$A$2))</f>
+        <v>20.149627171231938</v>
+      </c>
+      <c r="J3">
+        <f t="shared" si="2"/>
+        <v>27.801038275533536</v>
+      </c>
+      <c r="K3">
+        <f t="shared" si="2"/>
+        <v>34.63261353326736</v>
+      </c>
+      <c r="L3">
+        <f t="shared" si="2"/>
+        <v>38.046022739216987</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2035</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>324.05584872080431</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>151.85576767409884</v>
+      </c>
+      <c r="D4">
+        <f>D$13*EXP(D$14*($A4-$A$3))</f>
+        <v>222.20418252872307</v>
+      </c>
+      <c r="E4">
+        <f>E$13*EXP(E$14*($A4-$A$2))</f>
+        <v>113.58161991619573</v>
+      </c>
+      <c r="F4">
+        <f>F$13*EXP(F$14*($A4-$A$2))</f>
+        <v>138.51479289940823</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="1"/>
+        <v>8.3260258026966696E-2</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="2"/>
+        <v>30.074627788122108</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="2"/>
+        <v>57.251683644272632</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="2"/>
+        <v>88.845771862566906</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="2"/>
+        <v>107.22221083503824</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2040</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>276.22460866960239</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>129.4415767084011</v>
+      </c>
+      <c r="D5">
+        <f>D$13*EXP(D$14*($A5-$A$3))</f>
+        <v>186.3196178613513</v>
+      </c>
+      <c r="E5">
+        <f>E$13*EXP(E$14*($A5-$A$2))</f>
+        <v>102.30528503268064</v>
+      </c>
+      <c r="F5">
+        <f>F$13*EXP(F$14*($A5-$A$2))</f>
+        <v>125.40096635271868</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>7.5377630048082275E-2</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="2"/>
+        <v>44.888336092165353</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="2"/>
+        <v>117.90046283949337</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="2"/>
+        <v>227.9230578504532</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="2"/>
+        <v>302.17619789473957</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2045</v>
+      </c>
+      <c r="B6">
+        <f t="shared" si="0"/>
+        <v>235.45334773578654</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>110.33576160712865</v>
+      </c>
+      <c r="D6">
+        <f>D$13*EXP(D$14*($A6-$A$3))</f>
+        <v>156.23018255073828</v>
+      </c>
+      <c r="E6">
+        <f>E$13*EXP(E$14*($A6-$A$2))</f>
+        <v>92.14845987705111</v>
+      </c>
+      <c r="F6">
+        <f>F$13*EXP(F$14*($A6-$A$2))</f>
+        <v>113.52868551459144</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="1"/>
+        <v>6.8241286374891033E-2</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="2"/>
+        <v>66.998758266228606</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="2"/>
+        <v>242.79668741510181</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="2"/>
+        <v>584.70897613742852</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="2"/>
+        <v>851.60018491506594</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2050</v>
+      </c>
+      <c r="B7">
+        <f>B2*B17</f>
+        <v>200.70000000000002</v>
+      </c>
+      <c r="C7">
+        <f>C2*C17</f>
+        <v>94.05</v>
+      </c>
+      <c r="D7">
+        <v>131</v>
+      </c>
+      <c r="E7">
+        <v>83</v>
+      </c>
+      <c r="F7">
+        <f>F$13*EXP(F$14*($A7-$A$2))</f>
+        <v>102.78040759605021</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>6.1780572871942753E-2</v>
+      </c>
+      <c r="I7">
+        <v>100</v>
+      </c>
+      <c r="J7">
+        <v>500</v>
+      </c>
+      <c r="K7">
+        <v>1500</v>
+      </c>
+      <c r="L7">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9">
+        <v>432</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" t="s">
+        <v>29</v>
+      </c>
+      <c r="J11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <f>EXP(LN(B2)-B14*0)</f>
+        <v>446.00000000000006</v>
+      </c>
+      <c r="C13">
+        <f>EXP(LN(C2)-C14*0)</f>
+        <v>208.99999999999997</v>
+      </c>
+      <c r="D13">
+        <f>EXP(LN(D3)-D14*0)</f>
+        <v>264.99999999999994</v>
+      </c>
+      <c r="E13">
+        <f t="shared" ref="E13:F13" si="3">EXP(LN(E2)-E14*0)</f>
+        <v>139.99999999999994</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="3"/>
+        <v>169</v>
+      </c>
+      <c r="I13">
+        <f t="shared" ref="I13:L13" si="4">EXP(LN(I2)-I14*0)</f>
+        <v>13.5</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="4"/>
+        <v>13.5</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="4"/>
+        <v>13.5</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="4"/>
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <f>(LN(B2)-LN(B7))/($A2-$A7)</f>
+        <v>-3.1940307848710853E-2</v>
+      </c>
+      <c r="C14">
+        <f>(LN(C2)-LN(C7))/($A2-$A7)</f>
+        <v>-3.1940307848710853E-2</v>
+      </c>
+      <c r="D14">
+        <f>(LN(D3)-LN(D7))/($A3-$A7)</f>
+        <v>-3.5226625139253544E-2</v>
+      </c>
+      <c r="E14">
+        <f>(LN(E2)-LN(E7))/($A2-$A7)</f>
+        <v>-2.0912072592508223E-2</v>
+      </c>
+      <c r="F14">
+        <f>(LN(F2)-LN(F3))/($A2-$A3)</f>
+        <v>-1.9892158706127639E-2</v>
+      </c>
+      <c r="I14">
+        <f>(LN(I2)-LN(I7))/($A2-$A7)</f>
+        <v>8.0099220021748324E-2</v>
+      </c>
+      <c r="J14">
+        <f t="shared" ref="J14:L14" si="5">(LN(J2)-LN(J7))/($A2-$A7)</f>
+        <v>0.1444767365191123</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="5"/>
+        <v>0.18842122806583672</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="5"/>
+        <v>0.20722137323566614</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="1">
+        <v>0.45</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.45</v>
+      </c>
+      <c r="H17" t="s">
+        <v>30</v>
+      </c>
+      <c r="I17" t="s">
+        <v>4</v>
+      </c>
+      <c r="J17" t="s">
+        <v>4</v>
+      </c>
+      <c r="K17" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18">
+        <v>25</v>
+      </c>
+      <c r="C18">
+        <v>25</v>
+      </c>
+      <c r="H18" t="s">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>42</v>
+      </c>
+      <c r="J18">
+        <v>42</v>
+      </c>
+      <c r="K18">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20">
+        <v>44</v>
+      </c>
+      <c r="C20">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F8" r:id="rId1" display="https://info.opisnet.com/hubfs/CDR Price Survey White Paper-Email.pdf" xr:uid="{A8AC4E09-B357-43EA-99AB-751470BD001F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
TEW cost curves update
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72670DB3-492D-4E4A-9735-0B2F85F86583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E875FED6-3C51-46D0-80AA-5D657876D744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="40">
   <si>
     <t>Tech</t>
   </si>
@@ -149,6 +149,15 @@
   </si>
   <si>
     <t>Very High</t>
+  </si>
+  <si>
+    <t>Illinois 2030 and 2050 from Figure 5c less costs (TEW worksheet)</t>
+  </si>
+  <si>
+    <t>TEW (Nature Paper)</t>
+  </si>
+  <si>
+    <t>TEW (Ours) - less input costs</t>
   </si>
 </sst>
 </file>
@@ -499,7 +508,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TEW</c:v>
+                  <c:v>TEW (Nature Paper)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -582,7 +591,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Baseline Parameters'!$E$1</c:f>
+              <c:f>'Baseline Parameters'!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -632,7 +641,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Baseline Parameters'!$E$2:$E$7</c:f>
+              <c:f>'Baseline Parameters'!$F$2:$F$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -669,7 +678,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Baseline Parameters'!$F$1</c:f>
+              <c:f>'Baseline Parameters'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -719,7 +728,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Baseline Parameters'!$F$2:$F$7</c:f>
+              <c:f>'Baseline Parameters'!$G$2:$G$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1077,8 +1086,8 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
+          <c:idx val="1"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
               <c:f>'S2'!$B$1</c:f>
@@ -1086,93 +1095,6 @@
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>DAC (sorbent)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>2025</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2030</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2035</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2040</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2045</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2050</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'S2'!$B$2:$B$7</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>446.00000000000006</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>323.85932014785305</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>231.91484742105459</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>186.57431874175384</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>159.03560570091938</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>135.56165742010066</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F4B6-4FC6-913E-28DF2E67F4D4}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'S2'!$C$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>DAC (solvent)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1218,27 +1140,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$C$2:$C$7</c:f>
+              <c:f>'S2'!$B$2:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>208.99999999999997</c:v>
+                  <c:v>446.00000000000006</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>151.76367244596696</c:v>
+                  <c:v>323.85932014785305</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>108.67758545067353</c:v>
+                  <c:v>231.91484742105459</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>87.43056640588911</c:v>
+                  <c:v>186.57431874175384</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>74.52565379258327</c:v>
+                  <c:v>159.03560570091938</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>63.525530046639084</c:v>
+                  <c:v>135.56165742010066</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1255,11 +1177,11 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$D$1</c:f>
+              <c:f>'S2'!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TEW</c:v>
+                  <c:v>DAC (solvent)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1305,27 +1227,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$D$2:$D$7</c:f>
+              <c:f>'S2'!$C$2:$C$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>316.03815554156989</c:v>
+                  <c:v>208.99999999999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>230.55794999999995</c:v>
+                  <c:v>151.76367244596696</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>165.92430717784811</c:v>
+                  <c:v>108.67758545067353</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>134.15012486017295</c:v>
+                  <c:v>87.43056640588911</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>112.48573143653158</c:v>
+                  <c:v>74.52565379258327</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>94.319999999999965</c:v>
+                  <c:v>63.525530046639084</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1342,11 +1264,11 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$E$1</c:f>
+              <c:f>'S2'!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>OEW</c:v>
+                  <c:v>TEW (Nature Paper)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1392,27 +1314,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$E$2:$E$7</c:f>
+              <c:f>'S2'!$D$2:$D$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>139.99999999999994</c:v>
+                  <c:v>316.03815554156989</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>109.7115308653982</c:v>
+                  <c:v>230.55794999999995</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>84.813667223821682</c:v>
+                  <c:v>165.92430717784811</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>73.659805223530071</c:v>
+                  <c:v>134.15012486017295</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>66.346891111476808</c:v>
+                  <c:v>112.48573143653158</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>59.760000000000026</c:v>
+                  <c:v>94.319999999999965</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1429,11 +1351,11 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$F$1</c:f>
+              <c:f>'S2'!$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>BECCS</c:v>
+                  <c:v>TEW (Ours) - less input costs</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1479,27 +1401,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$F$2:$F$7</c:f>
+              <c:f>'S2'!$E$2:$E$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>231.99999999999997</c:v>
+                  <c:v>269.98072031209182</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>184.44635999999997</c:v>
+                  <c:v>180.92669318181808</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>144.65768827586206</c:v>
+                  <c:v>119.608451259473</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>127.45712247324612</c:v>
+                  <c:v>88.832573878156737</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>116.46943950141454</c:v>
+                  <c:v>68.423913755896564</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>106.42897057887879</c:v>
+                  <c:v>52.703999999999972</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1508,6 +1430,182 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-F4B6-4FC6-913E-28DF2E67F4D4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'S2'!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>OEW</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'S2'!$F$2:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>139.99999999999994</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>109.7115308653982</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>84.813667223821682</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>73.659805223530071</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>66.346891111476808</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>59.760000000000026</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-688B-4E2A-921E-865D173543CD}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'S2'!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>BECCS</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'S2'!$G$2:$G$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>231.99999999999997</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>184.44635999999997</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>144.65768827586206</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>127.45712247324612</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>116.46943950141454</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>106.42897057887879</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-688B-4E2A-921E-865D173543CD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1522,6 +1620,117 @@
         <c:smooth val="0"/>
         <c:axId val="262440576"/>
         <c:axId val="262441536"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'S2'!$A$1</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>Tech</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:cat>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'S2'!$A$2:$A$7</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="6"/>
+                      <c:pt idx="0">
+                        <c:v>2025</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>2030</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>2035</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>2040</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>2045</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>2050</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'S2'!$A$2:$A$7</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="6"/>
+                      <c:pt idx="0">
+                        <c:v>2025</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>2030</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>2035</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>2040</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>2045</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>2050</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-F4B6-4FC6-913E-28DF2E67F4D4}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+          </c:ext>
+        </c:extLst>
       </c:lineChart>
       <c:catAx>
         <c:axId val="262440576"/>
@@ -2877,13 +3086,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>25</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>26</xdr:col>
       <xdr:colOff>485775</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -2925,13 +3134,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>128587</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>238125</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>14287</xdr:rowOff>
@@ -2966,13 +3175,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>195262</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>176212</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>500062</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>61912</xdr:rowOff>
@@ -3320,13 +3529,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{812C07AE-8A39-4CED-9C15-8283B0F8343C}">
-  <dimension ref="A1:Z24"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3337,31 +3546,34 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>28</v>
       </c>
       <c r="G1" t="s">
         <v>28</v>
       </c>
-      <c r="I1" t="s">
+      <c r="H1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>24</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -3376,17 +3588,18 @@
         <v>316.03815554156989</v>
       </c>
       <c r="E2">
+        <f>E$13*EXP(E$14*($A2-$A$3))</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="F2">
         <v>140</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>232</v>
       </c>
-      <c r="G2">
-        <f>F2/6.1/1000*44/12</f>
+      <c r="H2">
+        <f>G2/6.1/1000*44/12</f>
         <v>0.13945355191256831</v>
-      </c>
-      <c r="I2">
-        <v>13.5</v>
       </c>
       <c r="J2">
         <v>13.5</v>
@@ -3397,8 +3610,11 @@
       <c r="L2">
         <v>13.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2030</v>
       </c>
@@ -3414,34 +3630,38 @@
         <v>265</v>
       </c>
       <c r="E3">
-        <f>E$13*EXP(E$14*($A3-$A$2))</f>
+        <f>0.125*6.1*12/44*1000</f>
+        <v>207.95454545454541</v>
+      </c>
+      <c r="F3">
+        <f>F$13*EXP(F$14*($A3-$A$2))</f>
         <v>126.10085958575935</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>212</v>
       </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G7" si="1">F3/6.1/1000*44/12</f>
+      <c r="H3">
+        <f t="shared" ref="H3:H7" si="1">G3/6.1/1000*44/12</f>
         <v>0.12743169398907103</v>
       </c>
-      <c r="I3">
-        <f t="shared" ref="I3:L6" si="2">I$13*EXP(I$14*($A3-$A$2))</f>
+      <c r="J3">
+        <f t="shared" ref="J3:M6" si="2">J$13*EXP(J$14*($A3-$A$2))</f>
         <v>20.149627171231938</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <f t="shared" si="2"/>
         <v>27.801038275533536</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <f t="shared" si="2"/>
         <v>34.63261353326736</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <f t="shared" si="2"/>
         <v>38.046022739216987</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2035</v>
       </c>
@@ -3454,39 +3674,43 @@
         <v>151.85576767409884</v>
       </c>
       <c r="D4">
-        <f>D$13*EXP(D$14*($A4-$A$3))</f>
+        <f t="shared" ref="D4:E6" si="3">D$13*EXP(D$14*($A4-$A$3))</f>
         <v>222.20418252872307</v>
       </c>
       <c r="E4">
-        <f>E$13*EXP(E$14*($A4-$A$2))</f>
-        <v>113.58161991619573</v>
+        <f t="shared" si="3"/>
+        <v>160.17844876188263</v>
       </c>
       <c r="F4">
         <f>F$13*EXP(F$14*($A4-$A$2))</f>
+        <v>113.58161991619573</v>
+      </c>
+      <c r="G4">
+        <f>G$13*EXP(G$14*($A4-$A$2))</f>
         <v>193.72413793103445</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <f t="shared" si="1"/>
         <v>0.1164462031279442</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f t="shared" si="2"/>
         <v>30.074627788122108</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <f t="shared" si="2"/>
         <v>57.251683644272632</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <f t="shared" si="2"/>
         <v>88.845771862566906</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <f t="shared" si="2"/>
         <v>107.22221083503824</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2040</v>
       </c>
@@ -3499,39 +3723,43 @@
         <v>129.4415767084011</v>
       </c>
       <c r="D5">
-        <f>D$13*EXP(D$14*($A5-$A$3))</f>
+        <f t="shared" si="3"/>
         <v>186.3196178613513</v>
       </c>
       <c r="E5">
-        <f>E$13*EXP(E$14*($A5-$A$2))</f>
-        <v>102.30528503268064</v>
+        <f t="shared" si="3"/>
+        <v>123.37857483077323</v>
       </c>
       <c r="F5">
         <f>F$13*EXP(F$14*($A5-$A$2))</f>
+        <v>102.30528503268064</v>
+      </c>
+      <c r="G5">
+        <f>G$13*EXP(G$14*($A5-$A$2))</f>
         <v>177.02378121284181</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <f t="shared" si="1"/>
         <v>0.10640773734105245</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f t="shared" si="2"/>
         <v>44.888336092165353</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <f t="shared" si="2"/>
         <v>117.90046283949337</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <f t="shared" si="2"/>
         <v>227.9230578504532</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <f t="shared" si="2"/>
         <v>302.17619789473957</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2045</v>
       </c>
@@ -3544,39 +3772,43 @@
         <v>110.33576160712865</v>
       </c>
       <c r="D6">
-        <f>D$13*EXP(D$14*($A6-$A$3))</f>
+        <f t="shared" si="3"/>
         <v>156.23018255073828</v>
       </c>
       <c r="E6">
-        <f>E$13*EXP(E$14*($A6-$A$2))</f>
-        <v>92.14845987705111</v>
+        <f t="shared" si="3"/>
+        <v>95.033213549856328</v>
       </c>
       <c r="F6">
         <f>F$13*EXP(F$14*($A6-$A$2))</f>
+        <v>92.14845987705111</v>
+      </c>
+      <c r="G6">
+        <f>G$13*EXP(G$14*($A6-$A$2))</f>
         <v>161.7631104186313</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <f t="shared" si="1"/>
         <v>9.7234656535789318E-2</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f t="shared" si="2"/>
         <v>66.998758266228606</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <f t="shared" si="2"/>
         <v>242.79668741510181</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <f t="shared" si="2"/>
         <v>584.70897613742852</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <f t="shared" si="2"/>
         <v>851.60018491506594</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2050</v>
       </c>
@@ -3592,30 +3824,34 @@
         <v>131</v>
       </c>
       <c r="E7">
+        <f>0.044*6.1*12/44*1000</f>
+        <v>73.199999999999989</v>
+      </c>
+      <c r="F7">
         <v>83</v>
       </c>
-      <c r="F7">
-        <f>F$13*EXP(F$14*($A7-$A$2))</f>
+      <c r="G7">
+        <f>G$13*EXP(G$14*($A7-$A$2))</f>
         <v>147.8180146928872</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <f t="shared" si="1"/>
         <v>8.8852358558566089E-2</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>100</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>500</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>1500</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>2400</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -3625,17 +3861,17 @@
       <c r="C8" t="s">
         <v>6</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>25</v>
@@ -3646,8 +3882,11 @@
       <c r="L8" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -3661,13 +3900,16 @@
         <v>432</v>
       </c>
       <c r="E9">
+        <v>433</v>
+      </c>
+      <c r="F9">
         <v>8</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -3678,13 +3920,16 @@
         <v>16</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -3704,10 +3949,10 @@
         <v>26</v>
       </c>
       <c r="G11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" t="s">
         <v>27</v>
-      </c>
-      <c r="I11" t="s">
-        <v>29</v>
       </c>
       <c r="J11" t="s">
         <v>29</v>
@@ -3715,8 +3960,11 @@
       <c r="K11" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -3733,31 +3981,35 @@
         <v>264.99999999999994</v>
       </c>
       <c r="E13">
-        <f t="shared" ref="E13:F13" si="3">EXP(LN(E2)-E14*0)</f>
+        <f>EXP(LN(E3)-E14*0)</f>
+        <v>207.95454545454535</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13:G13" si="4">EXP(LN(F2)-F14*0)</f>
         <v>139.99999999999994</v>
       </c>
-      <c r="F13">
-        <f t="shared" si="3"/>
+      <c r="G13">
+        <f t="shared" si="4"/>
         <v>231.99999999999997</v>
-      </c>
-      <c r="I13">
-        <f t="shared" ref="I13" si="4">EXP(LN(I2)-I14*0)</f>
-        <v>13.5</v>
       </c>
       <c r="J13">
         <f t="shared" ref="J13" si="5">EXP(LN(J2)-J14*0)</f>
         <v>13.5</v>
       </c>
       <c r="K13">
-        <f t="shared" ref="K13:L13" si="6">EXP(LN(K2)-K14*0)</f>
+        <f t="shared" ref="K13" si="6">EXP(LN(K2)-K14*0)</f>
         <v>13.5</v>
       </c>
       <c r="L13">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="L13:M13" si="7">EXP(LN(L2)-L14*0)</f>
         <v>13.5</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13">
+        <f t="shared" si="7"/>
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -3774,31 +4026,35 @@
         <v>-3.5226625139253544E-2</v>
       </c>
       <c r="E14">
-        <f>(LN(E2)-LN(E7))/($A2-$A7)</f>
+        <f>(LN(E3)-LN(E7))/($A3-$A7)</f>
+        <v>-5.2206205169202005E-2</v>
+      </c>
+      <c r="F14">
+        <f>(LN(F2)-LN(F7))/($A2-$A7)</f>
         <v>-2.0912072592508223E-2</v>
       </c>
-      <c r="F14">
-        <f>(LN(F2)-LN(F3))/($A2-$A3)</f>
+      <c r="G14">
+        <f>(LN(G2)-LN(G3))/($A2-$A3)</f>
         <v>-1.8030219398859515E-2</v>
       </c>
-      <c r="I14">
-        <f>(LN(I2)-LN(I7))/($A2-$A7)</f>
+      <c r="J14">
+        <f>(LN(J2)-LN(J7))/($A2-$A7)</f>
         <v>8.0099220021748324E-2</v>
       </c>
-      <c r="J14">
-        <f t="shared" ref="J14:K14" si="7">(LN(J2)-LN(J7))/($A2-$A7)</f>
+      <c r="K14">
+        <f t="shared" ref="K14:L14" si="8">(LN(K2)-LN(K7))/($A2-$A7)</f>
         <v>0.1444767365191123</v>
       </c>
-      <c r="K14">
-        <f t="shared" si="7"/>
+      <c r="L14">
+        <f t="shared" si="8"/>
         <v>0.18842122806583672</v>
       </c>
-      <c r="L14">
-        <f t="shared" ref="L14" si="8">(LN(L2)-LN(L7))/($A2-$A7)</f>
+      <c r="M14">
+        <f t="shared" ref="M14" si="9">(LN(M2)-LN(M7))/($A2-$A7)</f>
         <v>0.20722137323566614</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -3808,11 +4064,9 @@
       <c r="C17" s="1">
         <v>0.45</v>
       </c>
-      <c r="H17" t="s">
+      <c r="D17" s="1"/>
+      <c r="I17" t="s">
         <v>30</v>
-      </c>
-      <c r="I17" t="s">
-        <v>4</v>
       </c>
       <c r="J17" t="s">
         <v>4</v>
@@ -3820,8 +4074,11 @@
       <c r="K17" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="L17" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -3831,11 +4088,8 @@
       <c r="C18">
         <v>25</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>1</v>
-      </c>
-      <c r="I18">
-        <v>42</v>
       </c>
       <c r="J18">
         <v>42</v>
@@ -3843,8 +4097,11 @@
       <c r="K18">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -3855,7 +4112,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -3866,30 +4123,32 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="T23" s="2"/>
-      <c r="Z23" s="1"/>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="T24" s="2"/>
-      <c r="Z24" s="1"/>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="U23" s="2"/>
+      <c r="AA23" s="1"/>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="U24" s="2"/>
+      <c r="AA24" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="F8" r:id="rId1" display="https://info.opisnet.com/hubfs/CDR Price Survey White Paper-Email.pdf" xr:uid="{CC158B7C-E4A0-48D9-9303-73D590522FCC}"/>
+    <hyperlink ref="G8" r:id="rId1" display="https://info.opisnet.com/hubfs/CDR Price Survey White Paper-Email.pdf" xr:uid="{CC158B7C-E4A0-48D9-9303-73D590522FCC}"/>
+    <hyperlink ref="D8" r:id="rId2" xr:uid="{EFC78798-2563-4766-9FAD-EF08B1A29709}"/>
+    <hyperlink ref="E8" r:id="rId3" xr:uid="{5DABCDEF-5B5D-4B35-9C6F-0E02DE3477A2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23D47325-8713-4C29-9B32-6AF71A8D6F7B}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3900,16 +4159,19 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -3918,7 +4180,7 @@
         <v>446.00000000000006</v>
       </c>
       <c r="C2">
-        <f t="shared" ref="C2:F2" si="0">(1-C14)*(1-C22)*C$10*EXP(C$11*($A2-$A$2+C30))</f>
+        <f t="shared" ref="C2:G2" si="0">(1-C14)*(1-C22)*C$10*EXP(C$11*($A2-$A$2+C30))</f>
         <v>208.99999999999997</v>
       </c>
       <c r="D2">
@@ -3926,20 +4188,24 @@
         <v>316.03815554156989</v>
       </c>
       <c r="E2">
+        <f>(1-E14)*(1-E22)*E$10*EXP(E$11*($A2-$A$3+E30))</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="F2">
         <f t="shared" si="0"/>
         <v>139.99999999999994</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f t="shared" si="0"/>
         <v>231.99999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2030</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:F7" si="1">(1-B15)*(1-B23)*B$10*EXP(B$11*($A3-$A$2+B31))</f>
+        <f t="shared" ref="B3:G7" si="1">(1-B15)*(1-B23)*B$10*EXP(B$11*($A3-$A$2+B31))</f>
         <v>323.85932014785305</v>
       </c>
       <c r="C3">
@@ -3947,19 +4213,23 @@
         <v>151.76367244596696</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D7" si="2">(1-D15)*(1-D23)*D$10*EXP(D$11*($A3-$A$3+D31))</f>
+        <f t="shared" ref="D3:E7" si="2">(1-D15)*(1-D23)*D$10*EXP(D$11*($A3-$A$3+D31))</f>
         <v>230.55794999999995</v>
       </c>
       <c r="E3">
+        <f t="shared" si="2"/>
+        <v>180.92669318181808</v>
+      </c>
+      <c r="F3">
         <f t="shared" si="1"/>
         <v>109.7115308653982</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f t="shared" si="1"/>
         <v>184.44635999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2035</v>
       </c>
@@ -3976,15 +4246,19 @@
         <v>165.92430717784811</v>
       </c>
       <c r="E4">
+        <f t="shared" si="2"/>
+        <v>119.608451259473</v>
+      </c>
+      <c r="F4">
         <f t="shared" si="1"/>
         <v>84.813667223821682</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f t="shared" si="1"/>
         <v>144.65768827586206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2040</v>
       </c>
@@ -4001,15 +4275,19 @@
         <v>134.15012486017295</v>
       </c>
       <c r="E5">
+        <f t="shared" si="2"/>
+        <v>88.832573878156737</v>
+      </c>
+      <c r="F5">
         <f t="shared" si="1"/>
         <v>73.659805223530071</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f t="shared" si="1"/>
         <v>127.45712247324612</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2045</v>
       </c>
@@ -4026,15 +4304,19 @@
         <v>112.48573143653158</v>
       </c>
       <c r="E6">
+        <f t="shared" si="2"/>
+        <v>68.423913755896564</v>
+      </c>
+      <c r="F6">
         <f t="shared" si="1"/>
         <v>66.346891111476808</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <f t="shared" si="1"/>
         <v>116.46943950141454</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2050</v>
       </c>
@@ -4051,15 +4333,19 @@
         <v>94.319999999999965</v>
       </c>
       <c r="E7">
+        <f t="shared" si="2"/>
+        <v>52.703999999999972</v>
+      </c>
+      <c r="F7">
         <f t="shared" si="1"/>
         <v>59.760000000000026</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <f t="shared" si="1"/>
         <v>106.42897057887879</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -4077,14 +4363,18 @@
       </c>
       <c r="E10">
         <f>'Baseline Parameters'!E13</f>
-        <v>139.99999999999994</v>
+        <v>207.95454545454535</v>
       </c>
       <c r="F10">
         <f>'Baseline Parameters'!F13</f>
+        <v>139.99999999999994</v>
+      </c>
+      <c r="G10">
+        <f>'Baseline Parameters'!G13</f>
         <v>231.99999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -4102,14 +4392,18 @@
       </c>
       <c r="E11">
         <f>'Baseline Parameters'!E14</f>
-        <v>-2.0912072592508223E-2</v>
+        <v>-5.2206205169202005E-2</v>
       </c>
       <c r="F11">
         <f>'Baseline Parameters'!F14</f>
+        <v>-2.0912072592508223E-2</v>
+      </c>
+      <c r="G11">
+        <f>'Baseline Parameters'!G14</f>
         <v>-1.8030219398859515E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4123,16 +4417,19 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
+        <v>2</v>
+      </c>
+      <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>28</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -4151,11 +4448,14 @@
       <c r="F14" s="6">
         <v>0</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2030</v>
       </c>
@@ -4174,11 +4474,14 @@
       <c r="F15" s="6">
         <v>3.3300000000000003E-2</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="6">
+        <v>3.3300000000000003E-2</v>
+      </c>
+      <c r="H15" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2035</v>
       </c>
@@ -4197,11 +4500,14 @@
       <c r="F16" s="6">
         <v>6.6600000000000006E-2</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="6">
+        <v>6.6600000000000006E-2</v>
+      </c>
+      <c r="H16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2040</v>
       </c>
@@ -4220,11 +4526,14 @@
       <c r="F17" s="6">
         <v>0.1</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="H17" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2045</v>
       </c>
@@ -4243,11 +4552,14 @@
       <c r="F18" s="6">
         <v>0.1</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="H18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2050</v>
       </c>
@@ -4266,11 +4578,14 @@
       <c r="F19" s="6">
         <v>0.1</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="H19" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -4284,16 +4599,19 @@
         <v>2</v>
       </c>
       <c r="E21" t="s">
+        <v>2</v>
+      </c>
+      <c r="F21" t="s">
         <v>3</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>28</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -4312,11 +4630,14 @@
       <c r="F22" s="1">
         <v>0</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="1">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2030</v>
       </c>
@@ -4335,11 +4656,14 @@
       <c r="F23" s="1">
         <v>0.1</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="H23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2035</v>
       </c>
@@ -4358,11 +4682,14 @@
       <c r="F24" s="1">
         <v>0.2</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="H24" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2040</v>
       </c>
@@ -4381,11 +4708,14 @@
       <c r="F25" s="1">
         <v>0.2</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="H25" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2045</v>
       </c>
@@ -4404,11 +4734,14 @@
       <c r="F26" s="1">
         <v>0.2</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="H26" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2050</v>
       </c>
@@ -4427,11 +4760,14 @@
       <c r="F27" s="1">
         <v>0.2</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="H27" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -4445,16 +4781,19 @@
         <v>2</v>
       </c>
       <c r="E29" t="s">
+        <v>2</v>
+      </c>
+      <c r="F29" t="s">
         <v>3</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>28</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2025</v>
       </c>
@@ -4473,11 +4812,14 @@
       <c r="F30" s="5">
         <v>0</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="5">
+        <v>0</v>
+      </c>
+      <c r="H30" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2030</v>
       </c>
@@ -4496,11 +4838,14 @@
       <c r="F31" s="5">
         <v>0</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="5">
+        <v>0</v>
+      </c>
+      <c r="H31" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2035</v>
       </c>
@@ -4519,11 +4864,14 @@
       <c r="F32" s="5">
         <v>0</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="5">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2040</v>
       </c>
@@ -4542,11 +4890,14 @@
       <c r="F33" s="5">
         <v>0</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="5">
+        <v>0</v>
+      </c>
+      <c r="H33" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2045</v>
       </c>
@@ -4565,11 +4916,14 @@
       <c r="F34" s="5">
         <v>0</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34" s="5">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2050</v>
       </c>
@@ -4588,7 +4942,10 @@
       <c r="F35" s="5">
         <v>0</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" s="5">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
higher BECCS minimum prices for 2025
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0828AEE4-0E6A-453E-8FCC-2A119ADB46F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F23EE365-3344-469C-8497-2FBE8A0737A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
@@ -5013,11 +5013,11 @@
         <v>140</v>
       </c>
       <c r="F2">
-        <v>169</v>
+        <v>301</v>
       </c>
       <c r="G2">
         <f>F2/6.1/1000*44/12</f>
-        <v>0.10158469945355192</v>
+        <v>0.18092896174863385</v>
       </c>
       <c r="I2">
         <v>13.5</v>
@@ -5052,11 +5052,11 @@
         <v>126.10085958575935</v>
       </c>
       <c r="F3">
-        <v>153</v>
+        <v>265</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G7" si="1">F3/6.1/1000*44/12</f>
-        <v>9.1967213114754101E-2</v>
+        <v>0.1592896174863388</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:L6" si="2">I$13*EXP(I$14*($A3-$A$2))</f>
@@ -5097,11 +5097,11 @@
       </c>
       <c r="F4">
         <f>F$13*EXP(F$14*($A4-$A$2))</f>
-        <v>138.51479289940823</v>
+        <v>233.30564784053155</v>
       </c>
       <c r="G4">
         <f t="shared" si="1"/>
-        <v>8.3260258026966696E-2</v>
+        <v>0.1402383675544179</v>
       </c>
       <c r="I4">
         <f t="shared" si="2"/>
@@ -5142,11 +5142,11 @@
       </c>
       <c r="F5">
         <f>F$13*EXP(F$14*($A5-$A$2))</f>
-        <v>125.40096635271868</v>
+        <v>205.40198231807599</v>
       </c>
       <c r="G5">
         <f t="shared" si="1"/>
-        <v>7.5377630048082275E-2</v>
+        <v>0.12346567243163038</v>
       </c>
       <c r="I5">
         <f t="shared" si="2"/>
@@ -5187,11 +5187,11 @@
       </c>
       <c r="F6">
         <f>F$13*EXP(F$14*($A6-$A$2))</f>
-        <v>113.52868551459144</v>
+        <v>180.83563227338919</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>6.8241286374891033E-2</v>
+        <v>0.1086990139348241</v>
       </c>
       <c r="I6">
         <f t="shared" si="2"/>
@@ -5230,11 +5230,11 @@
       </c>
       <c r="F7">
         <f>F$13*EXP(F$14*($A7-$A$2))</f>
-        <v>102.78040759605021</v>
+        <v>159.20745034035926</v>
       </c>
       <c r="G7">
         <f t="shared" si="1"/>
-        <v>6.1780572871942753E-2</v>
+        <v>9.5698467417702285E-2</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="F13">
         <f t="shared" si="3"/>
-        <v>169</v>
+        <v>300.99999999999989</v>
       </c>
       <c r="I13">
         <f t="shared" ref="I13:L13" si="4">EXP(LN(I2)-I14*0)</f>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="F14">
         <f>(LN(F2)-LN(F3))/($A2-$A3)</f>
-        <v>-1.9892158706127639E-2</v>
+        <v>-2.5476087752530675E-2</v>
       </c>
       <c r="I14">
         <f>(LN(I2)-LN(I7))/($A2-$A7)</f>

</xml_diff>

<commit_message>
no ghg tax in US in 2025
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F23EE365-3344-469C-8497-2FBE8A0737A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4214B55-6F12-40A0-A7D7-BDE587C32C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -4205,11 +4205,11 @@
         <v>2030</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:G7" si="1">(1-B15)*(1-B23)*B$10*EXP(B$11*($A3-$A$2+B31))</f>
+        <f>(1-B15)*(1-B23)*B$10*EXP(B$11*($A3-$A$2+B31))</f>
         <v>323.85932014785305</v>
       </c>
       <c r="C3">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B3:G7" si="1">(1-C15)*(1-C23)*C$10*EXP(C$11*($A3-$A$2+C31))</f>
         <v>151.76367244596696</v>
       </c>
       <c r="D3">

</xml_diff>

<commit_message>
3 config files for procurement scenarios
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4214B55-6F12-40A0-A7D7-BDE587C32C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DFE942-FD8F-4C7A-92D4-55032FF2D3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" activeTab="3" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="S2" sheetId="2" r:id="rId2"/>
     <sheet name="verify-2025" sheetId="3" r:id="rId3"/>
+    <sheet name="Procurement" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="55">
   <si>
     <t>Tech</t>
   </si>
@@ -158,6 +159,51 @@
   </si>
   <si>
     <t>TEW (Ours) - less input costs</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Scaling</t>
+  </si>
+  <si>
+    <t>3B</t>
+  </si>
+  <si>
+    <t>https://www.congress.gov/bill/118th-congress/senate-bill/3615/text</t>
+  </si>
+  <si>
+    <t>CDR (Mt)</t>
+  </si>
+  <si>
+    <t>Rhodium</t>
+  </si>
+  <si>
+    <t>CDR (USD)</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>3B (Million USD)</t>
+  </si>
+  <si>
+    <t>Rhodium (2024)</t>
+  </si>
+  <si>
+    <t>EFI (2022)</t>
+  </si>
+  <si>
+    <t>Rhodium (Million)</t>
+  </si>
+  <si>
+    <t>Low baseline scenario</t>
+  </si>
+  <si>
+    <t>Avg. Price CDR (Low scenario)</t>
+  </si>
+  <si>
+    <t>HIGH</t>
   </si>
 </sst>
 </file>
@@ -5506,4 +5552,486 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8195A587-BA09-4421-98D4-BDAFBA104359}">
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3">
+        <v>0.05</v>
+      </c>
+      <c r="C3">
+        <f>K3/$J3</f>
+        <v>9.1538218144439369</v>
+      </c>
+      <c r="D3">
+        <f>L3/$J3</f>
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <f>A3</f>
+        <v>2025</v>
+      </c>
+      <c r="J3">
+        <v>360.50516023732143</v>
+      </c>
+      <c r="K3">
+        <v>3300</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2030</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <f t="shared" ref="C4:C8" si="0">K4/$J4</f>
+        <v>11.117978504373452</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D8" si="1">L4/$J4</f>
+        <v>67.381687905293646</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:I8" si="2">A4</f>
+        <v>2030</v>
+      </c>
+      <c r="J4">
+        <v>296.81654796345282</v>
+      </c>
+      <c r="K4">
+        <v>3300</v>
+      </c>
+      <c r="L4">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2035</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>14.945046646834507</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
+        <v>158.50807049672963</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="2"/>
+        <v>2035</v>
+      </c>
+      <c r="J5">
+        <v>220.8089461332641</v>
+      </c>
+      <c r="K5">
+        <v>3300</v>
+      </c>
+      <c r="L5">
+        <f>(L4+L6)/2</f>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2040</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="1"/>
+        <v>246.90690563233255</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="2"/>
+        <v>2040</v>
+      </c>
+      <c r="J6">
+        <v>202.50547416626196</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2045</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="1"/>
+        <v>406.1713779405772</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="2"/>
+        <v>2045</v>
+      </c>
+      <c r="J7">
+        <v>184.65112037257458</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <f>(L6+L8)/2</f>
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2050</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="1"/>
+        <v>578.25596171173243</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="2"/>
+        <v>2050</v>
+      </c>
+      <c r="J8">
+        <v>172.93379856211703</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="J9" t="s">
+        <v>52</v>
+      </c>
+      <c r="K9" t="s">
+        <v>50</v>
+      </c>
+      <c r="L9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="I13" t="s">
+        <v>40</v>
+      </c>
+      <c r="J13" t="s">
+        <v>53</v>
+      </c>
+      <c r="K13" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2025</v>
+      </c>
+      <c r="B14">
+        <v>0.05</v>
+      </c>
+      <c r="C14">
+        <f>K14/$J14</f>
+        <v>9.1527704871198079</v>
+      </c>
+      <c r="D14">
+        <f>L14/$J14</f>
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <f>A14</f>
+        <v>2025</v>
+      </c>
+      <c r="J14">
+        <v>360.54656943970235</v>
+      </c>
+      <c r="K14">
+        <v>3300</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2030</v>
+      </c>
+      <c r="B15">
+        <v>5</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ref="C15:C19" si="3">K15/$J15</f>
+        <v>11.123317675046577</v>
+      </c>
+      <c r="D15">
+        <f t="shared" ref="D15:D19" si="4">L15/$J15</f>
+        <v>67.41404651543381</v>
+      </c>
+      <c r="I15">
+        <f t="shared" ref="I15:I19" si="5">A15</f>
+        <v>2030</v>
+      </c>
+      <c r="J15">
+        <v>296.67407660243612</v>
+      </c>
+      <c r="K15">
+        <v>3300</v>
+      </c>
+      <c r="L15">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2035</v>
+      </c>
+      <c r="B16">
+        <v>10</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="3"/>
+        <v>14.849857137390348</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="4"/>
+        <v>157.49848479050368</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="5"/>
+        <v>2035</v>
+      </c>
+      <c r="J16">
+        <v>222.22436010451264</v>
+      </c>
+      <c r="K16">
+        <v>3300</v>
+      </c>
+      <c r="L16">
+        <f>(L15+L17)/2</f>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2040</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="4"/>
+        <v>243.06758416564975</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="5"/>
+        <v>2040</v>
+      </c>
+      <c r="J17">
+        <v>205.70410559527826</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2045</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="4"/>
+        <v>380.4751980809001</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="5"/>
+        <v>2045</v>
+      </c>
+      <c r="J18">
+        <v>197.12191590489118</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <f>(L17+L19)/2</f>
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2050</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="4"/>
+        <v>474.18677475115379</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="5"/>
+        <v>2050</v>
+      </c>
+      <c r="J19">
+        <v>210.88736617017318</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="J20" t="s">
+        <v>52</v>
+      </c>
+      <c r="K20" t="s">
+        <v>50</v>
+      </c>
+      <c r="L20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
verification of cost trajectories
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6939F477-9163-4096-A2E0-A5F34D37CE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C271B9-6B57-49A1-928F-677B3088BB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" activeTab="3" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -3913,7 +3913,7 @@
       <c r="E8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -3946,7 +3946,7 @@
         <v>432</v>
       </c>
       <c r="E9">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="F9">
         <v>8</v>
@@ -4183,9 +4183,10 @@
     <hyperlink ref="G8" r:id="rId1" display="https://info.opisnet.com/hubfs/CDR Price Survey White Paper-Email.pdf" xr:uid="{CC158B7C-E4A0-48D9-9303-73D590522FCC}"/>
     <hyperlink ref="D8" r:id="rId2" xr:uid="{EFC78798-2563-4766-9FAD-EF08B1A29709}"/>
     <hyperlink ref="E8" r:id="rId3" xr:uid="{5DABCDEF-5B5D-4B35-9C6F-0E02DE3477A2}"/>
+    <hyperlink ref="F8" r:id="rId4" xr:uid="{EE1C265B-61F3-4F37-850F-40A9D6842C42}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update learning by research in cost curves
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C271B9-6B57-49A1-928F-677B3088BB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D725B470-7CB3-4F48-8777-63CEC138394C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
-    <sheet name="S2" sheetId="2" r:id="rId2"/>
-    <sheet name="verify-2025" sheetId="3" r:id="rId3"/>
-    <sheet name="Procurement" sheetId="4" r:id="rId4"/>
+    <sheet name="Learning Rates" sheetId="5" r:id="rId2"/>
+    <sheet name="S2" sheetId="2" r:id="rId3"/>
+    <sheet name="verify-2025" sheetId="3" r:id="rId4"/>
+    <sheet name="Procurement" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="95">
   <si>
     <t>Tech</t>
   </si>
@@ -204,16 +205,137 @@
   </si>
   <si>
     <t>HIGH</t>
+  </si>
+  <si>
+    <t>Learning by research rates</t>
+  </si>
+  <si>
+    <t>Comp</t>
+  </si>
+  <si>
+    <t>Offshore wind</t>
+  </si>
+  <si>
+    <t>thermal solar</t>
+  </si>
+  <si>
+    <t>wind power</t>
+  </si>
+  <si>
+    <t>waste to electricity</t>
+  </si>
+  <si>
+    <t>https://journals.sagepub.com/doi/pdf/10.5547/ISSN0195-6574-EJ-Vol28-No3-4</t>
+  </si>
+  <si>
+    <t>Learning by research (table 4 and 5)</t>
+  </si>
+  <si>
+    <t>R&amp;D to early market formation</t>
+  </si>
+  <si>
+    <t>Early market formation to full commercialization</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>10-44%</t>
+  </si>
+  <si>
+    <t>Wind</t>
+  </si>
+  <si>
+    <t>3-14%</t>
+  </si>
+  <si>
+    <t>Impacts of innovation on renewable energy technology cost reductions</t>
+  </si>
+  <si>
+    <t>4-5%</t>
+  </si>
+  <si>
+    <t>Solar</t>
+  </si>
+  <si>
+    <t>Table 3</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>elasticity</t>
+  </si>
+  <si>
+    <t>Elasticity</t>
+  </si>
+  <si>
+    <t>Public R&amp;D</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>After 100 $ 100 mil in investment</t>
+  </si>
+  <si>
+    <t>Learning Rate Verification</t>
+  </si>
+  <si>
+    <t>All CDR</t>
+  </si>
+  <si>
+    <t>DAC Sorbent</t>
+  </si>
+  <si>
+    <t>DAC Solvent</t>
+  </si>
+  <si>
+    <t>This Study</t>
+  </si>
+  <si>
+    <t>Learning Rate</t>
+  </si>
+  <si>
+    <t>Cumulative Public R&amp;D</t>
+  </si>
+  <si>
+    <t>Learning Elasticity</t>
+  </si>
+  <si>
+    <t>Alpha</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Testing Equations</t>
+  </si>
+  <si>
+    <t>Additional R&amp;D Spending (2025 Million USD)</t>
+  </si>
+  <si>
+    <t>Cumulative R&amp;D Spending (2025 Million USD)</t>
+  </si>
+  <si>
+    <t>Baseline Costs (2025USD/t CDR)</t>
+  </si>
+  <si>
+    <t>Updated Costs (2025USD/t CDR)</t>
+  </si>
+  <si>
+    <t>Cost Savings (2025USD/t CDR)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,13 +365,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -261,11 +412,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -273,10 +426,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4191,6 +4362,1677 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05431749-67AB-462A-BE29-983F9537704D}">
+  <dimension ref="A1:V48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" s="10">
+        <f>1-2^I3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="J2" s="10">
+        <f t="shared" ref="J2:N2" si="0">1-2^J3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="K2" s="10">
+        <f t="shared" si="0"/>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="L2" s="10">
+        <f t="shared" si="0"/>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="M2" s="10">
+        <f t="shared" si="0"/>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="N2" s="10">
+        <f t="shared" si="0"/>
+        <v>4.9999617125113915E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>-7.1999999999999995E-2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="J3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="K3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="L3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="M3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="N3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="B4" s="5">
+        <v>-7.8E-2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="I4" s="9">
+        <v>500</v>
+      </c>
+      <c r="J4" s="9">
+        <v>500</v>
+      </c>
+      <c r="K4" s="9">
+        <v>500</v>
+      </c>
+      <c r="L4" s="9">
+        <v>500</v>
+      </c>
+      <c r="M4" s="9">
+        <v>500</v>
+      </c>
+      <c r="N4" s="9">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="B5" s="5">
+        <v>-0.45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="P5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>0.437</v>
+      </c>
+      <c r="B6" s="5">
+        <v>-0.82899999999999996</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K6" t="s">
+        <v>82</v>
+      </c>
+      <c r="L6" t="s">
+        <v>2</v>
+      </c>
+      <c r="M6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N6" t="s">
+        <v>80</v>
+      </c>
+      <c r="P6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" t="s">
+        <v>81</v>
+      </c>
+      <c r="S6" t="s">
+        <v>82</v>
+      </c>
+      <c r="T6" t="s">
+        <v>2</v>
+      </c>
+      <c r="U6" t="s">
+        <v>3</v>
+      </c>
+      <c r="V6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H7" s="16">
+        <v>2025</v>
+      </c>
+      <c r="I7" s="12">
+        <v>100</v>
+      </c>
+      <c r="J7" s="12">
+        <v>0</v>
+      </c>
+      <c r="K7" s="12">
+        <v>100</v>
+      </c>
+      <c r="L7" s="12">
+        <v>600</v>
+      </c>
+      <c r="M7" s="12">
+        <v>100</v>
+      </c>
+      <c r="N7" s="12">
+        <v>400</v>
+      </c>
+      <c r="P7">
+        <v>2025</v>
+      </c>
+      <c r="Q7">
+        <f>I25/(I$4^I$3)</f>
+        <v>367.46143374277835</v>
+      </c>
+      <c r="R7">
+        <f t="shared" ref="R7:V12" si="1">J25/(J$4^J$3)</f>
+        <v>706.41292866068591</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="1"/>
+        <v>331.03206746655462</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="1"/>
+        <v>427.61854555512627</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="1"/>
+        <v>221.74396863788348</v>
+      </c>
+      <c r="V7">
+        <f t="shared" si="1"/>
+        <v>570.9988924675697</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" s="16">
+        <v>2030</v>
+      </c>
+      <c r="I8" s="12">
+        <v>0</v>
+      </c>
+      <c r="J8" s="12">
+        <v>300</v>
+      </c>
+      <c r="K8" s="12">
+        <v>200</v>
+      </c>
+      <c r="L8" s="12">
+        <v>500</v>
+      </c>
+      <c r="M8" s="12">
+        <v>100</v>
+      </c>
+      <c r="N8" s="12">
+        <v>400</v>
+      </c>
+      <c r="P8">
+        <v>2030</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" ref="Q8:Q11" si="2">I26/(I$4^I$3)</f>
+        <v>335.7837239373664</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="1"/>
+        <v>602.14507946302194</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="1"/>
+        <v>282.17112468110213</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="1"/>
+        <v>329.37618718127163</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="1"/>
+        <v>199.72932180853405</v>
+      </c>
+      <c r="V8">
+        <f t="shared" si="1"/>
+        <v>470.12342359151938</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="D9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="16">
+        <v>2035</v>
+      </c>
+      <c r="I9" s="12">
+        <v>0</v>
+      </c>
+      <c r="J9" s="12">
+        <v>300</v>
+      </c>
+      <c r="K9" s="12">
+        <v>300</v>
+      </c>
+      <c r="L9" s="12">
+        <v>400</v>
+      </c>
+      <c r="M9" s="12">
+        <v>100</v>
+      </c>
+      <c r="N9" s="12">
+        <v>400</v>
+      </c>
+      <c r="P9">
+        <v>2035</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="2"/>
+        <v>306.83685118414513</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="1"/>
+        <v>513.26735682620529</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="1"/>
+        <v>240.52214703290781</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="1"/>
+        <v>253.70432084799805</v>
+      </c>
+      <c r="U9">
+        <f t="shared" si="1"/>
+        <v>179.90027974669221</v>
+      </c>
+      <c r="V9">
+        <f t="shared" si="1"/>
+        <v>349.73608590241867</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="16">
+        <v>2040</v>
+      </c>
+      <c r="I10" s="12">
+        <v>0</v>
+      </c>
+      <c r="J10" s="12">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12">
+        <v>400</v>
+      </c>
+      <c r="L10" s="12">
+        <v>300</v>
+      </c>
+      <c r="M10" s="12">
+        <v>100</v>
+      </c>
+      <c r="N10" s="12">
+        <v>400</v>
+      </c>
+      <c r="P10">
+        <v>2040</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="2"/>
+        <v>280.38539849585669</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="1"/>
+        <v>437.50814972745678</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="1"/>
+        <v>205.02063518618488</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="1"/>
+        <v>195.4175344847267</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="1"/>
+        <v>162.03985654126046</v>
+      </c>
+      <c r="V10">
+        <f t="shared" si="1"/>
+        <v>320.74548223230937</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" s="16">
+        <v>2045</v>
+      </c>
+      <c r="I11" s="12">
+        <v>0</v>
+      </c>
+      <c r="J11" s="12">
+        <v>0</v>
+      </c>
+      <c r="K11" s="12">
+        <v>500</v>
+      </c>
+      <c r="L11" s="12">
+        <v>200</v>
+      </c>
+      <c r="M11" s="12">
+        <v>100</v>
+      </c>
+      <c r="N11" s="12">
+        <v>400</v>
+      </c>
+      <c r="P11">
+        <v>2045</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="2"/>
+        <v>256.21424345311044</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="1"/>
+        <v>372.93114111434943</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="1"/>
+        <v>174.75921186748658</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="1"/>
+        <v>150.52172803540446</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="1"/>
+        <v>145.95260855004346</v>
+      </c>
+      <c r="V11">
+        <f t="shared" si="1"/>
+        <v>292.46623032033017</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="C12" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="D12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" s="16">
+        <v>2050</v>
+      </c>
+      <c r="I12" s="12">
+        <v>0</v>
+      </c>
+      <c r="J12" s="12">
+        <v>0</v>
+      </c>
+      <c r="K12" s="12">
+        <v>600</v>
+      </c>
+      <c r="L12" s="12">
+        <v>100</v>
+      </c>
+      <c r="M12" s="12">
+        <v>100</v>
+      </c>
+      <c r="N12" s="12">
+        <v>400</v>
+      </c>
+      <c r="P12">
+        <v>2050</v>
+      </c>
+      <c r="Q12">
+        <f>I30/(I$4^I$3)</f>
+        <v>234.12680867266985</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="1"/>
+        <v>317.8858178973087</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="1"/>
+        <v>148.96443035994957</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="1"/>
+        <v>115.94041788780763</v>
+      </c>
+      <c r="U12">
+        <f t="shared" si="1"/>
+        <v>131.4624956924595</v>
+      </c>
+      <c r="V12">
+        <f t="shared" si="1"/>
+        <v>273.90733431991526</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15">
+        <f>B18/(B16^B17)</f>
+        <v>3084.0998748711568</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ref="C15:E15" si="3">C18/(C16^C17)</f>
+        <v>9616.9213175821751</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="3"/>
+        <v>113244.05359147559</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="3"/>
+        <v>12395053.207512364</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="I15" t="s">
+        <v>28</v>
+      </c>
+      <c r="J15" t="s">
+        <v>81</v>
+      </c>
+      <c r="K15" t="s">
+        <v>82</v>
+      </c>
+      <c r="L15" t="s">
+        <v>2</v>
+      </c>
+      <c r="M15" t="s">
+        <v>3</v>
+      </c>
+      <c r="N15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16">
+        <v>261</v>
+      </c>
+      <c r="C16">
+        <v>4498</v>
+      </c>
+      <c r="D16">
+        <v>7099</v>
+      </c>
+      <c r="E16">
+        <v>18928</v>
+      </c>
+      <c r="H16" s="18">
+        <v>2025</v>
+      </c>
+      <c r="I16" s="12">
+        <f>I4+I7</f>
+        <v>600</v>
+      </c>
+      <c r="J16" s="12">
+        <f t="shared" ref="J16:N16" si="4">J4+J7</f>
+        <v>500</v>
+      </c>
+      <c r="K16" s="12">
+        <f t="shared" si="4"/>
+        <v>600</v>
+      </c>
+      <c r="L16" s="12">
+        <f t="shared" si="4"/>
+        <v>1100</v>
+      </c>
+      <c r="M16" s="12">
+        <f t="shared" si="4"/>
+        <v>600</v>
+      </c>
+      <c r="N16" s="12">
+        <f t="shared" si="4"/>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="5">
+        <f>B3</f>
+        <v>-7.1999999999999995E-2</v>
+      </c>
+      <c r="C17" s="5">
+        <f>B4</f>
+        <v>-7.8E-2</v>
+      </c>
+      <c r="D17" s="5">
+        <f>B5</f>
+        <v>-0.45</v>
+      </c>
+      <c r="E17" s="5">
+        <f>B6</f>
+        <v>-0.82899999999999996</v>
+      </c>
+      <c r="H17" s="18">
+        <v>2030</v>
+      </c>
+      <c r="I17" s="12">
+        <f>I16+I8</f>
+        <v>600</v>
+      </c>
+      <c r="J17" s="12">
+        <f t="shared" ref="J17:N20" si="5">J16+J8</f>
+        <v>800</v>
+      </c>
+      <c r="K17" s="12">
+        <f t="shared" si="5"/>
+        <v>800</v>
+      </c>
+      <c r="L17" s="12">
+        <f t="shared" si="5"/>
+        <v>1600</v>
+      </c>
+      <c r="M17" s="12">
+        <f t="shared" si="5"/>
+        <v>700</v>
+      </c>
+      <c r="N17" s="12">
+        <f t="shared" si="5"/>
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18">
+        <v>2066</v>
+      </c>
+      <c r="C18">
+        <v>4990</v>
+      </c>
+      <c r="D18">
+        <v>2094</v>
+      </c>
+      <c r="E18">
+        <v>3528</v>
+      </c>
+      <c r="H18" s="18">
+        <v>2035</v>
+      </c>
+      <c r="I18" s="12">
+        <f t="shared" ref="I18:I20" si="6">I17+I9</f>
+        <v>600</v>
+      </c>
+      <c r="J18" s="12">
+        <f t="shared" si="5"/>
+        <v>1100</v>
+      </c>
+      <c r="K18" s="12">
+        <f t="shared" si="5"/>
+        <v>1100</v>
+      </c>
+      <c r="L18" s="12">
+        <f t="shared" si="5"/>
+        <v>2000</v>
+      </c>
+      <c r="M18" s="12">
+        <f t="shared" si="5"/>
+        <v>800</v>
+      </c>
+      <c r="N18" s="12">
+        <f t="shared" si="5"/>
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H19" s="18">
+        <v>2040</v>
+      </c>
+      <c r="I19" s="12">
+        <f t="shared" si="6"/>
+        <v>600</v>
+      </c>
+      <c r="J19" s="12">
+        <f t="shared" si="5"/>
+        <v>1100</v>
+      </c>
+      <c r="K19" s="12">
+        <f t="shared" si="5"/>
+        <v>1500</v>
+      </c>
+      <c r="L19" s="12">
+        <f t="shared" si="5"/>
+        <v>2300</v>
+      </c>
+      <c r="M19" s="12">
+        <f t="shared" si="5"/>
+        <v>900</v>
+      </c>
+      <c r="N19" s="12">
+        <f t="shared" si="5"/>
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20">
+        <f>B15</f>
+        <v>3084.0998748711568</v>
+      </c>
+      <c r="C20">
+        <f t="shared" ref="C20:E20" si="7">C15</f>
+        <v>9616.9213175821751</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="7"/>
+        <v>113244.05359147559</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="7"/>
+        <v>12395053.207512364</v>
+      </c>
+      <c r="H20" s="18">
+        <v>2045</v>
+      </c>
+      <c r="I20" s="12">
+        <f t="shared" si="6"/>
+        <v>600</v>
+      </c>
+      <c r="J20" s="12">
+        <f t="shared" si="5"/>
+        <v>1100</v>
+      </c>
+      <c r="K20" s="12">
+        <f t="shared" si="5"/>
+        <v>2000</v>
+      </c>
+      <c r="L20" s="12">
+        <f t="shared" si="5"/>
+        <v>2500</v>
+      </c>
+      <c r="M20" s="12">
+        <f t="shared" si="5"/>
+        <v>1000</v>
+      </c>
+      <c r="N20" s="12">
+        <f t="shared" si="5"/>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21">
+        <f>B16+100</f>
+        <v>361</v>
+      </c>
+      <c r="C21">
+        <f t="shared" ref="C21:E21" si="8">C16+100</f>
+        <v>4598</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="8"/>
+        <v>7199</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="8"/>
+        <v>19028</v>
+      </c>
+      <c r="H21" s="18">
+        <v>2050</v>
+      </c>
+      <c r="I21" s="12">
+        <f>I20+I12</f>
+        <v>600</v>
+      </c>
+      <c r="J21" s="12">
+        <f t="shared" ref="J21:N21" si="9">J20+J12</f>
+        <v>1100</v>
+      </c>
+      <c r="K21" s="12">
+        <f t="shared" si="9"/>
+        <v>2600</v>
+      </c>
+      <c r="L21" s="12">
+        <f t="shared" si="9"/>
+        <v>2600</v>
+      </c>
+      <c r="M21" s="12">
+        <f t="shared" si="9"/>
+        <v>1100</v>
+      </c>
+      <c r="N21" s="12">
+        <f t="shared" si="9"/>
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="5">
+        <f>B17</f>
+        <v>-7.1999999999999995E-2</v>
+      </c>
+      <c r="C22" s="5">
+        <f t="shared" ref="C22:E22" si="10">C17</f>
+        <v>-7.8E-2</v>
+      </c>
+      <c r="D22" s="5">
+        <f t="shared" si="10"/>
+        <v>-0.45</v>
+      </c>
+      <c r="E22" s="5">
+        <f t="shared" si="10"/>
+        <v>-0.82899999999999996</v>
+      </c>
+      <c r="H22" s="18"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23">
+        <f>B20*(B21^B22)</f>
+        <v>2018.3102007173761</v>
+      </c>
+      <c r="C23">
+        <f t="shared" ref="C23:E23" si="11">C20*(C21^C22)</f>
+        <v>4981.4489427856479</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="11"/>
+        <v>2080.8603191100246</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="11"/>
+        <v>3512.6225095265308</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H24" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L24" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="M24" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="N24" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H25" s="18">
+        <v>2025</v>
+      </c>
+      <c r="I25" s="12">
+        <f>'Baseline Parameters'!G2</f>
+        <v>232</v>
+      </c>
+      <c r="J25" s="12">
+        <f>'Baseline Parameters'!B2</f>
+        <v>446</v>
+      </c>
+      <c r="K25" s="12">
+        <f>'Baseline Parameters'!C2</f>
+        <v>209</v>
+      </c>
+      <c r="L25" s="12">
+        <f>'Baseline Parameters'!E2</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="M25" s="12">
+        <f>'Baseline Parameters'!F2</f>
+        <v>140</v>
+      </c>
+      <c r="N25" s="12">
+        <f>Procurement!J3</f>
+        <v>360.50516023732143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H26" s="18">
+        <v>2030</v>
+      </c>
+      <c r="I26" s="12">
+        <f>'Baseline Parameters'!G3</f>
+        <v>212</v>
+      </c>
+      <c r="J26" s="12">
+        <f>'Baseline Parameters'!B3</f>
+        <v>380.16957864810638</v>
+      </c>
+      <c r="K26" s="12">
+        <f>'Baseline Parameters'!C3</f>
+        <v>178.15121510639958</v>
+      </c>
+      <c r="L26" s="12">
+        <f>'Baseline Parameters'!E3</f>
+        <v>207.95454545454541</v>
+      </c>
+      <c r="M26" s="12">
+        <f>'Baseline Parameters'!F3</f>
+        <v>126.10085958575935</v>
+      </c>
+      <c r="N26" s="12">
+        <f>Procurement!J4</f>
+        <v>296.81654796345282</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H27" s="18">
+        <v>2035</v>
+      </c>
+      <c r="I27" s="12">
+        <f>'Baseline Parameters'!G4</f>
+        <v>193.72413793103445</v>
+      </c>
+      <c r="J27" s="12">
+        <f>'Baseline Parameters'!B4</f>
+        <v>324.05584872080431</v>
+      </c>
+      <c r="K27" s="12">
+        <f>'Baseline Parameters'!C4</f>
+        <v>151.85576767409884</v>
+      </c>
+      <c r="L27" s="12">
+        <f>'Baseline Parameters'!E4</f>
+        <v>160.17844876188263</v>
+      </c>
+      <c r="M27" s="12">
+        <f>'Baseline Parameters'!F4</f>
+        <v>113.58161991619573</v>
+      </c>
+      <c r="N27" s="12">
+        <f>Procurement!J5</f>
+        <v>220.8089461332641</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H28" s="18">
+        <v>2040</v>
+      </c>
+      <c r="I28" s="12">
+        <f>'Baseline Parameters'!G5</f>
+        <v>177.02378121284181</v>
+      </c>
+      <c r="J28" s="12">
+        <f>'Baseline Parameters'!B5</f>
+        <v>276.22460866960239</v>
+      </c>
+      <c r="K28" s="12">
+        <f>'Baseline Parameters'!C5</f>
+        <v>129.4415767084011</v>
+      </c>
+      <c r="L28" s="12">
+        <f>'Baseline Parameters'!E5</f>
+        <v>123.37857483077323</v>
+      </c>
+      <c r="M28" s="12">
+        <f>'Baseline Parameters'!F5</f>
+        <v>102.30528503268064</v>
+      </c>
+      <c r="N28" s="12">
+        <f>Procurement!J6</f>
+        <v>202.50547416626196</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H29" s="18">
+        <v>2045</v>
+      </c>
+      <c r="I29" s="12">
+        <f>'Baseline Parameters'!G6</f>
+        <v>161.7631104186313</v>
+      </c>
+      <c r="J29" s="12">
+        <f>'Baseline Parameters'!B6</f>
+        <v>235.45334773578654</v>
+      </c>
+      <c r="K29" s="12">
+        <f>'Baseline Parameters'!C6</f>
+        <v>110.33576160712865</v>
+      </c>
+      <c r="L29" s="12">
+        <f>'Baseline Parameters'!E6</f>
+        <v>95.033213549856328</v>
+      </c>
+      <c r="M29" s="12">
+        <f>'Baseline Parameters'!F6</f>
+        <v>92.14845987705111</v>
+      </c>
+      <c r="N29" s="12">
+        <f>Procurement!J7</f>
+        <v>184.65112037257458</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H30" s="18">
+        <v>2050</v>
+      </c>
+      <c r="I30" s="12">
+        <f>'Baseline Parameters'!G7</f>
+        <v>147.8180146928872</v>
+      </c>
+      <c r="J30" s="12">
+        <f>'Baseline Parameters'!B7</f>
+        <v>200.70000000000002</v>
+      </c>
+      <c r="K30" s="12">
+        <f>'Baseline Parameters'!C7</f>
+        <v>94.05</v>
+      </c>
+      <c r="L30" s="12">
+        <f>'Baseline Parameters'!E7</f>
+        <v>73.199999999999989</v>
+      </c>
+      <c r="M30" s="12">
+        <f>'Baseline Parameters'!F7</f>
+        <v>83</v>
+      </c>
+      <c r="N30" s="12">
+        <f>Procurement!J8</f>
+        <v>172.93379856211703</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H31" s="18"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H32" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="I32" s="13"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
+      <c r="L32" s="13"/>
+      <c r="M32" s="13"/>
+      <c r="N32" s="13"/>
+    </row>
+    <row r="33" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H33" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K33" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L33" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="M33" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="N33" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H34" s="18">
+        <v>2025</v>
+      </c>
+      <c r="I34" s="12">
+        <f>Q7*I16^I$3</f>
+        <v>228.8909241816344</v>
+      </c>
+      <c r="J34" s="12">
+        <f t="shared" ref="J34:N39" si="12">R7*J16^J$3</f>
+        <v>446</v>
+      </c>
+      <c r="K34" s="12">
+        <f t="shared" si="12"/>
+        <v>206.19915152569649</v>
+      </c>
+      <c r="L34" s="12">
+        <f t="shared" si="12"/>
+        <v>254.67919785643252</v>
+      </c>
+      <c r="M34" s="12">
+        <f t="shared" si="12"/>
+        <v>138.12383355788282</v>
+      </c>
+      <c r="N34" s="12">
+        <f t="shared" si="12"/>
+        <v>345.16068338004146</v>
+      </c>
+    </row>
+    <row r="35" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H35" s="18">
+        <v>2030</v>
+      </c>
+      <c r="I35" s="12">
+        <f t="shared" ref="I35:I39" si="13">Q8*I17^I$3</f>
+        <v>209.15894795907971</v>
+      </c>
+      <c r="J35" s="12">
+        <f t="shared" si="12"/>
+        <v>367.17447515029585</v>
+      </c>
+      <c r="K35" s="12">
+        <f t="shared" si="12"/>
+        <v>172.0615814045108</v>
+      </c>
+      <c r="L35" s="12">
+        <f t="shared" si="12"/>
+        <v>190.80393155301951</v>
+      </c>
+      <c r="M35" s="12">
+        <f t="shared" si="12"/>
+        <v>122.99984732811295</v>
+      </c>
+      <c r="N35" s="12">
+        <f t="shared" si="12"/>
+        <v>276.55408770473178</v>
+      </c>
+    </row>
+    <row r="36" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H36" s="18">
+        <v>2035</v>
+      </c>
+      <c r="I36" s="12">
+        <f t="shared" si="13"/>
+        <v>191.12800416950384</v>
+      </c>
+      <c r="J36" s="12">
+        <f t="shared" si="12"/>
+        <v>305.68954522936554</v>
+      </c>
+      <c r="K36" s="12">
+        <f t="shared" si="12"/>
+        <v>143.24913666577888</v>
+      </c>
+      <c r="L36" s="12">
+        <f t="shared" si="12"/>
+        <v>144.56116653140265</v>
+      </c>
+      <c r="M36" s="12">
+        <f t="shared" si="12"/>
+        <v>109.69912907747937</v>
+      </c>
+      <c r="N36" s="12">
+        <f t="shared" si="12"/>
+        <v>201.69132781051039</v>
+      </c>
+    </row>
+    <row r="37" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H37" s="18">
+        <v>2040</v>
+      </c>
+      <c r="I37" s="12">
+        <f t="shared" si="13"/>
+        <v>174.65145208592588</v>
+      </c>
+      <c r="J37" s="12">
+        <f t="shared" si="12"/>
+        <v>260.56920539681425</v>
+      </c>
+      <c r="K37" s="12">
+        <f t="shared" si="12"/>
+        <v>119.33472084678709</v>
+      </c>
+      <c r="L37" s="12">
+        <f t="shared" si="12"/>
+        <v>110.20357158277476</v>
+      </c>
+      <c r="M37" s="12">
+        <f t="shared" si="12"/>
+        <v>97.950781264889969</v>
+      </c>
+      <c r="N37" s="12">
+        <f t="shared" si="12"/>
+        <v>182.1026727916458</v>
+      </c>
+    </row>
+    <row r="38" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H38" s="18">
+        <v>2045</v>
+      </c>
+      <c r="I38" s="12">
+        <f t="shared" si="13"/>
+        <v>159.59529242334608</v>
+      </c>
+      <c r="J38" s="12">
+        <f t="shared" si="12"/>
+        <v>222.10871081699267</v>
+      </c>
+      <c r="K38" s="12">
+        <f t="shared" si="12"/>
+        <v>99.578105115554848</v>
+      </c>
+      <c r="L38" s="12">
+        <f t="shared" si="12"/>
+        <v>84.362926134929509</v>
+      </c>
+      <c r="M38" s="12">
+        <f t="shared" si="12"/>
+        <v>87.541072164529638</v>
+      </c>
+      <c r="N38" s="12">
+        <f t="shared" si="12"/>
+        <v>163.91857380000212</v>
+      </c>
+    </row>
+    <row r="39" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H39" s="18">
+        <v>2050</v>
+      </c>
+      <c r="I39" s="12">
+        <f t="shared" si="13"/>
+        <v>145.83707755926449</v>
+      </c>
+      <c r="J39" s="12">
+        <f t="shared" si="12"/>
+        <v>189.32505606585244</v>
+      </c>
+      <c r="K39" s="12">
+        <f t="shared" si="12"/>
+        <v>83.24814259608965</v>
+      </c>
+      <c r="L39" s="12">
+        <f t="shared" si="12"/>
+        <v>64.792812738264345</v>
+      </c>
+      <c r="M39" s="12">
+        <f t="shared" si="12"/>
+        <v>78.295862747711766</v>
+      </c>
+      <c r="N39" s="12">
+        <f t="shared" si="12"/>
+        <v>151.84000504571642</v>
+      </c>
+    </row>
+    <row r="40" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H40" s="18"/>
+      <c r="I40" s="12"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="12"/>
+      <c r="M40" s="12"/>
+      <c r="N40" s="12"/>
+    </row>
+    <row r="41" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H41" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+      <c r="N41" s="13"/>
+    </row>
+    <row r="42" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H42" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="I42" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J42" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K42" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L42" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="M42" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="N42" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H43" s="18">
+        <v>2025</v>
+      </c>
+      <c r="I43" s="12">
+        <f>I25-I34</f>
+        <v>3.1090758183655964</v>
+      </c>
+      <c r="J43" s="12">
+        <f t="shared" ref="J43:N43" si="14">J25-J34</f>
+        <v>0</v>
+      </c>
+      <c r="K43" s="12">
+        <f t="shared" si="14"/>
+        <v>2.8008484743035069</v>
+      </c>
+      <c r="L43" s="12">
+        <f t="shared" si="14"/>
+        <v>15.301522455659295</v>
+      </c>
+      <c r="M43" s="12">
+        <f t="shared" si="14"/>
+        <v>1.8761664421171815</v>
+      </c>
+      <c r="N43" s="12">
+        <f t="shared" si="14"/>
+        <v>15.344476857279972</v>
+      </c>
+    </row>
+    <row r="44" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H44" s="18">
+        <v>2030</v>
+      </c>
+      <c r="I44" s="12">
+        <f t="shared" ref="I44:N48" si="15">I26-I35</f>
+        <v>2.8410520409202888</v>
+      </c>
+      <c r="J44" s="12">
+        <f t="shared" si="15"/>
+        <v>12.995103497810533</v>
+      </c>
+      <c r="K44" s="12">
+        <f t="shared" si="15"/>
+        <v>6.0896337018887721</v>
+      </c>
+      <c r="L44" s="12">
+        <f t="shared" si="15"/>
+        <v>17.150613901525901</v>
+      </c>
+      <c r="M44" s="12">
+        <f t="shared" si="15"/>
+        <v>3.1010122576464028</v>
+      </c>
+      <c r="N44" s="12">
+        <f t="shared" si="15"/>
+        <v>20.262460258721035</v>
+      </c>
+    </row>
+    <row r="45" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H45" s="18">
+        <v>2035</v>
+      </c>
+      <c r="I45" s="12">
+        <f t="shared" si="15"/>
+        <v>2.5961337615306093</v>
+      </c>
+      <c r="J45" s="12">
+        <f t="shared" si="15"/>
+        <v>18.366303491438771</v>
+      </c>
+      <c r="K45" s="12">
+        <f t="shared" si="15"/>
+        <v>8.6066310083199653</v>
+      </c>
+      <c r="L45" s="12">
+        <f t="shared" si="15"/>
+        <v>15.617282230479987</v>
+      </c>
+      <c r="M45" s="12">
+        <f t="shared" si="15"/>
+        <v>3.8824908387163646</v>
+      </c>
+      <c r="N45" s="12">
+        <f t="shared" si="15"/>
+        <v>19.117618322753714</v>
+      </c>
+    </row>
+    <row r="46" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H46" s="18">
+        <v>2040</v>
+      </c>
+      <c r="I46" s="12">
+        <f t="shared" si="15"/>
+        <v>2.372329126915929</v>
+      </c>
+      <c r="J46" s="12">
+        <f t="shared" si="15"/>
+        <v>15.655403272788135</v>
+      </c>
+      <c r="K46" s="12">
+        <f t="shared" si="15"/>
+        <v>10.106855861614008</v>
+      </c>
+      <c r="L46" s="12">
+        <f t="shared" si="15"/>
+        <v>13.175003247998475</v>
+      </c>
+      <c r="M46" s="12">
+        <f t="shared" si="15"/>
+        <v>4.3545037677906748</v>
+      </c>
+      <c r="N46" s="12">
+        <f t="shared" si="15"/>
+        <v>20.402801374616161</v>
+      </c>
+    </row>
+    <row r="47" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H47" s="18">
+        <v>2045</v>
+      </c>
+      <c r="I47" s="12">
+        <f t="shared" si="15"/>
+        <v>2.167817995285219</v>
+      </c>
+      <c r="J47" s="12">
+        <f t="shared" si="15"/>
+        <v>13.344636918793867</v>
+      </c>
+      <c r="K47" s="12">
+        <f t="shared" si="15"/>
+        <v>10.757656491573798</v>
+      </c>
+      <c r="L47" s="12">
+        <f t="shared" si="15"/>
+        <v>10.670287414926818</v>
+      </c>
+      <c r="M47" s="12">
+        <f t="shared" si="15"/>
+        <v>4.6073877125214722</v>
+      </c>
+      <c r="N47" s="12">
+        <f t="shared" si="15"/>
+        <v>20.73254657257246</v>
+      </c>
+    </row>
+    <row r="48" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H48" s="18">
+        <v>2050</v>
+      </c>
+      <c r="I48" s="12">
+        <f t="shared" si="15"/>
+        <v>1.9809371336227173</v>
+      </c>
+      <c r="J48" s="12">
+        <f t="shared" si="15"/>
+        <v>11.374943934147581</v>
+      </c>
+      <c r="K48" s="12">
+        <f t="shared" si="15"/>
+        <v>10.801857403910347</v>
+      </c>
+      <c r="L48" s="12">
+        <f t="shared" si="15"/>
+        <v>8.4071872617356433</v>
+      </c>
+      <c r="M48" s="12">
+        <f t="shared" si="15"/>
+        <v>4.7041372522882341</v>
+      </c>
+      <c r="N48" s="12">
+        <f t="shared" si="15"/>
+        <v>21.093793516400609</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="H41:N41"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H32:N32"/>
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="P5:V5"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="I43:N48">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{24FFCE81-5015-4DFC-9C15-040909BF294A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23D47325-8713-4C29-9B32-6AF71A8D6F7B}">
   <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5002,7 +6844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16D7DDB-ECAA-4988-BB02-23E7116C40BF}">
   <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5555,7 +7397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8195A587-BA09-4421-98D4-BDAFBA104359}">
   <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
5 innovation policy scenarios
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D725B470-7CB3-4F48-8777-63CEC138394C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF37EA2-74DA-4772-877C-2EC8E4B3613B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
@@ -19,7 +19,11 @@
     <sheet name="verify-2025" sheetId="3" r:id="rId4"/>
     <sheet name="Procurement" sheetId="4" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Learning Rates'!$Y$1:$AA$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="117">
   <si>
     <t>Tech</t>
   </si>
@@ -291,9 +295,6 @@
     <t>DAC Solvent</t>
   </si>
   <si>
-    <t>This Study</t>
-  </si>
-  <si>
     <t>Learning Rate</t>
   </si>
   <si>
@@ -325,6 +326,75 @@
   </si>
   <si>
     <t>Cost Savings (2025USD/t CDR)</t>
+  </si>
+  <si>
+    <t>Percentage Cost Savings</t>
+  </si>
+  <si>
+    <t>All Technologies</t>
+  </si>
+  <si>
+    <t>CDR Policy Scenarios</t>
+  </si>
+  <si>
+    <t>Policy 1</t>
+  </si>
+  <si>
+    <t>Policy 2</t>
+  </si>
+  <si>
+    <t>Policy 3</t>
+  </si>
+  <si>
+    <t>Policy 4</t>
+  </si>
+  <si>
+    <t>Policy 5</t>
+  </si>
+  <si>
+    <t>Policy 6</t>
+  </si>
+  <si>
+    <t>Rhodium $6B</t>
+  </si>
+  <si>
+    <t>Maintain current appropriations</t>
+  </si>
+  <si>
+    <t>Triple R&amp;D</t>
+  </si>
+  <si>
+    <t>CATF (2025)</t>
+  </si>
+  <si>
+    <t>DAC Hubs (Sorbent)</t>
+  </si>
+  <si>
+    <t>DAC Hubs (Solvent)</t>
+  </si>
+  <si>
+    <t>CDR R&amp;D</t>
+  </si>
+  <si>
+    <t>https://www.congress.gov/crs-product/IF11861#:~:text=For%20carbon%20removal%2C%20Congress%</t>
+  </si>
+  <si>
+    <t>2009-2018</t>
+  </si>
+  <si>
+    <t>https://bipartisanpolicy.org/download/?file=/wp-content/uploads/2019/06/Carbon-Removal-Comparing-Historical-Investments-with-the-National-Academies-Recommendations.pdf</t>
+  </si>
+  <si>
+    <t>Same as 2022 non-supplemental investments</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Rhodium $18B</t>
+  </si>
+  <si>
+    <t>Cumulative Public R&amp;D (Million USD)</t>
   </si>
 </sst>
 </file>
@@ -398,7 +468,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -418,7 +488,7 @@
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -428,20 +498,21 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -4363,7 +4434,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05431749-67AB-462A-BE29-983F9537704D}">
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:AA66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -4372,19 +4443,20 @@
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="H1" s="14" t="s">
-        <v>83</v>
+        <v>87</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>95</v>
       </c>
       <c r="I1" t="s">
         <v>28</v>
@@ -4404,8 +4476,38 @@
       <c r="N1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="P1" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>97</v>
+      </c>
+      <c r="R1" t="s">
+        <v>98</v>
+      </c>
+      <c r="S1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T1" t="s">
+        <v>100</v>
+      </c>
+      <c r="U1" t="s">
+        <v>101</v>
+      </c>
+      <c r="V1" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -4418,35 +4520,71 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="I2" s="10">
+      <c r="H2" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="I2" s="9">
         <f>1-2^I3</f>
         <v>4.9999617125113915E-2</v>
       </c>
-      <c r="J2" s="10">
+      <c r="J2" s="9">
         <f t="shared" ref="J2:N2" si="0">1-2^J3</f>
         <v>4.9999617125113915E-2</v>
       </c>
-      <c r="K2" s="10">
+      <c r="K2" s="9">
         <f t="shared" si="0"/>
         <v>4.9999617125113915E-2</v>
       </c>
-      <c r="L2" s="10">
+      <c r="L2" s="9">
         <f t="shared" si="0"/>
         <v>4.9999617125113915E-2</v>
       </c>
-      <c r="M2" s="10">
+      <c r="M2" s="9">
         <f t="shared" si="0"/>
         <v>4.9999617125113915E-2</v>
       </c>
-      <c r="N2" s="10">
+      <c r="N2" s="9">
         <f t="shared" si="0"/>
         <v>4.9999617125113915E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="P2" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q2" s="9">
+        <f>1-2^Q3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="R2" s="9">
+        <f t="shared" ref="R2" si="1">1-2^R3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="S2" s="9">
+        <f t="shared" ref="S2" si="2">1-2^S3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="T2" s="9">
+        <f t="shared" ref="T2" si="3">1-2^T3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="U2" s="9">
+        <f t="shared" ref="U2" si="4">1-2^U3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="V2" s="9">
+        <f t="shared" ref="V2" si="5">1-2^V3</f>
+        <v>4.9999617125113915E-2</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z2">
+        <v>1045</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>4.9000000000000002E-2</v>
       </c>
@@ -4462,8 +4600,8 @@
       <c r="E3" t="s">
         <v>62</v>
       </c>
-      <c r="H3" s="16" t="s">
-        <v>86</v>
+      <c r="H3" s="13" t="s">
+        <v>85</v>
       </c>
       <c r="I3">
         <v>-7.3999999999999996E-2</v>
@@ -4483,8 +4621,38 @@
       <c r="N3">
         <v>-7.3999999999999996E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="P3" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="R3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="S3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="T3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="U3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="V3">
+        <v>-7.3999999999999996E-2</v>
+      </c>
+      <c r="Y3">
+        <v>2019</v>
+      </c>
+      <c r="Z3">
+        <v>104</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
         <v>5.2999999999999999E-2</v>
       </c>
@@ -4500,29 +4668,71 @@
       <c r="E4" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="I4" s="9">
-        <v>500</v>
-      </c>
-      <c r="J4" s="9">
-        <v>500</v>
-      </c>
-      <c r="K4" s="9">
-        <v>500</v>
-      </c>
-      <c r="L4" s="9">
-        <v>500</v>
-      </c>
-      <c r="M4" s="9">
-        <v>500</v>
-      </c>
-      <c r="N4" s="9">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H4" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:N4" si="6">$Z$9</f>
+        <v>1719</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="6"/>
+        <v>1719</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="6"/>
+        <v>1719</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="6"/>
+        <v>1719</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="6"/>
+        <v>1719</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="6"/>
+        <v>1719</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q4">
+        <f>$Z$9</f>
+        <v>1719</v>
+      </c>
+      <c r="R4">
+        <f>Q4</f>
+        <v>1719</v>
+      </c>
+      <c r="S4">
+        <f>R4</f>
+        <v>1719</v>
+      </c>
+      <c r="T4">
+        <f>S4</f>
+        <v>1719</v>
+      </c>
+      <c r="U4">
+        <f>T4</f>
+        <v>1719</v>
+      </c>
+      <c r="V4">
+        <f>T4</f>
+        <v>1719</v>
+      </c>
+      <c r="Y4">
+        <v>2020</v>
+      </c>
+      <c r="Z4">
+        <v>104</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="7">
         <v>0.26800000000000002</v>
       </c>
@@ -4538,26 +4748,35 @@
       <c r="E5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="P5" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H5" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="P5" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="Y5">
+        <v>2021</v>
+      </c>
+      <c r="Z5">
+        <v>104</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>0.437</v>
       </c>
@@ -4573,7 +4792,7 @@
       <c r="E6" t="s">
         <v>62</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="H6" t="s">
         <v>40</v>
       </c>
       <c r="I6" t="s">
@@ -4598,75 +4817,99 @@
         <v>40</v>
       </c>
       <c r="Q6" t="s">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="R6" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="S6" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="T6" t="s">
-        <v>2</v>
+        <v>107</v>
       </c>
       <c r="U6" t="s">
-        <v>3</v>
+        <v>108</v>
       </c>
       <c r="V6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H7" s="16">
+        <v>115</v>
+      </c>
+      <c r="Y6">
+        <v>2022</v>
+      </c>
+      <c r="Z6">
+        <v>104</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="H7">
         <v>2025</v>
       </c>
-      <c r="I7" s="12">
-        <v>100</v>
-      </c>
-      <c r="J7" s="12">
-        <v>0</v>
-      </c>
-      <c r="K7" s="12">
-        <v>100</v>
-      </c>
-      <c r="L7" s="12">
-        <v>600</v>
-      </c>
-      <c r="M7" s="12">
-        <v>100</v>
-      </c>
-      <c r="N7" s="12">
-        <v>400</v>
+      <c r="I7">
+        <f t="shared" ref="I7:N12" si="7">I34/(I$4^I$3)</f>
+        <v>402.62283243923065</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="7"/>
+        <v>774.00768649955546</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="7"/>
+        <v>362.70763784396212</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="7"/>
+        <v>468.53621687947475</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="7"/>
+        <v>242.96205405815644</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="7"/>
+        <v>625.63624449874601</v>
       </c>
       <c r="P7">
         <v>2025</v>
       </c>
       <c r="Q7">
-        <f>I25/(I$4^I$3)</f>
-        <v>367.46143374277835</v>
+        <f t="shared" ref="Q7:V12" si="8">Q34/(Q$4^Q$3)</f>
+        <v>625.63624449874601</v>
       </c>
       <c r="R7">
-        <f t="shared" ref="R7:V12" si="1">J25/(J$4^J$3)</f>
-        <v>706.41292866068591</v>
+        <f t="shared" si="8"/>
+        <v>625.63624449874601</v>
       </c>
       <c r="S7">
-        <f t="shared" si="1"/>
-        <v>331.03206746655462</v>
+        <f t="shared" si="8"/>
+        <v>625.63624449874601</v>
       </c>
       <c r="T7">
-        <f t="shared" si="1"/>
-        <v>427.61854555512627</v>
+        <f t="shared" si="8"/>
+        <v>774.00768649955546</v>
       </c>
       <c r="U7">
-        <f t="shared" si="1"/>
-        <v>221.74396863788348</v>
+        <f t="shared" si="8"/>
+        <v>362.70763784396212</v>
       </c>
       <c r="V7">
-        <f t="shared" si="1"/>
-        <v>570.9988924675697</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>625.63624449874601</v>
+      </c>
+      <c r="Y7">
+        <v>2023</v>
+      </c>
+      <c r="Z7">
+        <v>140</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>63</v>
       </c>
@@ -4679,56 +4922,71 @@
       <c r="E8" t="s">
         <v>5</v>
       </c>
-      <c r="H8" s="16">
+      <c r="H8">
         <v>2030</v>
       </c>
-      <c r="I8" s="12">
-        <v>0</v>
-      </c>
-      <c r="J8" s="12">
-        <v>300</v>
-      </c>
-      <c r="K8" s="12">
-        <v>200</v>
-      </c>
-      <c r="L8" s="12">
-        <v>500</v>
-      </c>
-      <c r="M8" s="12">
-        <v>100</v>
-      </c>
-      <c r="N8" s="12">
-        <v>400</v>
+      <c r="I8">
+        <f t="shared" si="7"/>
+        <v>367.91396757377976</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="7"/>
+        <v>659.76272656262699</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="7"/>
+        <v>309.17132253719507</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="7"/>
+        <v>360.89331081690437</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="7"/>
+        <v>218.84088473896614</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="7"/>
+        <v>515.10827265465582</v>
       </c>
       <c r="P8">
         <v>2030</v>
       </c>
       <c r="Q8">
-        <f t="shared" ref="Q8:Q11" si="2">I26/(I$4^I$3)</f>
-        <v>335.7837239373664</v>
+        <f t="shared" si="8"/>
+        <v>515.10827265465582</v>
       </c>
       <c r="R8">
-        <f t="shared" si="1"/>
-        <v>602.14507946302194</v>
+        <f t="shared" si="8"/>
+        <v>515.10827265465582</v>
       </c>
       <c r="S8">
-        <f t="shared" si="1"/>
-        <v>282.17112468110213</v>
+        <f t="shared" si="8"/>
+        <v>515.10827265465582</v>
       </c>
       <c r="T8">
-        <f t="shared" si="1"/>
-        <v>329.37618718127163</v>
+        <f t="shared" si="8"/>
+        <v>659.76272656262699</v>
       </c>
       <c r="U8">
-        <f t="shared" si="1"/>
-        <v>199.72932180853405</v>
+        <f t="shared" si="8"/>
+        <v>309.17132253719507</v>
       </c>
       <c r="V8">
-        <f t="shared" si="1"/>
-        <v>470.12342359151938</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>515.10827265465582</v>
+      </c>
+      <c r="Y8">
+        <v>2024</v>
+      </c>
+      <c r="Z8">
+        <v>118</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>66</v>
       </c>
@@ -4744,56 +5002,69 @@
       <c r="F9" t="s">
         <v>65</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9">
         <v>2035</v>
       </c>
-      <c r="I9" s="12">
-        <v>0</v>
-      </c>
-      <c r="J9" s="12">
-        <v>300</v>
-      </c>
-      <c r="K9" s="12">
-        <v>300</v>
-      </c>
-      <c r="L9" s="12">
-        <v>400</v>
-      </c>
-      <c r="M9" s="12">
-        <v>100</v>
-      </c>
-      <c r="N9" s="12">
-        <v>400</v>
+      <c r="I9">
+        <f t="shared" si="7"/>
+        <v>336.19724623121249</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="7"/>
+        <v>562.38053310547014</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="7"/>
+        <v>263.53706596198032</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="7"/>
+        <v>277.98060662168695</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="7"/>
+        <v>197.11445484351233</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="7"/>
+        <v>383.20139362110473</v>
       </c>
       <c r="P9">
         <v>2035</v>
       </c>
       <c r="Q9">
-        <f t="shared" si="2"/>
-        <v>306.83685118414513</v>
+        <f t="shared" si="8"/>
+        <v>383.20139362110473</v>
       </c>
       <c r="R9">
-        <f t="shared" si="1"/>
-        <v>513.26735682620529</v>
+        <f t="shared" si="8"/>
+        <v>383.20139362110473</v>
       </c>
       <c r="S9">
-        <f t="shared" si="1"/>
-        <v>240.52214703290781</v>
+        <f t="shared" si="8"/>
+        <v>383.20139362110473</v>
       </c>
       <c r="T9">
-        <f t="shared" si="1"/>
-        <v>253.70432084799805</v>
+        <f t="shared" si="8"/>
+        <v>562.38053310547014</v>
       </c>
       <c r="U9">
-        <f t="shared" si="1"/>
-        <v>179.90027974669221</v>
+        <f t="shared" si="8"/>
+        <v>263.53706596198032</v>
       </c>
       <c r="V9">
-        <f t="shared" si="1"/>
-        <v>349.73608590241867</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>383.20139362110473</v>
+      </c>
+      <c r="Y9" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z9" s="17">
+        <f>SUM(Z2:Z8)</f>
+        <v>1719</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>68</v>
       </c>
@@ -4806,56 +5077,62 @@
       <c r="F10" t="s">
         <v>65</v>
       </c>
-      <c r="H10" s="16">
+      <c r="H10">
         <v>2040</v>
       </c>
-      <c r="I10" s="12">
-        <v>0</v>
-      </c>
-      <c r="J10" s="12">
-        <v>0</v>
-      </c>
-      <c r="K10" s="12">
-        <v>400</v>
-      </c>
-      <c r="L10" s="12">
-        <v>300</v>
-      </c>
-      <c r="M10" s="12">
-        <v>100</v>
-      </c>
-      <c r="N10" s="12">
-        <v>400</v>
+      <c r="I10">
+        <f t="shared" si="7"/>
+        <v>307.21472500438381</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="7"/>
+        <v>479.37213074126458</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="7"/>
+        <v>224.63850969713965</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="7"/>
+        <v>214.11651405466162</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="7"/>
+        <v>177.54501566103755</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="7"/>
+        <v>351.43675686754244</v>
       </c>
       <c r="P10">
         <v>2040</v>
       </c>
       <c r="Q10">
-        <f t="shared" si="2"/>
-        <v>280.38539849585669</v>
+        <f t="shared" si="8"/>
+        <v>351.43675686754244</v>
       </c>
       <c r="R10">
-        <f t="shared" si="1"/>
-        <v>437.50814972745678</v>
+        <f t="shared" si="8"/>
+        <v>351.43675686754244</v>
       </c>
       <c r="S10">
-        <f t="shared" si="1"/>
-        <v>205.02063518618488</v>
+        <f t="shared" si="8"/>
+        <v>351.43675686754244</v>
       </c>
       <c r="T10">
-        <f t="shared" si="1"/>
-        <v>195.4175344847267</v>
+        <f t="shared" si="8"/>
+        <v>479.37213074126458</v>
       </c>
       <c r="U10">
-        <f t="shared" si="1"/>
-        <v>162.03985654126046</v>
+        <f t="shared" si="8"/>
+        <v>224.63850969713965</v>
       </c>
       <c r="V10">
-        <f t="shared" si="1"/>
-        <v>320.74548223230937</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>351.43675686754244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>70</v>
       </c>
@@ -4868,56 +5145,62 @@
       <c r="F11" t="s">
         <v>72</v>
       </c>
-      <c r="H11" s="16">
+      <c r="H11">
         <v>2045</v>
       </c>
-      <c r="I11" s="12">
-        <v>0</v>
-      </c>
-      <c r="J11" s="12">
-        <v>0</v>
-      </c>
-      <c r="K11" s="12">
-        <v>500</v>
-      </c>
-      <c r="L11" s="12">
-        <v>200</v>
-      </c>
-      <c r="M11" s="12">
-        <v>100</v>
-      </c>
-      <c r="N11" s="12">
-        <v>400</v>
+      <c r="I11">
+        <f t="shared" si="7"/>
+        <v>280.73069698676449</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="7"/>
+        <v>408.61592143397195</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="7"/>
+        <v>191.48145197242181</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="7"/>
+        <v>164.92474834157514</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="7"/>
+        <v>159.91842207159965</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="7"/>
+        <v>320.45153921329012</v>
       </c>
       <c r="P11">
         <v>2045</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="2"/>
-        <v>256.21424345311044</v>
+        <f t="shared" si="8"/>
+        <v>320.45153921329012</v>
       </c>
       <c r="R11">
-        <f t="shared" si="1"/>
-        <v>372.93114111434943</v>
+        <f t="shared" si="8"/>
+        <v>320.45153921329012</v>
       </c>
       <c r="S11">
-        <f t="shared" si="1"/>
-        <v>174.75921186748658</v>
+        <f t="shared" si="8"/>
+        <v>320.45153921329012</v>
       </c>
       <c r="T11">
-        <f t="shared" si="1"/>
-        <v>150.52172803540446</v>
+        <f t="shared" si="8"/>
+        <v>408.61592143397195</v>
       </c>
       <c r="U11">
-        <f t="shared" si="1"/>
-        <v>145.95260855004346</v>
+        <f t="shared" si="8"/>
+        <v>191.48145197242181</v>
       </c>
       <c r="V11">
-        <f t="shared" si="1"/>
-        <v>292.46623032033017</v>
-      </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>320.45153921329012</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C12" s="1">
         <v>0.05</v>
       </c>
@@ -4930,61 +5213,68 @@
       <c r="F12" t="s">
         <v>72</v>
       </c>
-      <c r="H12" s="16">
+      <c r="H12">
         <v>2050</v>
       </c>
-      <c r="I12" s="12">
-        <v>0</v>
-      </c>
-      <c r="J12" s="12">
-        <v>0</v>
-      </c>
-      <c r="K12" s="12">
-        <v>600</v>
-      </c>
-      <c r="L12" s="12">
-        <v>100</v>
-      </c>
-      <c r="M12" s="12">
-        <v>100</v>
-      </c>
-      <c r="N12" s="12">
-        <v>400</v>
+      <c r="I12">
+        <f t="shared" si="7"/>
+        <v>256.52977483273304</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="7"/>
+        <v>348.3034589248</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="7"/>
+        <v>163.21843702978293</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="7"/>
+        <v>127.03444540755035</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="7"/>
+        <v>144.04178919162132</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="7"/>
+        <v>300.11679224808154</v>
       </c>
       <c r="P12">
         <v>2050</v>
       </c>
       <c r="Q12">
-        <f>I30/(I$4^I$3)</f>
-        <v>234.12680867266985</v>
+        <f t="shared" si="8"/>
+        <v>300.11679224808154</v>
       </c>
       <c r="R12">
-        <f t="shared" si="1"/>
-        <v>317.8858178973087</v>
+        <f t="shared" si="8"/>
+        <v>300.11679224808154</v>
       </c>
       <c r="S12">
-        <f t="shared" si="1"/>
-        <v>148.96443035994957</v>
+        <f t="shared" si="8"/>
+        <v>300.11679224808154</v>
       </c>
       <c r="T12">
-        <f t="shared" si="1"/>
-        <v>115.94041788780763</v>
+        <f t="shared" si="8"/>
+        <v>348.3034589248</v>
       </c>
       <c r="U12">
-        <f t="shared" si="1"/>
-        <v>131.4624956924595</v>
+        <f t="shared" si="8"/>
+        <v>163.21843702978293</v>
       </c>
       <c r="V12">
-        <f t="shared" si="1"/>
-        <v>273.90733431991526</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="8"/>
+        <v>300.11679224808154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="P13" s="13"/>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>79</v>
       </c>
@@ -5000,17 +5290,26 @@
       <c r="E14" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H14" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="P14" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>77</v>
       </c>
@@ -5019,18 +5318,18 @@
         <v>3084.0998748711568</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:E15" si="3">C18/(C16^C17)</f>
+        <f t="shared" ref="C15:E15" si="9">C18/(C16^C17)</f>
         <v>9616.9213175821751</v>
       </c>
       <c r="D15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>113244.05359147559</v>
       </c>
       <c r="E15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>12395053.207512364</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="13" t="s">
         <v>40</v>
       </c>
       <c r="I15" t="s">
@@ -5051,8 +5350,29 @@
       <c r="N15" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="P15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>103</v>
+      </c>
+      <c r="R15" t="s">
+        <v>104</v>
+      </c>
+      <c r="S15" t="s">
+        <v>105</v>
+      </c>
+      <c r="T15" t="s">
+        <v>107</v>
+      </c>
+      <c r="U15" t="s">
+        <v>108</v>
+      </c>
+      <c r="V15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -5068,35 +5388,51 @@
       <c r="E16">
         <v>18928</v>
       </c>
-      <c r="H16" s="18">
+      <c r="H16" s="13">
         <v>2025</v>
       </c>
-      <c r="I16" s="12">
-        <f>I4+I7</f>
+      <c r="I16" s="10">
+        <v>100</v>
+      </c>
+      <c r="J16" s="10">
+        <v>0</v>
+      </c>
+      <c r="K16" s="10">
+        <v>100</v>
+      </c>
+      <c r="L16" s="10">
         <v>600</v>
       </c>
-      <c r="J16" s="12">
-        <f t="shared" ref="J16:N16" si="4">J4+J7</f>
-        <v>500</v>
-      </c>
-      <c r="K16" s="12">
-        <f t="shared" si="4"/>
-        <v>600</v>
-      </c>
-      <c r="L16" s="12">
-        <f t="shared" si="4"/>
-        <v>1100</v>
-      </c>
-      <c r="M16" s="12">
-        <f t="shared" si="4"/>
-        <v>600</v>
-      </c>
-      <c r="N16" s="12">
-        <f t="shared" si="4"/>
-        <v>900</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M16" s="10">
+        <v>100</v>
+      </c>
+      <c r="N16" s="10">
+        <v>400</v>
+      </c>
+      <c r="P16" s="13">
+        <v>2025</v>
+      </c>
+      <c r="Q16" s="16">
+        <v>0</v>
+      </c>
+      <c r="R16" s="16">
+        <v>118</v>
+      </c>
+      <c r="S16" s="16">
+        <f>R16*3</f>
+        <v>354</v>
+      </c>
+      <c r="T16" s="16">
+        <v>700</v>
+      </c>
+      <c r="U16" s="16">
+        <v>700</v>
+      </c>
+      <c r="V16" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>74</v>
       </c>
@@ -5116,35 +5452,51 @@
         <f>B6</f>
         <v>-0.82899999999999996</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="13">
         <v>2030</v>
       </c>
-      <c r="I17" s="12">
-        <f>I16+I8</f>
+      <c r="I17" s="10">
+        <v>0</v>
+      </c>
+      <c r="J17" s="10">
+        <v>300</v>
+      </c>
+      <c r="K17" s="10">
+        <v>200</v>
+      </c>
+      <c r="L17" s="10">
+        <v>500</v>
+      </c>
+      <c r="M17" s="10">
+        <v>100</v>
+      </c>
+      <c r="N17" s="10">
+        <v>400</v>
+      </c>
+      <c r="P17" s="13">
+        <v>2030</v>
+      </c>
+      <c r="Q17" s="16">
         <v>600</v>
       </c>
-      <c r="J17" s="12">
-        <f t="shared" ref="J17:N20" si="5">J16+J8</f>
-        <v>800</v>
-      </c>
-      <c r="K17" s="12">
-        <f t="shared" si="5"/>
-        <v>800</v>
-      </c>
-      <c r="L17" s="12">
-        <f t="shared" si="5"/>
-        <v>1600</v>
-      </c>
-      <c r="M17" s="12">
-        <f t="shared" si="5"/>
-        <v>700</v>
-      </c>
-      <c r="N17" s="12">
-        <f t="shared" si="5"/>
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="R17" s="16">
+        <v>118</v>
+      </c>
+      <c r="S17" s="16">
+        <f t="shared" ref="S17:S21" si="10">R17*3</f>
+        <v>354</v>
+      </c>
+      <c r="T17" s="16">
+        <v>0</v>
+      </c>
+      <c r="U17" s="16">
+        <v>0</v>
+      </c>
+      <c r="V17" s="16">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -5160,67 +5512,99 @@
       <c r="E18">
         <v>3528</v>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="13">
         <v>2035</v>
       </c>
-      <c r="I18" s="12">
-        <f t="shared" ref="I18:I20" si="6">I17+I9</f>
+      <c r="I18" s="10">
+        <v>0</v>
+      </c>
+      <c r="J18" s="10">
+        <v>300</v>
+      </c>
+      <c r="K18" s="10">
+        <v>300</v>
+      </c>
+      <c r="L18" s="10">
+        <v>400</v>
+      </c>
+      <c r="M18" s="10">
+        <v>100</v>
+      </c>
+      <c r="N18" s="10">
+        <v>400</v>
+      </c>
+      <c r="P18" s="13">
+        <v>2035</v>
+      </c>
+      <c r="Q18" s="16">
         <v>600</v>
       </c>
-      <c r="J18" s="12">
-        <f t="shared" si="5"/>
-        <v>1100</v>
-      </c>
-      <c r="K18" s="12">
-        <f t="shared" si="5"/>
-        <v>1100</v>
-      </c>
-      <c r="L18" s="12">
-        <f t="shared" si="5"/>
-        <v>2000</v>
-      </c>
-      <c r="M18" s="12">
-        <f t="shared" si="5"/>
-        <v>800</v>
-      </c>
-      <c r="N18" s="12">
-        <f t="shared" si="5"/>
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="R18" s="16">
+        <v>118</v>
+      </c>
+      <c r="S18" s="16">
+        <f t="shared" si="10"/>
+        <v>354</v>
+      </c>
+      <c r="T18" s="16">
+        <v>0</v>
+      </c>
+      <c r="U18" s="16">
+        <v>0</v>
+      </c>
+      <c r="V18" s="16">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="13">
         <v>2040</v>
       </c>
-      <c r="I19" s="12">
-        <f t="shared" si="6"/>
-        <v>600</v>
-      </c>
-      <c r="J19" s="12">
-        <f t="shared" si="5"/>
-        <v>1100</v>
-      </c>
-      <c r="K19" s="12">
-        <f t="shared" si="5"/>
-        <v>1500</v>
-      </c>
-      <c r="L19" s="12">
-        <f t="shared" si="5"/>
-        <v>2300</v>
-      </c>
-      <c r="M19" s="12">
-        <f t="shared" si="5"/>
-        <v>900</v>
-      </c>
-      <c r="N19" s="12">
-        <f t="shared" si="5"/>
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I19" s="10">
+        <v>0</v>
+      </c>
+      <c r="J19" s="10">
+        <v>0</v>
+      </c>
+      <c r="K19" s="10">
+        <v>400</v>
+      </c>
+      <c r="L19" s="10">
+        <v>300</v>
+      </c>
+      <c r="M19" s="10">
+        <v>100</v>
+      </c>
+      <c r="N19" s="10">
+        <v>400</v>
+      </c>
+      <c r="P19" s="13">
+        <v>2040</v>
+      </c>
+      <c r="Q19" s="16">
+        <v>0</v>
+      </c>
+      <c r="R19" s="16">
+        <v>118</v>
+      </c>
+      <c r="S19" s="16">
+        <f t="shared" si="10"/>
+        <v>354</v>
+      </c>
+      <c r="T19" s="16">
+        <v>0</v>
+      </c>
+      <c r="U19" s="16">
+        <v>0</v>
+      </c>
+      <c r="V19" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>77</v>
       </c>
@@ -5229,46 +5613,62 @@
         <v>3084.0998748711568</v>
       </c>
       <c r="C20">
-        <f t="shared" ref="C20:E20" si="7">C15</f>
+        <f t="shared" ref="C20:E20" si="11">C15</f>
         <v>9616.9213175821751</v>
       </c>
       <c r="D20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>113244.05359147559</v>
       </c>
       <c r="E20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>12395053.207512364</v>
       </c>
-      <c r="H20" s="18">
+      <c r="H20" s="13">
         <v>2045</v>
       </c>
-      <c r="I20" s="12">
-        <f t="shared" si="6"/>
-        <v>600</v>
-      </c>
-      <c r="J20" s="12">
-        <f t="shared" si="5"/>
-        <v>1100</v>
-      </c>
-      <c r="K20" s="12">
-        <f t="shared" si="5"/>
-        <v>2000</v>
-      </c>
-      <c r="L20" s="12">
-        <f t="shared" si="5"/>
-        <v>2500</v>
-      </c>
-      <c r="M20" s="12">
-        <f t="shared" si="5"/>
-        <v>1000</v>
-      </c>
-      <c r="N20" s="12">
-        <f t="shared" si="5"/>
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I20" s="10">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10">
+        <v>0</v>
+      </c>
+      <c r="K20" s="10">
+        <v>500</v>
+      </c>
+      <c r="L20" s="10">
+        <v>200</v>
+      </c>
+      <c r="M20" s="10">
+        <v>100</v>
+      </c>
+      <c r="N20" s="10">
+        <v>400</v>
+      </c>
+      <c r="P20" s="13">
+        <v>2045</v>
+      </c>
+      <c r="Q20" s="16">
+        <v>0</v>
+      </c>
+      <c r="R20" s="16">
+        <v>118</v>
+      </c>
+      <c r="S20" s="16">
+        <f t="shared" si="10"/>
+        <v>354</v>
+      </c>
+      <c r="T20" s="16">
+        <v>0</v>
+      </c>
+      <c r="U20" s="16">
+        <v>0</v>
+      </c>
+      <c r="V20" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>76</v>
       </c>
@@ -5277,46 +5677,62 @@
         <v>361</v>
       </c>
       <c r="C21">
-        <f t="shared" ref="C21:E21" si="8">C16+100</f>
+        <f t="shared" ref="C21:E21" si="12">C16+100</f>
         <v>4598</v>
       </c>
       <c r="D21">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>7199</v>
       </c>
       <c r="E21">
-        <f t="shared" si="8"/>
+        <f t="shared" si="12"/>
         <v>19028</v>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="13">
         <v>2050</v>
       </c>
-      <c r="I21" s="12">
-        <f>I20+I12</f>
+      <c r="I21" s="10">
+        <v>0</v>
+      </c>
+      <c r="J21" s="10">
+        <v>0</v>
+      </c>
+      <c r="K21" s="10">
         <v>600</v>
       </c>
-      <c r="J21" s="12">
-        <f t="shared" ref="J21:N21" si="9">J20+J12</f>
-        <v>1100</v>
-      </c>
-      <c r="K21" s="12">
-        <f t="shared" si="9"/>
-        <v>2600</v>
-      </c>
-      <c r="L21" s="12">
-        <f t="shared" si="9"/>
-        <v>2600</v>
-      </c>
-      <c r="M21" s="12">
-        <f t="shared" si="9"/>
-        <v>1100</v>
-      </c>
-      <c r="N21" s="12">
-        <f t="shared" si="9"/>
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L21" s="10">
+        <v>100</v>
+      </c>
+      <c r="M21" s="10">
+        <v>100</v>
+      </c>
+      <c r="N21" s="10">
+        <v>400</v>
+      </c>
+      <c r="P21" s="13">
+        <v>2050</v>
+      </c>
+      <c r="Q21" s="16">
+        <v>0</v>
+      </c>
+      <c r="R21" s="16">
+        <v>118</v>
+      </c>
+      <c r="S21" s="16">
+        <f t="shared" si="10"/>
+        <v>354</v>
+      </c>
+      <c r="T21" s="16">
+        <v>0</v>
+      </c>
+      <c r="U21" s="16">
+        <v>0</v>
+      </c>
+      <c r="V21" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -5325,26 +5741,40 @@
         <v>-7.1999999999999995E-2</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" ref="C22:E22" si="10">C17</f>
+        <f t="shared" ref="C22:E22" si="13">C17</f>
         <v>-7.8E-2</v>
       </c>
       <c r="D22" s="5">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>-0.45</v>
       </c>
       <c r="E22" s="5">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>-0.82899999999999996</v>
       </c>
-      <c r="H22" s="18"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
-      <c r="N22" s="12"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P22" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>49</v>
+      </c>
+      <c r="R22" t="s">
+        <v>106</v>
+      </c>
+      <c r="S22" t="s">
+        <v>106</v>
+      </c>
+      <c r="T22" t="s">
+        <v>106</v>
+      </c>
+      <c r="U22" t="s">
+        <v>106</v>
+      </c>
+      <c r="V22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -5353,669 +5783,2116 @@
         <v>2018.3102007173761</v>
       </c>
       <c r="C23">
-        <f t="shared" ref="C23:E23" si="11">C20*(C21^C22)</f>
+        <f t="shared" ref="C23:E23" si="14">C20*(C21^C22)</f>
         <v>4981.4489427856479</v>
       </c>
       <c r="D23">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>2080.8603191100246</v>
       </c>
       <c r="E23">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>3512.6225095265308</v>
       </c>
-      <c r="H23" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H24" s="18" t="s">
+      <c r="H23" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="P23" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="19"/>
+      <c r="U23" s="19"/>
+      <c r="V23" s="19"/>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H24" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="I24" s="12" t="s">
+      <c r="I24" t="s">
         <v>28</v>
       </c>
-      <c r="J24" s="12" t="s">
+      <c r="J24" t="s">
         <v>81</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="K24" t="s">
         <v>82</v>
       </c>
-      <c r="L24" s="12" t="s">
+      <c r="L24" t="s">
         <v>2</v>
       </c>
-      <c r="M24" s="12" t="s">
+      <c r="M24" t="s">
         <v>3</v>
       </c>
-      <c r="N24" s="12" t="s">
+      <c r="N24" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H25" s="18">
+      <c r="P24" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>103</v>
+      </c>
+      <c r="R24" t="s">
+        <v>104</v>
+      </c>
+      <c r="S24" t="s">
+        <v>105</v>
+      </c>
+      <c r="T24" t="s">
+        <v>107</v>
+      </c>
+      <c r="U24" t="s">
+        <v>108</v>
+      </c>
+      <c r="V24" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H25" s="14">
         <v>2025</v>
       </c>
-      <c r="I25" s="12">
+      <c r="I25" s="10">
+        <f t="shared" ref="I25:N25" si="15">I4+I16*5</f>
+        <v>2219</v>
+      </c>
+      <c r="J25" s="10">
+        <f t="shared" si="15"/>
+        <v>1719</v>
+      </c>
+      <c r="K25" s="10">
+        <f t="shared" si="15"/>
+        <v>2219</v>
+      </c>
+      <c r="L25" s="10">
+        <f t="shared" si="15"/>
+        <v>4719</v>
+      </c>
+      <c r="M25" s="10">
+        <f t="shared" si="15"/>
+        <v>2219</v>
+      </c>
+      <c r="N25" s="10">
+        <f t="shared" si="15"/>
+        <v>3719</v>
+      </c>
+      <c r="P25" s="14">
+        <v>2025</v>
+      </c>
+      <c r="Q25" s="10">
+        <f t="shared" ref="Q25:V25" si="16">Q4+Q16*5</f>
+        <v>1719</v>
+      </c>
+      <c r="R25" s="10">
+        <f t="shared" si="16"/>
+        <v>2309</v>
+      </c>
+      <c r="S25" s="10">
+        <f t="shared" si="16"/>
+        <v>3489</v>
+      </c>
+      <c r="T25" s="10">
+        <f t="shared" si="16"/>
+        <v>5219</v>
+      </c>
+      <c r="U25" s="10">
+        <f t="shared" si="16"/>
+        <v>5219</v>
+      </c>
+      <c r="V25" s="10">
+        <f t="shared" si="16"/>
+        <v>1719</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H26" s="14">
+        <v>2030</v>
+      </c>
+      <c r="I26" s="10">
+        <f t="shared" ref="I26:N26" si="17">I25+I17*5</f>
+        <v>2219</v>
+      </c>
+      <c r="J26" s="10">
+        <f t="shared" si="17"/>
+        <v>3219</v>
+      </c>
+      <c r="K26" s="10">
+        <f t="shared" si="17"/>
+        <v>3219</v>
+      </c>
+      <c r="L26" s="10">
+        <f t="shared" si="17"/>
+        <v>7219</v>
+      </c>
+      <c r="M26" s="10">
+        <f t="shared" si="17"/>
+        <v>2719</v>
+      </c>
+      <c r="N26" s="10">
+        <f t="shared" si="17"/>
+        <v>5719</v>
+      </c>
+      <c r="P26" s="14">
+        <v>2030</v>
+      </c>
+      <c r="Q26" s="10">
+        <f t="shared" ref="Q26:V26" si="18">Q25+Q17*5</f>
+        <v>4719</v>
+      </c>
+      <c r="R26" s="10">
+        <f t="shared" si="18"/>
+        <v>2899</v>
+      </c>
+      <c r="S26" s="10">
+        <f t="shared" si="18"/>
+        <v>5259</v>
+      </c>
+      <c r="T26" s="10">
+        <f t="shared" si="18"/>
+        <v>5219</v>
+      </c>
+      <c r="U26" s="10">
+        <f t="shared" si="18"/>
+        <v>5219</v>
+      </c>
+      <c r="V26" s="10">
+        <f t="shared" si="18"/>
+        <v>10719</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H27" s="14">
+        <v>2035</v>
+      </c>
+      <c r="I27" s="10">
+        <f t="shared" ref="I27:N30" si="19">I26+I18*5</f>
+        <v>2219</v>
+      </c>
+      <c r="J27" s="10">
+        <f t="shared" si="19"/>
+        <v>4719</v>
+      </c>
+      <c r="K27" s="10">
+        <f t="shared" si="19"/>
+        <v>4719</v>
+      </c>
+      <c r="L27" s="10">
+        <f t="shared" si="19"/>
+        <v>9219</v>
+      </c>
+      <c r="M27" s="10">
+        <f t="shared" si="19"/>
+        <v>3219</v>
+      </c>
+      <c r="N27" s="10">
+        <f t="shared" si="19"/>
+        <v>7719</v>
+      </c>
+      <c r="P27" s="14">
+        <v>2035</v>
+      </c>
+      <c r="Q27" s="10">
+        <f t="shared" ref="Q27:V30" si="20">Q26+Q18*5</f>
+        <v>7719</v>
+      </c>
+      <c r="R27" s="10">
+        <f t="shared" si="20"/>
+        <v>3489</v>
+      </c>
+      <c r="S27" s="10">
+        <f t="shared" si="20"/>
+        <v>7029</v>
+      </c>
+      <c r="T27" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="U27" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="V27" s="10">
+        <f t="shared" si="20"/>
+        <v>19719</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H28" s="14">
+        <v>2040</v>
+      </c>
+      <c r="I28" s="10">
+        <f t="shared" si="19"/>
+        <v>2219</v>
+      </c>
+      <c r="J28" s="10">
+        <f t="shared" si="19"/>
+        <v>4719</v>
+      </c>
+      <c r="K28" s="10">
+        <f t="shared" si="19"/>
+        <v>6719</v>
+      </c>
+      <c r="L28" s="10">
+        <f t="shared" si="19"/>
+        <v>10719</v>
+      </c>
+      <c r="M28" s="10">
+        <f t="shared" si="19"/>
+        <v>3719</v>
+      </c>
+      <c r="N28" s="10">
+        <f t="shared" si="19"/>
+        <v>9719</v>
+      </c>
+      <c r="P28" s="14">
+        <v>2040</v>
+      </c>
+      <c r="Q28" s="10">
+        <f t="shared" si="20"/>
+        <v>7719</v>
+      </c>
+      <c r="R28" s="10">
+        <f t="shared" si="20"/>
+        <v>4079</v>
+      </c>
+      <c r="S28" s="10">
+        <f t="shared" si="20"/>
+        <v>8799</v>
+      </c>
+      <c r="T28" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="U28" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="V28" s="10">
+        <f t="shared" si="20"/>
+        <v>19719</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H29" s="14">
+        <v>2045</v>
+      </c>
+      <c r="I29" s="10">
+        <f t="shared" si="19"/>
+        <v>2219</v>
+      </c>
+      <c r="J29" s="10">
+        <f t="shared" si="19"/>
+        <v>4719</v>
+      </c>
+      <c r="K29" s="10">
+        <f t="shared" si="19"/>
+        <v>9219</v>
+      </c>
+      <c r="L29" s="10">
+        <f t="shared" si="19"/>
+        <v>11719</v>
+      </c>
+      <c r="M29" s="10">
+        <f t="shared" si="19"/>
+        <v>4219</v>
+      </c>
+      <c r="N29" s="10">
+        <f t="shared" si="19"/>
+        <v>11719</v>
+      </c>
+      <c r="P29" s="14">
+        <v>2045</v>
+      </c>
+      <c r="Q29" s="10">
+        <f t="shared" si="20"/>
+        <v>7719</v>
+      </c>
+      <c r="R29" s="10">
+        <f t="shared" si="20"/>
+        <v>4669</v>
+      </c>
+      <c r="S29" s="10">
+        <f t="shared" si="20"/>
+        <v>10569</v>
+      </c>
+      <c r="T29" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="U29" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="V29" s="10">
+        <f t="shared" si="20"/>
+        <v>19719</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H30" s="14">
+        <v>2050</v>
+      </c>
+      <c r="I30" s="10">
+        <f t="shared" si="19"/>
+        <v>2219</v>
+      </c>
+      <c r="J30" s="10">
+        <f t="shared" si="19"/>
+        <v>4719</v>
+      </c>
+      <c r="K30" s="10">
+        <f t="shared" si="19"/>
+        <v>12219</v>
+      </c>
+      <c r="L30" s="10">
+        <f t="shared" si="19"/>
+        <v>12219</v>
+      </c>
+      <c r="M30" s="10">
+        <f t="shared" si="19"/>
+        <v>4719</v>
+      </c>
+      <c r="N30" s="10">
+        <f t="shared" si="19"/>
+        <v>13719</v>
+      </c>
+      <c r="P30" s="14">
+        <v>2050</v>
+      </c>
+      <c r="Q30" s="10">
+        <f t="shared" si="20"/>
+        <v>7719</v>
+      </c>
+      <c r="R30" s="10">
+        <f t="shared" si="20"/>
+        <v>5259</v>
+      </c>
+      <c r="S30" s="10">
+        <f t="shared" si="20"/>
+        <v>12339</v>
+      </c>
+      <c r="T30" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="U30" s="10">
+        <f t="shared" si="20"/>
+        <v>5219</v>
+      </c>
+      <c r="V30" s="10">
+        <f t="shared" si="20"/>
+        <v>19719</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H31" s="14"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="P31" s="14"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="10"/>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10"/>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H32" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+      <c r="P32" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q32" s="18"/>
+      <c r="R32" s="18"/>
+      <c r="S32" s="18"/>
+      <c r="T32" s="18"/>
+      <c r="U32" s="18"/>
+      <c r="V32" s="18"/>
+    </row>
+    <row r="33" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H33" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="I33" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="K33" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="L33" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="M33" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="N33" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="P33" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>103</v>
+      </c>
+      <c r="R33" t="s">
+        <v>104</v>
+      </c>
+      <c r="S33" t="s">
+        <v>105</v>
+      </c>
+      <c r="T33" t="s">
+        <v>107</v>
+      </c>
+      <c r="U33" t="s">
+        <v>108</v>
+      </c>
+      <c r="V33" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="34" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H34" s="14">
+        <v>2025</v>
+      </c>
+      <c r="I34" s="10">
         <f>'Baseline Parameters'!G2</f>
         <v>232</v>
       </c>
-      <c r="J25" s="12">
+      <c r="J34" s="10">
         <f>'Baseline Parameters'!B2</f>
         <v>446</v>
       </c>
-      <c r="K25" s="12">
+      <c r="K34" s="10">
         <f>'Baseline Parameters'!C2</f>
         <v>209</v>
       </c>
-      <c r="L25" s="12">
+      <c r="L34" s="10">
         <f>'Baseline Parameters'!E2</f>
         <v>269.98072031209182</v>
       </c>
-      <c r="M25" s="12">
+      <c r="M34" s="10">
         <f>'Baseline Parameters'!F2</f>
         <v>140</v>
       </c>
-      <c r="N25" s="12">
+      <c r="N34" s="10">
         <f>Procurement!J3</f>
         <v>360.50516023732143</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H26" s="18">
+      <c r="P34" s="14">
+        <v>2025</v>
+      </c>
+      <c r="Q34" s="10">
+        <f>$N34</f>
+        <v>360.50516023732143</v>
+      </c>
+      <c r="R34" s="10">
+        <f>$N34</f>
+        <v>360.50516023732143</v>
+      </c>
+      <c r="S34" s="10">
+        <f>$N34</f>
+        <v>360.50516023732143</v>
+      </c>
+      <c r="T34" s="10">
+        <f>J34</f>
+        <v>446</v>
+      </c>
+      <c r="U34" s="10">
+        <f>K34</f>
+        <v>209</v>
+      </c>
+      <c r="V34" s="10">
+        <f>$N34</f>
+        <v>360.50516023732143</v>
+      </c>
+    </row>
+    <row r="35" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H35" s="14">
         <v>2030</v>
       </c>
-      <c r="I26" s="12">
+      <c r="I35" s="10">
         <f>'Baseline Parameters'!G3</f>
         <v>212</v>
       </c>
-      <c r="J26" s="12">
+      <c r="J35" s="10">
         <f>'Baseline Parameters'!B3</f>
         <v>380.16957864810638</v>
       </c>
-      <c r="K26" s="12">
+      <c r="K35" s="10">
         <f>'Baseline Parameters'!C3</f>
         <v>178.15121510639958</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L35" s="10">
         <f>'Baseline Parameters'!E3</f>
         <v>207.95454545454541</v>
       </c>
-      <c r="M26" s="12">
+      <c r="M35" s="10">
         <f>'Baseline Parameters'!F3</f>
         <v>126.10085958575935</v>
       </c>
-      <c r="N26" s="12">
+      <c r="N35" s="10">
         <f>Procurement!J4</f>
         <v>296.81654796345282</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H27" s="18">
+      <c r="P35" s="14">
+        <v>2030</v>
+      </c>
+      <c r="Q35" s="10">
+        <f t="shared" ref="Q35:V39" si="21">$N35</f>
+        <v>296.81654796345282</v>
+      </c>
+      <c r="R35" s="10">
+        <f t="shared" si="21"/>
+        <v>296.81654796345282</v>
+      </c>
+      <c r="S35" s="10">
+        <f t="shared" si="21"/>
+        <v>296.81654796345282</v>
+      </c>
+      <c r="T35" s="10">
+        <f t="shared" ref="T35:T39" si="22">J35</f>
+        <v>380.16957864810638</v>
+      </c>
+      <c r="U35" s="10">
+        <f t="shared" ref="U35:U39" si="23">K35</f>
+        <v>178.15121510639958</v>
+      </c>
+      <c r="V35" s="10">
+        <f t="shared" si="21"/>
+        <v>296.81654796345282</v>
+      </c>
+    </row>
+    <row r="36" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H36" s="14">
         <v>2035</v>
       </c>
-      <c r="I27" s="12">
+      <c r="I36" s="10">
         <f>'Baseline Parameters'!G4</f>
         <v>193.72413793103445</v>
       </c>
-      <c r="J27" s="12">
+      <c r="J36" s="10">
         <f>'Baseline Parameters'!B4</f>
         <v>324.05584872080431</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K36" s="10">
         <f>'Baseline Parameters'!C4</f>
         <v>151.85576767409884</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L36" s="10">
         <f>'Baseline Parameters'!E4</f>
         <v>160.17844876188263</v>
       </c>
-      <c r="M27" s="12">
+      <c r="M36" s="10">
         <f>'Baseline Parameters'!F4</f>
         <v>113.58161991619573</v>
       </c>
-      <c r="N27" s="12">
+      <c r="N36" s="10">
         <f>Procurement!J5</f>
         <v>220.8089461332641</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H28" s="18">
+      <c r="P36" s="14">
+        <v>2035</v>
+      </c>
+      <c r="Q36" s="10">
+        <f t="shared" si="21"/>
+        <v>220.8089461332641</v>
+      </c>
+      <c r="R36" s="10">
+        <f t="shared" si="21"/>
+        <v>220.8089461332641</v>
+      </c>
+      <c r="S36" s="10">
+        <f t="shared" si="21"/>
+        <v>220.8089461332641</v>
+      </c>
+      <c r="T36" s="10">
+        <f t="shared" si="22"/>
+        <v>324.05584872080431</v>
+      </c>
+      <c r="U36" s="10">
+        <f t="shared" si="23"/>
+        <v>151.85576767409884</v>
+      </c>
+      <c r="V36" s="10">
+        <f t="shared" si="21"/>
+        <v>220.8089461332641</v>
+      </c>
+    </row>
+    <row r="37" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H37" s="14">
         <v>2040</v>
       </c>
-      <c r="I28" s="12">
+      <c r="I37" s="10">
         <f>'Baseline Parameters'!G5</f>
         <v>177.02378121284181</v>
       </c>
-      <c r="J28" s="12">
+      <c r="J37" s="10">
         <f>'Baseline Parameters'!B5</f>
         <v>276.22460866960239</v>
       </c>
-      <c r="K28" s="12">
+      <c r="K37" s="10">
         <f>'Baseline Parameters'!C5</f>
         <v>129.4415767084011</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L37" s="10">
         <f>'Baseline Parameters'!E5</f>
         <v>123.37857483077323</v>
       </c>
-      <c r="M28" s="12">
+      <c r="M37" s="10">
         <f>'Baseline Parameters'!F5</f>
         <v>102.30528503268064</v>
       </c>
-      <c r="N28" s="12">
+      <c r="N37" s="10">
         <f>Procurement!J6</f>
         <v>202.50547416626196</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H29" s="18">
+      <c r="P37" s="14">
+        <v>2040</v>
+      </c>
+      <c r="Q37" s="10">
+        <f t="shared" si="21"/>
+        <v>202.50547416626196</v>
+      </c>
+      <c r="R37" s="10">
+        <f t="shared" si="21"/>
+        <v>202.50547416626196</v>
+      </c>
+      <c r="S37" s="10">
+        <f t="shared" si="21"/>
+        <v>202.50547416626196</v>
+      </c>
+      <c r="T37" s="10">
+        <f t="shared" si="22"/>
+        <v>276.22460866960239</v>
+      </c>
+      <c r="U37" s="10">
+        <f t="shared" si="23"/>
+        <v>129.4415767084011</v>
+      </c>
+      <c r="V37" s="10">
+        <f t="shared" si="21"/>
+        <v>202.50547416626196</v>
+      </c>
+    </row>
+    <row r="38" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H38" s="14">
         <v>2045</v>
       </c>
-      <c r="I29" s="12">
+      <c r="I38" s="10">
         <f>'Baseline Parameters'!G6</f>
         <v>161.7631104186313</v>
       </c>
-      <c r="J29" s="12">
+      <c r="J38" s="10">
         <f>'Baseline Parameters'!B6</f>
         <v>235.45334773578654</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K38" s="10">
         <f>'Baseline Parameters'!C6</f>
         <v>110.33576160712865</v>
       </c>
-      <c r="L29" s="12">
+      <c r="L38" s="10">
         <f>'Baseline Parameters'!E6</f>
         <v>95.033213549856328</v>
       </c>
-      <c r="M29" s="12">
+      <c r="M38" s="10">
         <f>'Baseline Parameters'!F6</f>
         <v>92.14845987705111</v>
       </c>
-      <c r="N29" s="12">
+      <c r="N38" s="10">
         <f>Procurement!J7</f>
         <v>184.65112037257458</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H30" s="18">
+      <c r="P38" s="14">
+        <v>2045</v>
+      </c>
+      <c r="Q38" s="10">
+        <f t="shared" si="21"/>
+        <v>184.65112037257458</v>
+      </c>
+      <c r="R38" s="10">
+        <f t="shared" si="21"/>
+        <v>184.65112037257458</v>
+      </c>
+      <c r="S38" s="10">
+        <f t="shared" si="21"/>
+        <v>184.65112037257458</v>
+      </c>
+      <c r="T38" s="10">
+        <f t="shared" si="22"/>
+        <v>235.45334773578654</v>
+      </c>
+      <c r="U38" s="10">
+        <f t="shared" si="23"/>
+        <v>110.33576160712865</v>
+      </c>
+      <c r="V38" s="10">
+        <f t="shared" si="21"/>
+        <v>184.65112037257458</v>
+      </c>
+    </row>
+    <row r="39" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H39" s="14">
         <v>2050</v>
       </c>
-      <c r="I30" s="12">
+      <c r="I39" s="10">
         <f>'Baseline Parameters'!G7</f>
         <v>147.8180146928872</v>
       </c>
-      <c r="J30" s="12">
+      <c r="J39" s="10">
         <f>'Baseline Parameters'!B7</f>
         <v>200.70000000000002</v>
       </c>
-      <c r="K30" s="12">
+      <c r="K39" s="10">
         <f>'Baseline Parameters'!C7</f>
         <v>94.05</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L39" s="10">
         <f>'Baseline Parameters'!E7</f>
         <v>73.199999999999989</v>
       </c>
-      <c r="M30" s="12">
+      <c r="M39" s="10">
         <f>'Baseline Parameters'!F7</f>
         <v>83</v>
       </c>
-      <c r="N30" s="12">
+      <c r="N39" s="10">
         <f>Procurement!J8</f>
         <v>172.93379856211703</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H31" s="18"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-      <c r="L31" s="12"/>
-      <c r="M31" s="12"/>
-      <c r="N31" s="12"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H32" s="13" t="s">
+      <c r="P39" s="14">
+        <v>2050</v>
+      </c>
+      <c r="Q39" s="10">
+        <f t="shared" si="21"/>
+        <v>172.93379856211703</v>
+      </c>
+      <c r="R39" s="10">
+        <f t="shared" si="21"/>
+        <v>172.93379856211703</v>
+      </c>
+      <c r="S39" s="10">
+        <f t="shared" si="21"/>
+        <v>172.93379856211703</v>
+      </c>
+      <c r="T39" s="10">
+        <f t="shared" si="22"/>
+        <v>200.70000000000002</v>
+      </c>
+      <c r="U39" s="10">
+        <f t="shared" si="23"/>
+        <v>94.05</v>
+      </c>
+      <c r="V39" s="10">
+        <f t="shared" si="21"/>
+        <v>172.93379856211703</v>
+      </c>
+    </row>
+    <row r="40" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H40" s="14"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="P40" s="14"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="10"/>
+      <c r="S40" s="10"/>
+      <c r="T40" s="10"/>
+      <c r="U40" s="10"/>
+      <c r="V40" s="10"/>
+    </row>
+    <row r="41" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H41" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="I41" s="18"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="18"/>
+      <c r="M41" s="18"/>
+      <c r="N41" s="18"/>
+      <c r="P41" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q41" s="18"/>
+      <c r="R41" s="18"/>
+      <c r="S41" s="18"/>
+      <c r="T41" s="18"/>
+      <c r="U41" s="18"/>
+      <c r="V41" s="18"/>
+    </row>
+    <row r="42" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H42" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="I42" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J42" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="K42" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="L42" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="M42" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="N42" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="P42" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>103</v>
+      </c>
+      <c r="R42" t="s">
+        <v>104</v>
+      </c>
+      <c r="S42" t="s">
+        <v>105</v>
+      </c>
+      <c r="T42" t="s">
+        <v>107</v>
+      </c>
+      <c r="U42" t="s">
+        <v>108</v>
+      </c>
+      <c r="V42" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H43" s="14">
+        <v>2025</v>
+      </c>
+      <c r="I43" s="10">
+        <f t="shared" ref="I43:N48" si="24">I7*I25^I$3</f>
+        <v>227.65791780169334</v>
+      </c>
+      <c r="J43" s="10">
+        <f t="shared" si="24"/>
+        <v>446</v>
+      </c>
+      <c r="K43" s="10">
+        <f t="shared" si="24"/>
+        <v>205.08838284721514</v>
+      </c>
+      <c r="L43" s="10">
+        <f t="shared" si="24"/>
+        <v>250.54068948498627</v>
+      </c>
+      <c r="M43" s="10">
+        <f t="shared" si="24"/>
+        <v>137.37977798378049</v>
+      </c>
+      <c r="N43" s="10">
+        <f t="shared" si="24"/>
+        <v>340.49470546798307</v>
+      </c>
+      <c r="P43" s="14">
+        <v>2025</v>
+      </c>
+      <c r="Q43" s="10">
+        <f t="shared" ref="Q43:V48" si="25">Q7*Q25^Q$3</f>
+        <v>360.50516023732143</v>
+      </c>
+      <c r="R43" s="10">
+        <f t="shared" si="25"/>
+        <v>352.71873592109205</v>
+      </c>
+      <c r="S43" s="10">
+        <f t="shared" si="25"/>
+        <v>342.107053662032</v>
+      </c>
+      <c r="T43" s="10">
+        <f t="shared" si="25"/>
+        <v>410.81265512816464</v>
+      </c>
+      <c r="U43" s="10">
+        <f t="shared" si="25"/>
+        <v>192.51086305333277</v>
+      </c>
+      <c r="V43" s="10">
+        <f t="shared" si="25"/>
+        <v>360.50516023732143</v>
+      </c>
+    </row>
+    <row r="44" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H44" s="14">
+        <v>2030</v>
+      </c>
+      <c r="I44" s="10">
+        <f t="shared" si="24"/>
+        <v>208.03223523258188</v>
+      </c>
+      <c r="J44" s="10">
+        <f t="shared" si="24"/>
+        <v>362.92461439647064</v>
+      </c>
+      <c r="K44" s="10">
+        <f t="shared" si="24"/>
+        <v>170.07005472839089</v>
+      </c>
+      <c r="L44" s="10">
+        <f t="shared" si="24"/>
+        <v>187.00427351359522</v>
+      </c>
+      <c r="M44" s="10">
+        <f t="shared" si="24"/>
+        <v>121.89395837797517</v>
+      </c>
+      <c r="N44" s="10">
+        <f t="shared" si="24"/>
+        <v>271.5543959414494</v>
+      </c>
+      <c r="P44" s="14">
+        <v>2030</v>
+      </c>
+      <c r="Q44" s="10">
+        <f t="shared" si="25"/>
+        <v>275.44419650170983</v>
+      </c>
+      <c r="R44" s="10">
+        <f t="shared" si="25"/>
+        <v>285.55657003285313</v>
+      </c>
+      <c r="S44" s="10">
+        <f t="shared" si="25"/>
+        <v>273.24466425259618</v>
+      </c>
+      <c r="T44" s="10">
+        <f t="shared" si="25"/>
+        <v>350.17595068023365</v>
+      </c>
+      <c r="U44" s="10">
+        <f t="shared" si="25"/>
+        <v>164.09590513939193</v>
+      </c>
+      <c r="V44" s="10">
+        <f t="shared" si="25"/>
+        <v>259.2191658004752</v>
+      </c>
+    </row>
+    <row r="45" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H45" s="14">
+        <v>2035</v>
+      </c>
+      <c r="I45" s="10">
+        <f t="shared" si="24"/>
+        <v>190.09842185046273</v>
+      </c>
+      <c r="J45" s="10">
+        <f t="shared" si="24"/>
+        <v>300.72212444021858</v>
+      </c>
+      <c r="K45" s="10">
+        <f t="shared" si="24"/>
+        <v>140.92135427803959</v>
+      </c>
+      <c r="L45" s="10">
+        <f t="shared" si="24"/>
+        <v>141.45812458337952</v>
+      </c>
+      <c r="M45" s="10">
+        <f t="shared" si="24"/>
+        <v>108.4294165703549</v>
+      </c>
+      <c r="N45" s="10">
+        <f t="shared" si="24"/>
+        <v>197.58208444082797</v>
+      </c>
+      <c r="P45" s="14">
+        <v>2035</v>
+      </c>
+      <c r="Q45" s="10">
+        <f t="shared" si="25"/>
+        <v>197.58208444082797</v>
+      </c>
+      <c r="R45" s="10">
+        <f t="shared" si="25"/>
+        <v>209.54012956192068</v>
+      </c>
+      <c r="S45" s="10">
+        <f t="shared" si="25"/>
+        <v>198.9559618656977</v>
+      </c>
+      <c r="T45" s="10">
+        <f t="shared" si="25"/>
+        <v>298.48933547714006</v>
+      </c>
+      <c r="U45" s="10">
+        <f t="shared" si="25"/>
+        <v>139.8750473424266</v>
+      </c>
+      <c r="V45" s="10">
+        <f t="shared" si="25"/>
+        <v>184.33406406551856</v>
+      </c>
+    </row>
+    <row r="46" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H46" s="14">
+        <v>2040</v>
+      </c>
+      <c r="I46" s="10">
+        <f t="shared" si="24"/>
+        <v>173.71062686335384</v>
+      </c>
+      <c r="J46" s="10">
+        <f t="shared" si="24"/>
+        <v>256.33498506412843</v>
+      </c>
+      <c r="K46" s="10">
+        <f t="shared" si="24"/>
+        <v>117.02096248366335</v>
+      </c>
+      <c r="L46" s="10">
+        <f t="shared" si="24"/>
+        <v>107.75036454241936</v>
+      </c>
+      <c r="M46" s="10">
+        <f t="shared" si="24"/>
+        <v>96.62665541899338</v>
+      </c>
+      <c r="N46" s="10">
+        <f t="shared" si="24"/>
+        <v>178.14071267621432</v>
+      </c>
+      <c r="P46" s="14">
+        <v>2040</v>
+      </c>
+      <c r="Q46" s="10">
+        <f t="shared" si="25"/>
+        <v>181.20395209123592</v>
+      </c>
+      <c r="R46" s="10">
+        <f t="shared" si="25"/>
+        <v>189.9617703421664</v>
+      </c>
+      <c r="S46" s="10">
+        <f t="shared" si="25"/>
+        <v>179.45646847078069</v>
+      </c>
+      <c r="T46" s="10">
+        <f t="shared" si="25"/>
+        <v>254.43175986389599</v>
+      </c>
+      <c r="U46" s="10">
+        <f t="shared" si="25"/>
+        <v>119.22923276133241</v>
+      </c>
+      <c r="V46" s="10">
+        <f t="shared" si="25"/>
+        <v>169.05409722871059</v>
+      </c>
+    </row>
+    <row r="47" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H47" s="14">
+        <v>2045</v>
+      </c>
+      <c r="I47" s="10">
+        <f t="shared" si="24"/>
+        <v>158.73557282340954</v>
+      </c>
+      <c r="J47" s="10">
+        <f t="shared" si="24"/>
+        <v>218.49946920313531</v>
+      </c>
+      <c r="K47" s="10">
+        <f t="shared" si="24"/>
+        <v>97.440635941140712</v>
+      </c>
+      <c r="L47" s="10">
+        <f t="shared" si="24"/>
+        <v>82.449481539281351</v>
+      </c>
+      <c r="M47" s="10">
+        <f t="shared" si="24"/>
+        <v>86.224957908187065</v>
+      </c>
+      <c r="N47" s="10">
+        <f t="shared" si="24"/>
+        <v>160.20071900840423</v>
+      </c>
+      <c r="P47" s="14">
+        <v>2045</v>
+      </c>
+      <c r="Q47" s="10">
+        <f t="shared" si="25"/>
+        <v>165.2276952380752</v>
+      </c>
+      <c r="R47" s="10">
+        <f t="shared" si="25"/>
+        <v>171.49039287198505</v>
+      </c>
+      <c r="S47" s="10">
+        <f t="shared" si="25"/>
+        <v>161.42985382479438</v>
+      </c>
+      <c r="T47" s="10">
+        <f t="shared" si="25"/>
+        <v>216.87716354742938</v>
+      </c>
+      <c r="U47" s="10">
+        <f t="shared" si="25"/>
+        <v>101.63077843366084</v>
+      </c>
+      <c r="V47" s="10">
+        <f t="shared" si="25"/>
+        <v>154.14905984826089</v>
+      </c>
+    </row>
+    <row r="48" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H48" s="14">
+        <v>2050</v>
+      </c>
+      <c r="I48" s="10">
+        <f t="shared" si="24"/>
+        <v>145.05147171794317</v>
+      </c>
+      <c r="J48" s="10">
+        <f t="shared" si="24"/>
+        <v>186.24854516096593</v>
+      </c>
+      <c r="K48" s="10">
+        <f t="shared" si="24"/>
+        <v>81.344571464021328</v>
+      </c>
+      <c r="L48" s="10">
+        <f t="shared" si="24"/>
+        <v>63.311245413783745</v>
+      </c>
+      <c r="M48" s="10">
+        <f t="shared" si="24"/>
+        <v>77.023563768610728</v>
+      </c>
+      <c r="N48" s="10">
+        <f t="shared" si="24"/>
+        <v>148.29565759240268</v>
+      </c>
+      <c r="P48" s="14">
+        <v>2050</v>
+      </c>
+      <c r="Q48" s="10">
+        <f t="shared" si="25"/>
+        <v>154.74291684518829</v>
+      </c>
+      <c r="R48" s="10">
+        <f t="shared" si="25"/>
+        <v>159.200145848506</v>
+      </c>
+      <c r="S48" s="10">
+        <f t="shared" si="25"/>
+        <v>149.46364819523117</v>
+      </c>
+      <c r="T48" s="10">
+        <f t="shared" si="25"/>
+        <v>184.86569480767412</v>
+      </c>
+      <c r="U48" s="10">
+        <f t="shared" si="25"/>
+        <v>86.629888373999734</v>
+      </c>
+      <c r="V48" s="10">
+        <f t="shared" si="25"/>
+        <v>144.36729336140115</v>
+      </c>
+    </row>
+    <row r="49" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H49" s="14"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
+      <c r="L49" s="10"/>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
+      <c r="P49" s="14"/>
+      <c r="Q49" s="10"/>
+      <c r="R49" s="10"/>
+      <c r="S49" s="10"/>
+      <c r="T49" s="10"/>
+      <c r="U49" s="10"/>
+      <c r="V49" s="10"/>
+    </row>
+    <row r="50" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H50" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="13"/>
-      <c r="M32" s="13"/>
-      <c r="N32" s="13"/>
-    </row>
-    <row r="33" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H33" s="18" t="s">
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18"/>
+      <c r="N50" s="18"/>
+      <c r="P50" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q50" s="18"/>
+      <c r="R50" s="18"/>
+      <c r="S50" s="18"/>
+      <c r="T50" s="18"/>
+      <c r="U50" s="18"/>
+      <c r="V50" s="18"/>
+    </row>
+    <row r="51" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H51" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="I33" s="12" t="s">
+      <c r="I51" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J33" s="12" t="s">
+      <c r="J51" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="K33" s="12" t="s">
+      <c r="K51" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="L33" s="12" t="s">
+      <c r="L51" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="M33" s="12" t="s">
+      <c r="M51" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="N33" s="12" t="s">
+      <c r="N51" s="10" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="34" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H34" s="18">
+      <c r="P51" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>103</v>
+      </c>
+      <c r="R51" t="s">
+        <v>104</v>
+      </c>
+      <c r="S51" t="s">
+        <v>105</v>
+      </c>
+      <c r="T51" t="s">
+        <v>107</v>
+      </c>
+      <c r="U51" t="s">
+        <v>108</v>
+      </c>
+      <c r="V51" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="52" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H52" s="14">
         <v>2025</v>
       </c>
-      <c r="I34" s="12">
-        <f>Q7*I16^I$3</f>
-        <v>228.8909241816344</v>
-      </c>
-      <c r="J34" s="12">
-        <f t="shared" ref="J34:N39" si="12">R7*J16^J$3</f>
-        <v>446</v>
-      </c>
-      <c r="K34" s="12">
-        <f t="shared" si="12"/>
-        <v>206.19915152569649</v>
-      </c>
-      <c r="L34" s="12">
-        <f t="shared" si="12"/>
-        <v>254.67919785643252</v>
-      </c>
-      <c r="M34" s="12">
-        <f t="shared" si="12"/>
-        <v>138.12383355788282</v>
-      </c>
-      <c r="N34" s="12">
-        <f t="shared" si="12"/>
-        <v>345.16068338004146</v>
-      </c>
-    </row>
-    <row r="35" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H35" s="18">
+      <c r="I52" s="10">
+        <f>I34-I43</f>
+        <v>4.342082198306656</v>
+      </c>
+      <c r="J52" s="10">
+        <f t="shared" ref="J52:N52" si="26">J34-J43</f>
+        <v>0</v>
+      </c>
+      <c r="K52" s="10">
+        <f t="shared" si="26"/>
+        <v>3.9116171527848564</v>
+      </c>
+      <c r="L52" s="10">
+        <f t="shared" si="26"/>
+        <v>19.440030827105545</v>
+      </c>
+      <c r="M52" s="10">
+        <f t="shared" si="26"/>
+        <v>2.6202220162195147</v>
+      </c>
+      <c r="N52" s="10">
+        <f t="shared" si="26"/>
+        <v>20.010454769338367</v>
+      </c>
+      <c r="P52" s="14">
+        <v>2025</v>
+      </c>
+      <c r="Q52" s="10">
+        <f>Q34-Q43</f>
+        <v>0</v>
+      </c>
+      <c r="R52" s="10">
+        <f t="shared" ref="R52:V52" si="27">R34-R43</f>
+        <v>7.786424316229386</v>
+      </c>
+      <c r="S52" s="10">
+        <f t="shared" si="27"/>
+        <v>18.398106575289432</v>
+      </c>
+      <c r="T52" s="10">
+        <f t="shared" si="27"/>
+        <v>35.187344871835364</v>
+      </c>
+      <c r="U52" s="10">
+        <f t="shared" si="27"/>
+        <v>16.48913694666723</v>
+      </c>
+      <c r="V52" s="10">
+        <f t="shared" si="27"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H53" s="14">
         <v>2030</v>
       </c>
-      <c r="I35" s="12">
-        <f t="shared" ref="I35:I39" si="13">Q8*I17^I$3</f>
-        <v>209.15894795907971</v>
-      </c>
-      <c r="J35" s="12">
-        <f t="shared" si="12"/>
-        <v>367.17447515029585</v>
-      </c>
-      <c r="K35" s="12">
-        <f t="shared" si="12"/>
-        <v>172.0615814045108</v>
-      </c>
-      <c r="L35" s="12">
-        <f t="shared" si="12"/>
-        <v>190.80393155301951</v>
-      </c>
-      <c r="M35" s="12">
-        <f t="shared" si="12"/>
-        <v>122.99984732811295</v>
-      </c>
-      <c r="N35" s="12">
-        <f t="shared" si="12"/>
-        <v>276.55408770473178</v>
-      </c>
-    </row>
-    <row r="36" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H36" s="18">
+      <c r="I53" s="10">
+        <f t="shared" ref="I53:N57" si="28">I35-I44</f>
+        <v>3.9677647674181173</v>
+      </c>
+      <c r="J53" s="10">
+        <f t="shared" si="28"/>
+        <v>17.244964251635736</v>
+      </c>
+      <c r="K53" s="10">
+        <f t="shared" si="28"/>
+        <v>8.0811603780086898</v>
+      </c>
+      <c r="L53" s="10">
+        <f t="shared" si="28"/>
+        <v>20.950271940950188</v>
+      </c>
+      <c r="M53" s="10">
+        <f t="shared" si="28"/>
+        <v>4.2069012077841847</v>
+      </c>
+      <c r="N53" s="10">
+        <f t="shared" si="28"/>
+        <v>25.26215202200342</v>
+      </c>
+      <c r="P53" s="14">
+        <v>2030</v>
+      </c>
+      <c r="Q53" s="10">
+        <f t="shared" ref="Q53:V53" si="29">Q35-Q44</f>
+        <v>21.372351461742994</v>
+      </c>
+      <c r="R53" s="10">
+        <f t="shared" si="29"/>
+        <v>11.259977930599689</v>
+      </c>
+      <c r="S53" s="10">
+        <f t="shared" si="29"/>
+        <v>23.571883710856639</v>
+      </c>
+      <c r="T53" s="10">
+        <f t="shared" si="29"/>
+        <v>29.993627967872726</v>
+      </c>
+      <c r="U53" s="10">
+        <f t="shared" si="29"/>
+        <v>14.055309967007645</v>
+      </c>
+      <c r="V53" s="10">
+        <f t="shared" si="29"/>
+        <v>37.597382162977624</v>
+      </c>
+    </row>
+    <row r="54" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H54" s="14">
         <v>2035</v>
       </c>
-      <c r="I36" s="12">
-        <f t="shared" si="13"/>
-        <v>191.12800416950384</v>
-      </c>
-      <c r="J36" s="12">
-        <f t="shared" si="12"/>
-        <v>305.68954522936554</v>
-      </c>
-      <c r="K36" s="12">
-        <f t="shared" si="12"/>
-        <v>143.24913666577888</v>
-      </c>
-      <c r="L36" s="12">
-        <f t="shared" si="12"/>
-        <v>144.56116653140265</v>
-      </c>
-      <c r="M36" s="12">
-        <f t="shared" si="12"/>
-        <v>109.69912907747937</v>
-      </c>
-      <c r="N36" s="12">
-        <f t="shared" si="12"/>
-        <v>201.69132781051039</v>
-      </c>
-    </row>
-    <row r="37" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H37" s="18">
+      <c r="I54" s="10">
+        <f t="shared" si="28"/>
+        <v>3.6257160805717206</v>
+      </c>
+      <c r="J54" s="10">
+        <f t="shared" si="28"/>
+        <v>23.333724280585727</v>
+      </c>
+      <c r="K54" s="10">
+        <f t="shared" si="28"/>
+        <v>10.934413396059256</v>
+      </c>
+      <c r="L54" s="10">
+        <f t="shared" si="28"/>
+        <v>18.72032417850312</v>
+      </c>
+      <c r="M54" s="10">
+        <f t="shared" si="28"/>
+        <v>5.1522033458408316</v>
+      </c>
+      <c r="N54" s="10">
+        <f t="shared" si="28"/>
+        <v>23.226861692436131</v>
+      </c>
+      <c r="P54" s="14">
+        <v>2035</v>
+      </c>
+      <c r="Q54" s="10">
+        <f t="shared" ref="Q54:V54" si="30">Q36-Q45</f>
+        <v>23.226861692436131</v>
+      </c>
+      <c r="R54" s="10">
+        <f t="shared" si="30"/>
+        <v>11.268816571343422</v>
+      </c>
+      <c r="S54" s="10">
+        <f t="shared" si="30"/>
+        <v>21.852984267566399</v>
+      </c>
+      <c r="T54" s="10">
+        <f t="shared" si="30"/>
+        <v>25.566513243664247</v>
+      </c>
+      <c r="U54" s="10">
+        <f t="shared" si="30"/>
+        <v>11.980720331672245</v>
+      </c>
+      <c r="V54" s="10">
+        <f t="shared" si="30"/>
+        <v>36.47488206774554</v>
+      </c>
+    </row>
+    <row r="55" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H55" s="14">
         <v>2040</v>
       </c>
-      <c r="I37" s="12">
-        <f t="shared" si="13"/>
-        <v>174.65145208592588</v>
-      </c>
-      <c r="J37" s="12">
-        <f t="shared" si="12"/>
-        <v>260.56920539681425</v>
-      </c>
-      <c r="K37" s="12">
-        <f t="shared" si="12"/>
-        <v>119.33472084678709</v>
-      </c>
-      <c r="L37" s="12">
-        <f t="shared" si="12"/>
-        <v>110.20357158277476</v>
-      </c>
-      <c r="M37" s="12">
-        <f t="shared" si="12"/>
-        <v>97.950781264889969</v>
-      </c>
-      <c r="N37" s="12">
-        <f t="shared" si="12"/>
-        <v>182.1026727916458</v>
-      </c>
-    </row>
-    <row r="38" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H38" s="18">
+      <c r="I55" s="10">
+        <f t="shared" si="28"/>
+        <v>3.3131543494879736</v>
+      </c>
+      <c r="J55" s="10">
+        <f t="shared" si="28"/>
+        <v>19.889623605473957</v>
+      </c>
+      <c r="K55" s="10">
+        <f t="shared" si="28"/>
+        <v>12.420614224737747</v>
+      </c>
+      <c r="L55" s="10">
+        <f t="shared" si="28"/>
+        <v>15.62821028835387</v>
+      </c>
+      <c r="M55" s="10">
+        <f t="shared" si="28"/>
+        <v>5.6786296136872636</v>
+      </c>
+      <c r="N55" s="10">
+        <f t="shared" si="28"/>
+        <v>24.364761490047641</v>
+      </c>
+      <c r="P55" s="14">
+        <v>2040</v>
+      </c>
+      <c r="Q55" s="10">
+        <f t="shared" ref="Q55:V55" si="31">Q37-Q46</f>
+        <v>21.301522075026043</v>
+      </c>
+      <c r="R55" s="10">
+        <f t="shared" si="31"/>
+        <v>12.543703824095559</v>
+      </c>
+      <c r="S55" s="10">
+        <f t="shared" si="31"/>
+        <v>23.04900569548127</v>
+      </c>
+      <c r="T55" s="10">
+        <f t="shared" si="31"/>
+        <v>21.792848805706399</v>
+      </c>
+      <c r="U55" s="10">
+        <f t="shared" si="31"/>
+        <v>10.212343947068689</v>
+      </c>
+      <c r="V55" s="10">
+        <f t="shared" si="31"/>
+        <v>33.451376937551373</v>
+      </c>
+    </row>
+    <row r="56" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H56" s="14">
         <v>2045</v>
       </c>
-      <c r="I38" s="12">
-        <f t="shared" si="13"/>
-        <v>159.59529242334608</v>
-      </c>
-      <c r="J38" s="12">
-        <f t="shared" si="12"/>
-        <v>222.10871081699267</v>
-      </c>
-      <c r="K38" s="12">
-        <f t="shared" si="12"/>
-        <v>99.578105115554848</v>
-      </c>
-      <c r="L38" s="12">
-        <f t="shared" si="12"/>
-        <v>84.362926134929509</v>
-      </c>
-      <c r="M38" s="12">
-        <f t="shared" si="12"/>
-        <v>87.541072164529638</v>
-      </c>
-      <c r="N38" s="12">
-        <f t="shared" si="12"/>
-        <v>163.91857380000212</v>
-      </c>
-    </row>
-    <row r="39" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H39" s="18">
+      <c r="I56" s="10">
+        <f t="shared" si="28"/>
+        <v>3.0275375952217587</v>
+      </c>
+      <c r="J56" s="10">
+        <f t="shared" si="28"/>
+        <v>16.953878532651231</v>
+      </c>
+      <c r="K56" s="10">
+        <f t="shared" si="28"/>
+        <v>12.895125665987933</v>
+      </c>
+      <c r="L56" s="10">
+        <f t="shared" si="28"/>
+        <v>12.583732010574977</v>
+      </c>
+      <c r="M56" s="10">
+        <f t="shared" si="28"/>
+        <v>5.9235019688640449</v>
+      </c>
+      <c r="N56" s="10">
+        <f t="shared" si="28"/>
+        <v>24.450401364170347</v>
+      </c>
+      <c r="P56" s="14">
+        <v>2045</v>
+      </c>
+      <c r="Q56" s="10">
+        <f t="shared" ref="Q56:V56" si="32">Q38-Q47</f>
+        <v>19.423425134499382</v>
+      </c>
+      <c r="R56" s="10">
+        <f t="shared" si="32"/>
+        <v>13.16072750058953</v>
+      </c>
+      <c r="S56" s="10">
+        <f t="shared" si="32"/>
+        <v>23.221266547780203</v>
+      </c>
+      <c r="T56" s="10">
+        <f t="shared" si="32"/>
+        <v>18.576184188357161</v>
+      </c>
+      <c r="U56" s="10">
+        <f t="shared" si="32"/>
+        <v>8.7049831734678094</v>
+      </c>
+      <c r="V56" s="10">
+        <f t="shared" si="32"/>
+        <v>30.502060524313691</v>
+      </c>
+    </row>
+    <row r="57" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H57" s="14">
         <v>2050</v>
       </c>
-      <c r="I39" s="12">
-        <f t="shared" si="13"/>
-        <v>145.83707755926449</v>
-      </c>
-      <c r="J39" s="12">
-        <f t="shared" si="12"/>
-        <v>189.32505606585244</v>
-      </c>
-      <c r="K39" s="12">
-        <f t="shared" si="12"/>
-        <v>83.24814259608965</v>
-      </c>
-      <c r="L39" s="12">
-        <f t="shared" si="12"/>
-        <v>64.792812738264345</v>
-      </c>
-      <c r="M39" s="12">
-        <f t="shared" si="12"/>
-        <v>78.295862747711766</v>
-      </c>
-      <c r="N39" s="12">
-        <f t="shared" si="12"/>
-        <v>151.84000504571642</v>
-      </c>
-    </row>
-    <row r="40" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H40" s="18"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
-      <c r="L40" s="12"/>
-      <c r="M40" s="12"/>
-      <c r="N40" s="12"/>
-    </row>
-    <row r="41" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H41" s="13" t="s">
+      <c r="I57" s="10">
+        <f t="shared" si="28"/>
+        <v>2.7665429749440307</v>
+      </c>
+      <c r="J57" s="10">
+        <f t="shared" si="28"/>
+        <v>14.451454839034085</v>
+      </c>
+      <c r="K57" s="10">
+        <f t="shared" si="28"/>
+        <v>12.705428535978669</v>
+      </c>
+      <c r="L57" s="10">
+        <f t="shared" si="28"/>
+        <v>9.888754586216244</v>
+      </c>
+      <c r="M57" s="10">
+        <f t="shared" si="28"/>
+        <v>5.9764362313892718</v>
+      </c>
+      <c r="N57" s="10">
+        <f t="shared" si="28"/>
+        <v>24.638140969714357</v>
+      </c>
+      <c r="P57" s="14">
+        <v>2050</v>
+      </c>
+      <c r="Q57" s="10">
+        <f t="shared" ref="Q57:V57" si="33">Q39-Q48</f>
+        <v>18.190881716928743</v>
+      </c>
+      <c r="R57" s="10">
+        <f t="shared" si="33"/>
+        <v>13.733652713611036</v>
+      </c>
+      <c r="S57" s="10">
+        <f t="shared" si="33"/>
+        <v>23.470150366885861</v>
+      </c>
+      <c r="T57" s="10">
+        <f t="shared" si="33"/>
+        <v>15.8343051923259</v>
+      </c>
+      <c r="U57" s="10">
+        <f t="shared" si="33"/>
+        <v>7.4201116260002635</v>
+      </c>
+      <c r="V57" s="10">
+        <f t="shared" si="33"/>
+        <v>28.566505200715881</v>
+      </c>
+    </row>
+    <row r="58" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="P58" s="13"/>
+    </row>
+    <row r="59" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H59" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="I41" s="13"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="13"/>
-      <c r="L41" s="13"/>
-      <c r="M41" s="13"/>
-      <c r="N41" s="13"/>
-    </row>
-    <row r="42" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H42" s="18" t="s">
+      <c r="I59" s="18"/>
+      <c r="J59" s="18"/>
+      <c r="K59" s="18"/>
+      <c r="L59" s="18"/>
+      <c r="M59" s="18"/>
+      <c r="N59" s="18"/>
+      <c r="P59" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q59" s="18"/>
+      <c r="R59" s="18"/>
+      <c r="S59" s="18"/>
+      <c r="T59" s="18"/>
+      <c r="U59" s="18"/>
+      <c r="V59" s="18"/>
+    </row>
+    <row r="60" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H60" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="I42" s="12" t="s">
+      <c r="I60" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J42" s="12" t="s">
+      <c r="J60" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="K42" s="12" t="s">
+      <c r="K60" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="L42" s="12" t="s">
+      <c r="L60" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="M42" s="12" t="s">
+      <c r="M60" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="N42" s="12" t="s">
+      <c r="N60" s="10" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="43" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H43" s="18">
+      <c r="P60" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>103</v>
+      </c>
+      <c r="R60" t="s">
+        <v>104</v>
+      </c>
+      <c r="S60" t="s">
+        <v>105</v>
+      </c>
+      <c r="T60" t="s">
+        <v>107</v>
+      </c>
+      <c r="U60" t="s">
+        <v>108</v>
+      </c>
+      <c r="V60" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="61" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H61" s="14">
         <v>2025</v>
       </c>
-      <c r="I43" s="12">
-        <f>I25-I34</f>
-        <v>3.1090758183655964</v>
-      </c>
-      <c r="J43" s="12">
-        <f t="shared" ref="J43:N43" si="14">J25-J34</f>
+      <c r="I61" s="15">
+        <f>(1-(I52/I34))/I34</f>
+        <v>4.2296729674809255E-3</v>
+      </c>
+      <c r="J61" s="15">
+        <f t="shared" ref="J61:N61" si="34">(1-(J52/J34))/J34</f>
+        <v>2.242152466367713E-3</v>
+      </c>
+      <c r="K61" s="15">
+        <f t="shared" si="34"/>
+        <v>4.6951393706008366E-3</v>
+      </c>
+      <c r="L61" s="15">
+        <f t="shared" si="34"/>
+        <v>3.4372630131788207E-3</v>
+      </c>
+      <c r="M61" s="15">
+        <f t="shared" si="34"/>
+        <v>7.0091723461112492E-3</v>
+      </c>
+      <c r="N61" s="15">
+        <f t="shared" si="34"/>
+        <v>2.6199161506589817E-3</v>
+      </c>
+      <c r="P61" s="14">
+        <v>2025</v>
+      </c>
+      <c r="Q61" s="15">
+        <f t="shared" ref="Q61:V66" si="35">Q52/Q34</f>
         <v>0</v>
       </c>
-      <c r="K43" s="12">
-        <f t="shared" si="14"/>
-        <v>2.8008484743035069</v>
-      </c>
-      <c r="L43" s="12">
-        <f t="shared" si="14"/>
-        <v>15.301522455659295</v>
-      </c>
-      <c r="M43" s="12">
-        <f t="shared" si="14"/>
-        <v>1.8761664421171815</v>
-      </c>
-      <c r="N43" s="12">
-        <f t="shared" si="14"/>
-        <v>15.344476857279972</v>
-      </c>
-    </row>
-    <row r="44" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H44" s="18">
+      <c r="R61" s="15">
+        <f t="shared" si="35"/>
+        <v>2.159864871588402E-2</v>
+      </c>
+      <c r="S61" s="15">
+        <f t="shared" si="35"/>
+        <v>5.1034239185863285E-2</v>
+      </c>
+      <c r="T61" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316965E-2</v>
+      </c>
+      <c r="U61" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316896E-2</v>
+      </c>
+      <c r="V61" s="15">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H62" s="14">
         <v>2030</v>
       </c>
-      <c r="I44" s="12">
-        <f t="shared" ref="I44:N48" si="15">I26-I35</f>
-        <v>2.8410520409202888</v>
-      </c>
-      <c r="J44" s="12">
-        <f t="shared" si="15"/>
-        <v>12.995103497810533</v>
-      </c>
-      <c r="K44" s="12">
-        <f t="shared" si="15"/>
-        <v>6.0896337018887721</v>
-      </c>
-      <c r="L44" s="12">
-        <f t="shared" si="15"/>
-        <v>17.150613901525901</v>
-      </c>
-      <c r="M44" s="12">
-        <f t="shared" si="15"/>
-        <v>3.1010122576464028</v>
-      </c>
-      <c r="N44" s="12">
-        <f t="shared" si="15"/>
-        <v>20.262460258721035</v>
-      </c>
-    </row>
-    <row r="45" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H45" s="18">
+      <c r="I62" s="15">
+        <f t="shared" ref="I62:N66" si="36">(1-(I53/I35))/I35</f>
+        <v>4.6286987191300703E-3</v>
+      </c>
+      <c r="J62" s="15">
+        <f t="shared" si="36"/>
+        <v>2.5110866614096584E-3</v>
+      </c>
+      <c r="K62" s="15">
+        <f t="shared" si="36"/>
+        <v>5.358586846835922E-3</v>
+      </c>
+      <c r="L62" s="15">
+        <f t="shared" si="36"/>
+        <v>4.3242888533228281E-3</v>
+      </c>
+      <c r="M62" s="15">
+        <f t="shared" si="36"/>
+        <v>7.6655988170767544E-3</v>
+      </c>
+      <c r="N62" s="15">
+        <f t="shared" si="36"/>
+        <v>3.082340536972066E-3</v>
+      </c>
+      <c r="P62" s="14">
+        <v>2030</v>
+      </c>
+      <c r="Q62" s="15">
+        <f t="shared" si="35"/>
+        <v>7.2005255799870646E-2</v>
+      </c>
+      <c r="R62" s="15">
+        <f t="shared" si="35"/>
+        <v>3.7935815937008122E-2</v>
+      </c>
+      <c r="S62" s="15">
+        <f t="shared" si="35"/>
+        <v>7.9415665577240849E-2</v>
+      </c>
+      <c r="T62" s="15">
+        <f t="shared" si="35"/>
+        <v>7.889539208931684E-2</v>
+      </c>
+      <c r="U62" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316979E-2</v>
+      </c>
+      <c r="V62" s="15">
+        <f t="shared" si="35"/>
+        <v>0.12666875354809062</v>
+      </c>
+    </row>
+    <row r="63" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H63" s="14">
         <v>2035</v>
       </c>
-      <c r="I45" s="12">
-        <f t="shared" si="15"/>
-        <v>2.5961337615306093</v>
-      </c>
-      <c r="J45" s="12">
-        <f t="shared" si="15"/>
-        <v>18.366303491438771</v>
-      </c>
-      <c r="K45" s="12">
-        <f t="shared" si="15"/>
-        <v>8.6066310083199653</v>
-      </c>
-      <c r="L45" s="12">
-        <f t="shared" si="15"/>
-        <v>15.617282230479987</v>
-      </c>
-      <c r="M45" s="12">
-        <f t="shared" si="15"/>
-        <v>3.8824908387163646</v>
-      </c>
-      <c r="N45" s="12">
-        <f t="shared" si="15"/>
-        <v>19.117618322753714</v>
-      </c>
-    </row>
-    <row r="46" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H46" s="18">
+      <c r="I63" s="15">
+        <f t="shared" si="36"/>
+        <v>5.0653684096140404E-3</v>
+      </c>
+      <c r="J63" s="15">
+        <f t="shared" si="36"/>
+        <v>2.8636876879813964E-3</v>
+      </c>
+      <c r="K63" s="15">
+        <f t="shared" si="36"/>
+        <v>6.1110273150225018E-3</v>
+      </c>
+      <c r="L63" s="15">
+        <f t="shared" si="36"/>
+        <v>5.5134028844093996E-3</v>
+      </c>
+      <c r="M63" s="15">
+        <f t="shared" si="36"/>
+        <v>8.4048700724761085E-3</v>
+      </c>
+      <c r="N63" s="15">
+        <f t="shared" si="36"/>
+        <v>4.0524179733364973E-3</v>
+      </c>
+      <c r="P63" s="14">
+        <v>2035</v>
+      </c>
+      <c r="Q63" s="15">
+        <f t="shared" si="35"/>
+        <v>0.10518985801607014</v>
+      </c>
+      <c r="R63" s="15">
+        <f t="shared" si="35"/>
+        <v>5.1034239185863375E-2</v>
+      </c>
+      <c r="S63" s="15">
+        <f t="shared" si="35"/>
+        <v>9.8967839167066807E-2</v>
+      </c>
+      <c r="T63" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316993E-2</v>
+      </c>
+      <c r="U63" s="15">
+        <f t="shared" si="35"/>
+        <v>7.889539208931691E-2</v>
+      </c>
+      <c r="V63" s="15">
+        <f t="shared" si="35"/>
+        <v>0.1651875193758317</v>
+      </c>
+    </row>
+    <row r="64" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H64" s="14">
         <v>2040</v>
       </c>
-      <c r="I46" s="12">
-        <f t="shared" si="15"/>
-        <v>2.372329126915929</v>
-      </c>
-      <c r="J46" s="12">
-        <f t="shared" si="15"/>
-        <v>15.655403272788135</v>
-      </c>
-      <c r="K46" s="12">
-        <f t="shared" si="15"/>
-        <v>10.106855861614008</v>
-      </c>
-      <c r="L46" s="12">
-        <f t="shared" si="15"/>
-        <v>13.175003247998475</v>
-      </c>
-      <c r="M46" s="12">
-        <f t="shared" si="15"/>
-        <v>4.3545037677906748</v>
-      </c>
-      <c r="N46" s="12">
-        <f t="shared" si="15"/>
-        <v>20.402801374616161</v>
-      </c>
-    </row>
-    <row r="47" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H47" s="18">
+      <c r="I64" s="15">
+        <f t="shared" si="36"/>
+        <v>5.5432333539172512E-3</v>
+      </c>
+      <c r="J64" s="15">
+        <f t="shared" si="36"/>
+        <v>3.3595657847781462E-3</v>
+      </c>
+      <c r="K64" s="15">
+        <f t="shared" si="36"/>
+        <v>6.984190506932688E-3</v>
+      </c>
+      <c r="L64" s="15">
+        <f t="shared" si="36"/>
+        <v>7.078467616032813E-3</v>
+      </c>
+      <c r="M64" s="15">
+        <f t="shared" si="36"/>
+        <v>9.2321065465968011E-3</v>
+      </c>
+      <c r="N64" s="15">
+        <f t="shared" si="36"/>
+        <v>4.3439983353645469E-3</v>
+      </c>
+      <c r="P64" s="14">
+        <v>2040</v>
+      </c>
+      <c r="Q64" s="15">
+        <f t="shared" si="35"/>
+        <v>0.10518985801607007</v>
+      </c>
+      <c r="R64" s="15">
+        <f t="shared" si="35"/>
+        <v>6.1942541927517823E-2</v>
+      </c>
+      <c r="S64" s="15">
+        <f t="shared" si="35"/>
+        <v>0.11381917348346579</v>
+      </c>
+      <c r="T64" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316882E-2</v>
+      </c>
+      <c r="U64" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316854E-2</v>
+      </c>
+      <c r="V64" s="15">
+        <f t="shared" si="35"/>
+        <v>0.16518751937583165</v>
+      </c>
+    </row>
+    <row r="65" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H65" s="14">
         <v>2045</v>
       </c>
-      <c r="I47" s="12">
-        <f t="shared" si="15"/>
-        <v>2.167817995285219</v>
-      </c>
-      <c r="J47" s="12">
-        <f t="shared" si="15"/>
-        <v>13.344636918793867</v>
-      </c>
-      <c r="K47" s="12">
-        <f t="shared" si="15"/>
-        <v>10.757656491573798</v>
-      </c>
-      <c r="L47" s="12">
-        <f t="shared" si="15"/>
-        <v>10.670287414926818</v>
-      </c>
-      <c r="M47" s="12">
-        <f t="shared" si="15"/>
-        <v>4.6073877125214722</v>
-      </c>
-      <c r="N47" s="12">
-        <f t="shared" si="15"/>
-        <v>20.73254657257246</v>
-      </c>
-    </row>
-    <row r="48" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H48" s="18">
+      <c r="I65" s="15">
+        <f t="shared" si="36"/>
+        <v>6.0661798967396345E-3</v>
+      </c>
+      <c r="J65" s="15">
+        <f t="shared" si="36"/>
+        <v>3.9413104681844512E-3</v>
+      </c>
+      <c r="K65" s="15">
+        <f t="shared" si="36"/>
+        <v>8.0040080256891903E-3</v>
+      </c>
+      <c r="L65" s="15">
+        <f t="shared" si="36"/>
+        <v>9.129292010114377E-3</v>
+      </c>
+      <c r="M65" s="15">
+        <f t="shared" si="36"/>
+        <v>1.0154459901310238E-2</v>
+      </c>
+      <c r="N65" s="15">
+        <f t="shared" si="36"/>
+        <v>4.6985144493336935E-3</v>
+      </c>
+      <c r="P65" s="14">
+        <v>2045</v>
+      </c>
+      <c r="Q65" s="15">
+        <f t="shared" si="35"/>
+        <v>0.10518985801607006</v>
+      </c>
+      <c r="R65" s="15">
+        <f t="shared" si="35"/>
+        <v>7.1273477648198635E-2</v>
+      </c>
+      <c r="S65" s="15">
+        <f t="shared" si="35"/>
+        <v>0.12575751774983088</v>
+      </c>
+      <c r="T65" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316924E-2</v>
+      </c>
+      <c r="U65" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316868E-2</v>
+      </c>
+      <c r="V65" s="15">
+        <f t="shared" si="35"/>
+        <v>0.16518751937583168</v>
+      </c>
+    </row>
+    <row r="66" spans="8:22" x14ac:dyDescent="0.25">
+      <c r="H66" s="14">
         <v>2050</v>
       </c>
-      <c r="I48" s="12">
-        <f t="shared" si="15"/>
-        <v>1.9809371336227173</v>
-      </c>
-      <c r="J48" s="12">
-        <f t="shared" si="15"/>
-        <v>11.374943934147581</v>
-      </c>
-      <c r="K48" s="12">
-        <f t="shared" si="15"/>
-        <v>10.801857403910347</v>
-      </c>
-      <c r="L48" s="12">
-        <f t="shared" si="15"/>
-        <v>8.4071872617356433</v>
-      </c>
-      <c r="M48" s="12">
-        <f t="shared" si="15"/>
-        <v>4.7041372522882341</v>
-      </c>
-      <c r="N48" s="12">
-        <f t="shared" si="15"/>
-        <v>21.093793516400609</v>
+      <c r="I66" s="15">
+        <f t="shared" si="36"/>
+        <v>6.6384610190735622E-3</v>
+      </c>
+      <c r="J66" s="15">
+        <f t="shared" si="36"/>
+        <v>4.62379045441021E-3</v>
+      </c>
+      <c r="K66" s="15">
+        <f t="shared" si="36"/>
+        <v>9.196254377799239E-3</v>
+      </c>
+      <c r="L66" s="15">
+        <f t="shared" si="36"/>
+        <v>1.1815679292787139E-2</v>
+      </c>
+      <c r="M66" s="15">
+        <f t="shared" si="36"/>
+        <v>1.1180659568676256E-2</v>
+      </c>
+      <c r="N66" s="15">
+        <f t="shared" si="36"/>
+        <v>4.9587095646873537E-3</v>
+      </c>
+      <c r="P66" s="14">
+        <v>2050</v>
+      </c>
+      <c r="Q66" s="15">
+        <f t="shared" si="35"/>
+        <v>0.10518985801607002</v>
+      </c>
+      <c r="R66" s="15">
+        <f t="shared" si="35"/>
+        <v>7.9415665577240932E-2</v>
+      </c>
+      <c r="S66" s="15">
+        <f t="shared" si="35"/>
+        <v>0.13571754371922554</v>
+      </c>
+      <c r="T66" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316882E-2</v>
+      </c>
+      <c r="U66" s="15">
+        <f t="shared" si="35"/>
+        <v>7.8895392089316993E-2</v>
+      </c>
+      <c r="V66" s="15">
+        <f t="shared" si="35"/>
+        <v>0.16518751937583168</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="14">
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P23:V23"/>
+    <mergeCell ref="P32:V32"/>
+    <mergeCell ref="P41:V41"/>
+    <mergeCell ref="P59:V59"/>
     <mergeCell ref="H41:N41"/>
-    <mergeCell ref="H5:N5"/>
-    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H50:N50"/>
     <mergeCell ref="H32:N32"/>
-    <mergeCell ref="H14:N14"/>
-    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="H59:N59"/>
+    <mergeCell ref="P50:V50"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="I43:N48">
+  <conditionalFormatting sqref="I52:N57">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I61:N66">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q52:V57">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q61:V66">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
compare cost of tax credit programs
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF37EA2-74DA-4772-877C-2EC8E4B3613B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8416BD9-4BAB-42FF-AAD8-E83D60A7E738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="Learning Rates" sheetId="5" r:id="rId2"/>
-    <sheet name="S2" sheetId="2" r:id="rId3"/>
+    <sheet name="Innovation Policy Scenarios" sheetId="2" r:id="rId3"/>
     <sheet name="verify-2025" sheetId="3" r:id="rId4"/>
     <sheet name="Procurement" sheetId="4" r:id="rId5"/>
   </sheets>
@@ -23,7 +23,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Learning Rates'!$Y$1:$AA$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="122">
   <si>
     <t>Tech</t>
   </si>
@@ -395,6 +394,21 @@
   </si>
   <si>
     <t>Cumulative Public R&amp;D (Million USD)</t>
+  </si>
+  <si>
+    <t>Baseline Parameters</t>
+  </si>
+  <si>
+    <t>BECCS (implemented)</t>
+  </si>
+  <si>
+    <t>Maintain Current Appropriations</t>
+  </si>
+  <si>
+    <t>Triple Appropriations</t>
+  </si>
+  <si>
+    <t>DAC Hubs</t>
   </si>
 </sst>
 </file>
@@ -488,7 +502,7 @@
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -507,10 +521,13 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1378,7 +1395,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$B$1</c:f>
+              <c:f>'Innovation Policy Scenarios'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1401,7 +1418,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$A$2:$A$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1428,7 +1445,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$B$2:$B$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$B$2:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1465,7 +1482,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$C$1</c:f>
+              <c:f>'Innovation Policy Scenarios'!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1488,7 +1505,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$A$2:$A$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1515,7 +1532,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$C$2:$C$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$C$2:$C$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1552,7 +1569,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$D$1</c:f>
+              <c:f>'Innovation Policy Scenarios'!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1575,7 +1592,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$A$2:$A$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1602,7 +1619,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$D$2:$D$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$D$2:$D$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1639,7 +1656,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$E$1</c:f>
+              <c:f>'Innovation Policy Scenarios'!$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1662,7 +1679,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$A$2:$A$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1689,7 +1706,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$E$2:$E$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$E$2:$E$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1726,7 +1743,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$F$1</c:f>
+              <c:f>'Innovation Policy Scenarios'!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1749,7 +1766,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$A$2:$A$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1776,7 +1793,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$F$2:$F$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$F$2:$F$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1813,7 +1830,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>'S2'!$G$1</c:f>
+              <c:f>'Innovation Policy Scenarios'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1838,7 +1855,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'S2'!$A$2:$A$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$A$2:$A$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1865,7 +1882,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'S2'!$G$2:$G$7</c:f>
+              <c:f>'Innovation Policy Scenarios'!$G$2:$G$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1919,7 +1936,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>'S2'!$A$1</c15:sqref>
+                          <c15:sqref>'Innovation Policy Scenarios'!$A$1</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -1948,7 +1965,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>'S2'!$A$2:$A$7</c15:sqref>
+                          <c15:sqref>'Innovation Policy Scenarios'!$A$2:$A$7</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -1981,7 +1998,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>'S2'!$A$2:$A$7</c15:sqref>
+                          <c15:sqref>'Innovation Policy Scenarios'!$A$2:$A$7</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -3463,16 +3480,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>195262</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>223837</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>14287</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>500062</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>61912</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>528637</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4748,24 +4765,24 @@
       <c r="E5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="P5" s="19" t="s">
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="P5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
       <c r="Y5">
         <v>2021</v>
       </c>
@@ -5290,24 +5307,24 @@
       <c r="E14" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="19"/>
-      <c r="P14" s="19" t="s">
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="P14" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="19"/>
-      <c r="R14" s="19"/>
-      <c r="S14" s="19"/>
-      <c r="T14" s="19"/>
-      <c r="U14" s="19"/>
-      <c r="V14" s="19"/>
+      <c r="Q14" s="18"/>
+      <c r="R14" s="18"/>
+      <c r="S14" s="18"/>
+      <c r="T14" s="18"/>
+      <c r="U14" s="18"/>
+      <c r="V14" s="18"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -5794,24 +5811,24 @@
         <f t="shared" si="14"/>
         <v>3512.6225095265308</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="P23" s="19" t="s">
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="18"/>
+      <c r="M23" s="18"/>
+      <c r="N23" s="18"/>
+      <c r="P23" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="19"/>
-      <c r="S23" s="19"/>
-      <c r="T23" s="19"/>
-      <c r="U23" s="19"/>
-      <c r="V23" s="19"/>
+      <c r="Q23" s="18"/>
+      <c r="R23" s="18"/>
+      <c r="S23" s="18"/>
+      <c r="T23" s="18"/>
+      <c r="U23" s="18"/>
+      <c r="V23" s="18"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="H24" s="13" t="s">
@@ -6210,24 +6227,24 @@
       <c r="V31" s="10"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H32" s="18" t="s">
+      <c r="H32" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="P32" s="18" t="s">
+      <c r="I32" s="19"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
+      <c r="P32" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="Q32" s="18"/>
-      <c r="R32" s="18"/>
-      <c r="S32" s="18"/>
-      <c r="T32" s="18"/>
-      <c r="U32" s="18"/>
-      <c r="V32" s="18"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="19"/>
+      <c r="S32" s="19"/>
+      <c r="T32" s="19"/>
+      <c r="U32" s="19"/>
+      <c r="V32" s="19"/>
     </row>
     <row r="33" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H33" s="14" t="s">
@@ -6626,24 +6643,24 @@
       <c r="V40" s="10"/>
     </row>
     <row r="41" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H41" s="18" t="s">
+      <c r="H41" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="I41" s="18"/>
-      <c r="J41" s="18"/>
-      <c r="K41" s="18"/>
-      <c r="L41" s="18"/>
-      <c r="M41" s="18"/>
-      <c r="N41" s="18"/>
-      <c r="P41" s="18" t="s">
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
+      <c r="N41" s="19"/>
+      <c r="P41" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="Q41" s="18"/>
-      <c r="R41" s="18"/>
-      <c r="S41" s="18"/>
-      <c r="T41" s="18"/>
-      <c r="U41" s="18"/>
-      <c r="V41" s="18"/>
+      <c r="Q41" s="19"/>
+      <c r="R41" s="19"/>
+      <c r="S41" s="19"/>
+      <c r="T41" s="19"/>
+      <c r="U41" s="19"/>
+      <c r="V41" s="19"/>
     </row>
     <row r="42" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H42" s="14" t="s">
@@ -7042,24 +7059,24 @@
       <c r="V49" s="10"/>
     </row>
     <row r="50" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H50" s="18" t="s">
+      <c r="H50" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="I50" s="18"/>
-      <c r="J50" s="18"/>
-      <c r="K50" s="18"/>
-      <c r="L50" s="18"/>
-      <c r="M50" s="18"/>
-      <c r="N50" s="18"/>
-      <c r="P50" s="18" t="s">
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
+      <c r="K50" s="19"/>
+      <c r="L50" s="19"/>
+      <c r="M50" s="19"/>
+      <c r="N50" s="19"/>
+      <c r="P50" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="Q50" s="18"/>
-      <c r="R50" s="18"/>
-      <c r="S50" s="18"/>
-      <c r="T50" s="18"/>
-      <c r="U50" s="18"/>
-      <c r="V50" s="18"/>
+      <c r="Q50" s="19"/>
+      <c r="R50" s="19"/>
+      <c r="S50" s="19"/>
+      <c r="T50" s="19"/>
+      <c r="U50" s="19"/>
+      <c r="V50" s="19"/>
     </row>
     <row r="51" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H51" s="14" t="s">
@@ -7445,24 +7462,24 @@
       <c r="P58" s="13"/>
     </row>
     <row r="59" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H59" s="18" t="s">
+      <c r="H59" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="I59" s="18"/>
-      <c r="J59" s="18"/>
-      <c r="K59" s="18"/>
-      <c r="L59" s="18"/>
-      <c r="M59" s="18"/>
-      <c r="N59" s="18"/>
-      <c r="P59" s="18" t="s">
+      <c r="I59" s="19"/>
+      <c r="J59" s="19"/>
+      <c r="K59" s="19"/>
+      <c r="L59" s="19"/>
+      <c r="M59" s="19"/>
+      <c r="N59" s="19"/>
+      <c r="P59" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="Q59" s="18"/>
-      <c r="R59" s="18"/>
-      <c r="S59" s="18"/>
-      <c r="T59" s="18"/>
-      <c r="U59" s="18"/>
-      <c r="V59" s="18"/>
+      <c r="Q59" s="19"/>
+      <c r="R59" s="19"/>
+      <c r="S59" s="19"/>
+      <c r="T59" s="19"/>
+      <c r="U59" s="19"/>
+      <c r="V59" s="19"/>
     </row>
     <row r="60" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H60" s="14" t="s">
@@ -7846,12 +7863,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H14:N14"/>
-    <mergeCell ref="H23:N23"/>
-    <mergeCell ref="H5:N5"/>
-    <mergeCell ref="P5:V5"/>
-    <mergeCell ref="P14:V14"/>
-    <mergeCell ref="P23:V23"/>
     <mergeCell ref="P32:V32"/>
     <mergeCell ref="P41:V41"/>
     <mergeCell ref="P59:V59"/>
@@ -7860,6 +7871,12 @@
     <mergeCell ref="H32:N32"/>
     <mergeCell ref="H59:N59"/>
     <mergeCell ref="P50:V50"/>
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P23:V23"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="I52:N57">
@@ -7911,10 +7928,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23D47325-8713-4C29-9B32-6AF71A8D6F7B}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7936,8 +7953,18 @@
       <c r="G1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L1" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -7965,8 +7992,32 @@
         <f t="shared" si="0"/>
         <v>231.99999999999997</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>3</v>
+      </c>
+      <c r="R2" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2030</v>
       </c>
@@ -7994,8 +8045,39 @@
         <f t="shared" si="1"/>
         <v>184.44635999999997</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <v>2025</v>
+      </c>
+      <c r="M3">
+        <f>'Baseline Parameters'!B2</f>
+        <v>446</v>
+      </c>
+      <c r="N3">
+        <f>'Baseline Parameters'!C2</f>
+        <v>209</v>
+      </c>
+      <c r="O3">
+        <f>'Baseline Parameters'!D2</f>
+        <v>316.03815554156989</v>
+      </c>
+      <c r="P3">
+        <f>'Baseline Parameters'!E2</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="Q3">
+        <f>'Baseline Parameters'!F2</f>
+        <v>140</v>
+      </c>
+      <c r="R3">
+        <f>'Baseline Parameters'!G2</f>
+        <v>232</v>
+      </c>
+      <c r="S3">
+        <f>'Baseline Parameters'!H2</f>
+        <v>0.13945355191256831</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2035</v>
       </c>
@@ -8023,8 +8105,39 @@
         <f t="shared" si="1"/>
         <v>144.65768827586206</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>2030</v>
+      </c>
+      <c r="M4">
+        <f>'Baseline Parameters'!B3</f>
+        <v>380.16957864810638</v>
+      </c>
+      <c r="N4">
+        <f>'Baseline Parameters'!C3</f>
+        <v>178.15121510639958</v>
+      </c>
+      <c r="O4">
+        <f>'Baseline Parameters'!D3</f>
+        <v>265</v>
+      </c>
+      <c r="P4">
+        <f>'Baseline Parameters'!E3</f>
+        <v>207.95454545454541</v>
+      </c>
+      <c r="Q4">
+        <f>'Baseline Parameters'!F3</f>
+        <v>126.10085958575935</v>
+      </c>
+      <c r="R4">
+        <f>'Baseline Parameters'!G3</f>
+        <v>212</v>
+      </c>
+      <c r="S4">
+        <f>'Baseline Parameters'!H3</f>
+        <v>0.12743169398907103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2040</v>
       </c>
@@ -8052,8 +8165,39 @@
         <f t="shared" si="1"/>
         <v>127.45712247324612</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>2035</v>
+      </c>
+      <c r="M5">
+        <f>'Baseline Parameters'!B4</f>
+        <v>324.05584872080431</v>
+      </c>
+      <c r="N5">
+        <f>'Baseline Parameters'!C4</f>
+        <v>151.85576767409884</v>
+      </c>
+      <c r="O5">
+        <f>'Baseline Parameters'!D4</f>
+        <v>222.20418252872307</v>
+      </c>
+      <c r="P5">
+        <f>'Baseline Parameters'!E4</f>
+        <v>160.17844876188263</v>
+      </c>
+      <c r="Q5">
+        <f>'Baseline Parameters'!F4</f>
+        <v>113.58161991619573</v>
+      </c>
+      <c r="R5">
+        <f>'Baseline Parameters'!G4</f>
+        <v>193.72413793103445</v>
+      </c>
+      <c r="S5">
+        <f>'Baseline Parameters'!H4</f>
+        <v>0.1164462031279442</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2045</v>
       </c>
@@ -8081,8 +8225,39 @@
         <f t="shared" si="1"/>
         <v>116.46943950141454</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>2040</v>
+      </c>
+      <c r="M6">
+        <f>'Baseline Parameters'!B5</f>
+        <v>276.22460866960239</v>
+      </c>
+      <c r="N6">
+        <f>'Baseline Parameters'!C5</f>
+        <v>129.4415767084011</v>
+      </c>
+      <c r="O6">
+        <f>'Baseline Parameters'!D5</f>
+        <v>186.3196178613513</v>
+      </c>
+      <c r="P6">
+        <f>'Baseline Parameters'!E5</f>
+        <v>123.37857483077323</v>
+      </c>
+      <c r="Q6">
+        <f>'Baseline Parameters'!F5</f>
+        <v>102.30528503268064</v>
+      </c>
+      <c r="R6">
+        <f>'Baseline Parameters'!G5</f>
+        <v>177.02378121284181</v>
+      </c>
+      <c r="S6">
+        <f>'Baseline Parameters'!H5</f>
+        <v>0.10640773734105245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2050</v>
       </c>
@@ -8110,8 +8285,72 @@
         <f t="shared" si="1"/>
         <v>106.42897057887879</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>2045</v>
+      </c>
+      <c r="M7">
+        <f>'Baseline Parameters'!B6</f>
+        <v>235.45334773578654</v>
+      </c>
+      <c r="N7">
+        <f>'Baseline Parameters'!C6</f>
+        <v>110.33576160712865</v>
+      </c>
+      <c r="O7">
+        <f>'Baseline Parameters'!D6</f>
+        <v>156.23018255073828</v>
+      </c>
+      <c r="P7">
+        <f>'Baseline Parameters'!E6</f>
+        <v>95.033213549856328</v>
+      </c>
+      <c r="Q7">
+        <f>'Baseline Parameters'!F6</f>
+        <v>92.14845987705111</v>
+      </c>
+      <c r="R7">
+        <f>'Baseline Parameters'!G6</f>
+        <v>161.7631104186313</v>
+      </c>
+      <c r="S7">
+        <f>'Baseline Parameters'!H6</f>
+        <v>9.7234656535789318E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>2050</v>
+      </c>
+      <c r="M8">
+        <f>'Baseline Parameters'!B7</f>
+        <v>200.70000000000002</v>
+      </c>
+      <c r="N8">
+        <f>'Baseline Parameters'!C7</f>
+        <v>94.05</v>
+      </c>
+      <c r="O8">
+        <f>'Baseline Parameters'!D7</f>
+        <v>131</v>
+      </c>
+      <c r="P8">
+        <f>'Baseline Parameters'!E7</f>
+        <v>73.199999999999989</v>
+      </c>
+      <c r="Q8">
+        <f>'Baseline Parameters'!F7</f>
+        <v>83</v>
+      </c>
+      <c r="R8">
+        <f>'Baseline Parameters'!G7</f>
+        <v>147.8180146928872</v>
+      </c>
+      <c r="S8">
+        <f>'Baseline Parameters'!H7</f>
+        <v>8.8852358558566089E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -8139,8 +8378,18 @@
         <f>'Baseline Parameters'!G13</f>
         <v>231.99999999999997</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L10" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="M10" s="20"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="20"/>
+      <c r="S10" s="20"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -8168,8 +8417,65 @@
         <f>'Baseline Parameters'!G14</f>
         <v>-1.8030219398859515E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L11" t="s">
+        <v>0</v>
+      </c>
+      <c r="M11" t="s">
+        <v>9</v>
+      </c>
+      <c r="N11" t="s">
+        <v>8</v>
+      </c>
+      <c r="O11" t="s">
+        <v>38</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>3</v>
+      </c>
+      <c r="R11" t="s">
+        <v>28</v>
+      </c>
+      <c r="S11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <v>2025</v>
+      </c>
+      <c r="M12">
+        <f>M3*(1-'Learning Rates'!$Q61)</f>
+        <v>446</v>
+      </c>
+      <c r="N12">
+        <f>N3*(1-'Learning Rates'!$Q61)</f>
+        <v>209</v>
+      </c>
+      <c r="O12">
+        <f>O3*(1-'Learning Rates'!$Q61)</f>
+        <v>316.03815554156989</v>
+      </c>
+      <c r="P12">
+        <f>P3*(1-'Learning Rates'!$Q61)</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="Q12">
+        <f>Q3*(1-'Learning Rates'!$Q61)</f>
+        <v>140</v>
+      </c>
+      <c r="R12">
+        <f>R3*(1-'Learning Rates'!$Q61)</f>
+        <v>232</v>
+      </c>
+      <c r="S12">
+        <f>S3*(1-'Learning Rates'!$Q61)</f>
+        <v>0.13945355191256831</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -8194,8 +8500,39 @@
       <c r="H13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>2030</v>
+      </c>
+      <c r="M13">
+        <f>M4*(1-'Learning Rates'!$Q62)</f>
+        <v>352.79537089022045</v>
+      </c>
+      <c r="N13">
+        <f>N4*(1-'Learning Rates'!$Q62)</f>
+        <v>165.3233912916055</v>
+      </c>
+      <c r="O13">
+        <f>O4*(1-'Learning Rates'!$Q62)</f>
+        <v>245.91860721303428</v>
+      </c>
+      <c r="P13">
+        <f>P4*(1-'Learning Rates'!$Q62)</f>
+        <v>192.98072521434506</v>
+      </c>
+      <c r="Q13">
+        <f>Q4*(1-'Learning Rates'!$Q62)</f>
+        <v>117.02093493470319</v>
+      </c>
+      <c r="R13">
+        <f>R4*(1-'Learning Rates'!$Q62)</f>
+        <v>196.73488577042744</v>
+      </c>
+      <c r="S13">
+        <f>S4*(1-'Learning Rates'!$Q62)</f>
+        <v>0.11825594226637715</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -8220,8 +8557,39 @@
       <c r="H14" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <v>2035</v>
+      </c>
+      <c r="M14">
+        <f>M5*(1-'Learning Rates'!$Q63)</f>
+        <v>289.96846000458578</v>
+      </c>
+      <c r="N14">
+        <f>N5*(1-'Learning Rates'!$Q63)</f>
+        <v>135.88208103353904</v>
+      </c>
+      <c r="O14">
+        <f>O5*(1-'Learning Rates'!$Q63)</f>
+        <v>198.83055611794975</v>
+      </c>
+      <c r="P14">
+        <f>P5*(1-'Learning Rates'!$Q63)</f>
+        <v>143.32930047938584</v>
+      </c>
+      <c r="Q14">
+        <f>Q5*(1-'Learning Rates'!$Q63)</f>
+        <v>101.63398544397586</v>
+      </c>
+      <c r="R14">
+        <f>R5*(1-'Learning Rates'!$Q63)</f>
+        <v>173.34632336778333</v>
+      </c>
+      <c r="S14">
+        <f>S5*(1-'Learning Rates'!$Q63)</f>
+        <v>0.10419724355440528</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2030</v>
       </c>
@@ -8246,8 +8614,39 @@
       <c r="H15" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <v>2040</v>
+      </c>
+      <c r="M15">
+        <f>M6*(1-'Learning Rates'!$Q64)</f>
+        <v>247.1685813031024</v>
+      </c>
+      <c r="N15">
+        <f>N6*(1-'Learning Rates'!$Q64)</f>
+        <v>115.82563563306815</v>
+      </c>
+      <c r="O15">
+        <f>O6*(1-'Learning Rates'!$Q64)</f>
+        <v>166.72068371290732</v>
+      </c>
+      <c r="P15">
+        <f>P6*(1-'Learning Rates'!$Q64)</f>
+        <v>110.40040006209912</v>
+      </c>
+      <c r="Q15">
+        <f>Q6*(1-'Learning Rates'!$Q64)</f>
+        <v>91.543806625799391</v>
+      </c>
+      <c r="R15">
+        <f>R6*(1-'Learning Rates'!$Q64)</f>
+        <v>158.40267480159514</v>
+      </c>
+      <c r="S15">
+        <f>S6*(1-'Learning Rates'!$Q64)</f>
+        <v>9.5214722558335865E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2035</v>
       </c>
@@ -8272,8 +8671,39 @@
       <c r="H16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>2045</v>
+      </c>
+      <c r="M16">
+        <f>M7*(1-'Learning Rates'!$Q65)</f>
+        <v>210.68604351805078</v>
+      </c>
+      <c r="N16">
+        <f>N7*(1-'Learning Rates'!$Q65)</f>
+        <v>98.729558509579832</v>
+      </c>
+      <c r="O16">
+        <f>O7*(1-'Learning Rates'!$Q65)</f>
+        <v>139.79635183040142</v>
+      </c>
+      <c r="P16">
+        <f>P7*(1-'Learning Rates'!$Q65)</f>
+        <v>85.036683309736077</v>
+      </c>
+      <c r="Q16">
+        <f>Q7*(1-'Learning Rates'!$Q65)</f>
+        <v>82.455376466184575</v>
+      </c>
+      <c r="R16">
+        <f>R7*(1-'Learning Rates'!$Q65)</f>
+        <v>144.7472718014576</v>
+      </c>
+      <c r="S16">
+        <f>S7*(1-'Learning Rates'!$Q65)</f>
+        <v>8.7006556820548295E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2040</v>
       </c>
@@ -8298,8 +8728,39 @@
       <c r="H17" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>2050</v>
+      </c>
+      <c r="M17">
+        <f>M8*(1-'Learning Rates'!$Q66)</f>
+        <v>179.58839549617474</v>
+      </c>
+      <c r="N17">
+        <f>N8*(1-'Learning Rates'!$Q66)</f>
+        <v>84.156893853588613</v>
+      </c>
+      <c r="O17">
+        <f>O8*(1-'Learning Rates'!$Q66)</f>
+        <v>117.22012859989482</v>
+      </c>
+      <c r="P17">
+        <f>P8*(1-'Learning Rates'!$Q66)</f>
+        <v>65.500102393223656</v>
+      </c>
+      <c r="Q17">
+        <f>Q8*(1-'Learning Rates'!$Q66)</f>
+        <v>74.269241784666178</v>
+      </c>
+      <c r="R17">
+        <f>R8*(1-'Learning Rates'!$Q66)</f>
+        <v>132.26905871512503</v>
+      </c>
+      <c r="S17">
+        <f>S8*(1-'Learning Rates'!$Q66)</f>
+        <v>7.9505991577397572E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2045</v>
       </c>
@@ -8325,7 +8786,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2050</v>
       </c>
@@ -8350,8 +8811,44 @@
       <c r="H19" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L19" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="M19" s="20"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="20"/>
+      <c r="P19" s="20"/>
+      <c r="Q19" s="20"/>
+      <c r="R19" s="20"/>
+      <c r="S19" s="20"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L20" t="s">
+        <v>0</v>
+      </c>
+      <c r="M20" t="s">
+        <v>9</v>
+      </c>
+      <c r="N20" t="s">
+        <v>8</v>
+      </c>
+      <c r="O20" t="s">
+        <v>38</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>3</v>
+      </c>
+      <c r="R20" t="s">
+        <v>28</v>
+      </c>
+      <c r="S20" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -8376,8 +8873,39 @@
       <c r="H21" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L21">
+        <v>2025</v>
+      </c>
+      <c r="M21">
+        <f>M3*(1-'Learning Rates'!$R61)</f>
+        <v>436.36700267271573</v>
+      </c>
+      <c r="N21">
+        <f>N3*(1-'Learning Rates'!$R61)</f>
+        <v>204.48588241838024</v>
+      </c>
+      <c r="O21">
+        <f>O3*(1-'Learning Rates'!$R61)</f>
+        <v>309.21215843921163</v>
+      </c>
+      <c r="P21">
+        <f>P3*(1-'Learning Rates'!$R61)</f>
+        <v>264.14950157400961</v>
+      </c>
+      <c r="Q21">
+        <f>Q3*(1-'Learning Rates'!$R61)</f>
+        <v>136.97618917977624</v>
+      </c>
+      <c r="R21">
+        <f>R3*(1-'Learning Rates'!$R61)</f>
+        <v>226.9891134979149</v>
+      </c>
+      <c r="S21">
+        <f>S3*(1-'Learning Rates'!$R61)</f>
+        <v>0.13644154363262645</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -8402,8 +8930,39 @@
       <c r="H22" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L22">
+        <v>2030</v>
+      </c>
+      <c r="M22">
+        <f>M4*(1-'Learning Rates'!$R62)</f>
+        <v>365.74753548766188</v>
+      </c>
+      <c r="N22">
+        <f>N4*(1-'Learning Rates'!$R62)</f>
+        <v>171.39290340116887</v>
+      </c>
+      <c r="O22">
+        <f>O4*(1-'Learning Rates'!$R62)</f>
+        <v>254.94700877669285</v>
+      </c>
+      <c r="P22">
+        <f>P4*(1-'Learning Rates'!$R62)</f>
+        <v>200.06562009491759</v>
+      </c>
+      <c r="Q22">
+        <f>Q4*(1-'Learning Rates'!$R62)</f>
+        <v>121.31712058701548</v>
+      </c>
+      <c r="R22">
+        <f>R4*(1-'Learning Rates'!$R62)</f>
+        <v>203.95760702135428</v>
+      </c>
+      <c r="S22">
+        <f>S4*(1-'Learning Rates'!$R62)</f>
+        <v>0.12259746870136048</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2030</v>
       </c>
@@ -8428,8 +8987,39 @@
       <c r="H23" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L23">
+        <v>2035</v>
+      </c>
+      <c r="M23">
+        <f>M5*(1-'Learning Rates'!$R63)</f>
+        <v>307.51790502760883</v>
+      </c>
+      <c r="N23">
+        <f>N5*(1-'Learning Rates'!$R63)</f>
+        <v>144.10592410486598</v>
+      </c>
+      <c r="O23">
+        <f>O5*(1-'Learning Rates'!$R63)</f>
+        <v>210.86416112945298</v>
+      </c>
+      <c r="P23">
+        <f>P5*(1-'Learning Rates'!$R63)</f>
+        <v>152.00386349534816</v>
+      </c>
+      <c r="Q23">
+        <f>Q5*(1-'Learning Rates'!$R63)</f>
+        <v>107.78506835827478</v>
+      </c>
+      <c r="R23">
+        <f>R5*(1-'Learning Rates'!$R63)</f>
+        <v>183.83757393978686</v>
+      </c>
+      <c r="S23">
+        <f>S5*(1-'Learning Rates'!$R63)</f>
+        <v>0.11050345974522706</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2035</v>
       </c>
@@ -8454,8 +9044,39 @@
       <c r="H24" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L24">
+        <v>2040</v>
+      </c>
+      <c r="M24">
+        <f>M6*(1-'Learning Rates'!$R64)</f>
+        <v>259.11455426567335</v>
+      </c>
+      <c r="N24">
+        <f>N6*(1-'Learning Rates'!$R64)</f>
+        <v>121.42363641597696</v>
+      </c>
+      <c r="O24">
+        <f>O6*(1-'Learning Rates'!$R64)</f>
+        <v>174.77850712005545</v>
+      </c>
+      <c r="P24">
+        <f>P6*(1-'Learning Rates'!$R64)</f>
+        <v>115.73619228636066</v>
+      </c>
+      <c r="Q24">
+        <f>Q6*(1-'Learning Rates'!$R64)</f>
+        <v>95.968235625137169</v>
+      </c>
+      <c r="R24">
+        <f>R6*(1-'Learning Rates'!$R64)</f>
+        <v>166.05847822289761</v>
+      </c>
+      <c r="S24">
+        <f>S6*(1-'Learning Rates'!$R64)</f>
+        <v>9.9816571609392016E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2040</v>
       </c>
@@ -8480,8 +9101,39 @@
       <c r="H25" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L25">
+        <v>2045</v>
+      </c>
+      <c r="M25">
+        <f>M7*(1-'Learning Rates'!$R65)</f>
+        <v>218.67176881874641</v>
+      </c>
+      <c r="N25">
+        <f>N7*(1-'Learning Rates'!$R65)</f>
+        <v>102.47174816842599</v>
+      </c>
+      <c r="O25">
+        <f>O7*(1-'Learning Rates'!$R65)</f>
+        <v>145.09511412673425</v>
+      </c>
+      <c r="P25">
+        <f>P7*(1-'Learning Rates'!$R65)</f>
+        <v>88.259865928074149</v>
+      </c>
+      <c r="Q25">
+        <f>Q7*(1-'Learning Rates'!$R65)</f>
+        <v>85.580718681688168</v>
+      </c>
+      <c r="R25">
+        <f>R7*(1-'Learning Rates'!$R65)</f>
+        <v>150.23369098390589</v>
+      </c>
+      <c r="S25">
+        <f>S7*(1-'Learning Rates'!$R65)</f>
+        <v>9.0304404416555462E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2045</v>
       </c>
@@ -8506,8 +9158,39 @@
       <c r="H26" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L26">
+        <v>2050</v>
+      </c>
+      <c r="M26">
+        <f>M8*(1-'Learning Rates'!$R66)</f>
+        <v>184.76127591864778</v>
+      </c>
+      <c r="N26">
+        <f>N8*(1-'Learning Rates'!$R66)</f>
+        <v>86.580956652460486</v>
+      </c>
+      <c r="O26">
+        <f>O8*(1-'Learning Rates'!$R66)</f>
+        <v>120.59654780938145</v>
+      </c>
+      <c r="P26">
+        <f>P8*(1-'Learning Rates'!$R66)</f>
+        <v>67.386773279745952</v>
+      </c>
+      <c r="Q26">
+        <f>Q8*(1-'Learning Rates'!$R66)</f>
+        <v>76.408499757089004</v>
+      </c>
+      <c r="R26">
+        <f>R8*(1-'Learning Rates'!$R66)</f>
+        <v>136.0789486717452</v>
+      </c>
+      <c r="S26">
+        <f>S8*(1-'Learning Rates'!$R66)</f>
+        <v>8.17960893655299E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2050</v>
       </c>
@@ -8533,7 +9216,19 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L28" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="M28" s="20"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="20"/>
+      <c r="P28" s="20"/>
+      <c r="Q28" s="20"/>
+      <c r="R28" s="20"/>
+      <c r="S28" s="20"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -8558,8 +9253,32 @@
       <c r="H29" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L29" t="s">
+        <v>0</v>
+      </c>
+      <c r="M29" t="s">
+        <v>9</v>
+      </c>
+      <c r="N29" t="s">
+        <v>8</v>
+      </c>
+      <c r="O29" t="s">
+        <v>38</v>
+      </c>
+      <c r="P29" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>3</v>
+      </c>
+      <c r="R29" t="s">
+        <v>28</v>
+      </c>
+      <c r="S29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2025</v>
       </c>
@@ -8584,8 +9303,39 @@
       <c r="H30" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L30">
+        <v>2025</v>
+      </c>
+      <c r="M30">
+        <f>M3*(1-'Learning Rates'!$S61)</f>
+        <v>423.23872932310496</v>
+      </c>
+      <c r="N30">
+        <f>N3*(1-'Learning Rates'!$S61)</f>
+        <v>198.33384401015459</v>
+      </c>
+      <c r="O30">
+        <f>O3*(1-'Learning Rates'!$S61)</f>
+        <v>299.90938871980234</v>
+      </c>
+      <c r="P30">
+        <f>P3*(1-'Learning Rates'!$S61)</f>
+        <v>256.20245965611286</v>
+      </c>
+      <c r="Q30">
+        <f>Q3*(1-'Learning Rates'!$S61)</f>
+        <v>132.85520651397914</v>
+      </c>
+      <c r="R30">
+        <f>R3*(1-'Learning Rates'!$S61)</f>
+        <v>220.16005650887973</v>
+      </c>
+      <c r="S30">
+        <f>S3*(1-'Learning Rates'!$S61)</f>
+        <v>0.1323366459889441</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2030</v>
       </c>
@@ -8610,8 +9360,39 @@
       <c r="H31" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L31">
+        <v>2030</v>
+      </c>
+      <c r="M31">
+        <f>M4*(1-'Learning Rates'!$S62)</f>
+        <v>349.97815852754781</v>
+      </c>
+      <c r="N31">
+        <f>N4*(1-'Learning Rates'!$S62)</f>
+        <v>164.00321778533063</v>
+      </c>
+      <c r="O31">
+        <f>O4*(1-'Learning Rates'!$S62)</f>
+        <v>243.95484862203116</v>
+      </c>
+      <c r="P31">
+        <f>P4*(1-'Learning Rates'!$S62)</f>
+        <v>191.43969681746009</v>
+      </c>
+      <c r="Q31">
+        <f>Q4*(1-'Learning Rates'!$S62)</f>
+        <v>116.08647589189408</v>
+      </c>
+      <c r="R31">
+        <f>R4*(1-'Learning Rates'!$S62)</f>
+        <v>195.16387889762493</v>
+      </c>
+      <c r="S31">
+        <f>S4*(1-'Learning Rates'!$S62)</f>
+        <v>0.11731162119529367</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2035</v>
       </c>
@@ -8636,8 +9417,39 @@
       <c r="H32" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L32">
+        <v>2035</v>
+      </c>
+      <c r="M32">
+        <f>M5*(1-'Learning Rates'!$S63)</f>
+        <v>291.98474160345643</v>
+      </c>
+      <c r="N32">
+        <f>N5*(1-'Learning Rates'!$S63)</f>
+        <v>136.82693048233716</v>
+      </c>
+      <c r="O32">
+        <f>O5*(1-'Learning Rates'!$S63)</f>
+        <v>200.21311472997087</v>
+      </c>
+      <c r="P32">
+        <f>P5*(1-'Learning Rates'!$S63)</f>
+        <v>144.3259338067864</v>
+      </c>
+      <c r="Q32">
+        <f>Q5*(1-'Learning Rates'!$S63)</f>
+        <v>102.34069242399477</v>
+      </c>
+      <c r="R32">
+        <f>R5*(1-'Learning Rates'!$S63)</f>
+        <v>174.55167860549719</v>
+      </c>
+      <c r="S32">
+        <f>S5*(1-'Learning Rates'!$S63)</f>
+        <v>0.10492177402516223</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2040</v>
       </c>
@@ -8662,8 +9474,39 @@
       <c r="H33" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L33">
+        <v>2040</v>
+      </c>
+      <c r="M33">
+        <f>M6*(1-'Learning Rates'!$S64)</f>
+        <v>244.78495201503446</v>
+      </c>
+      <c r="N33">
+        <f>N6*(1-'Learning Rates'!$S64)</f>
+        <v>114.70864343305425</v>
+      </c>
+      <c r="O33">
+        <f>O6*(1-'Learning Rates'!$S64)</f>
+        <v>165.1128729526171</v>
+      </c>
+      <c r="P33">
+        <f>P6*(1-'Learning Rates'!$S64)</f>
+        <v>109.33572741796668</v>
+      </c>
+      <c r="Q33">
+        <f>Q6*(1-'Learning Rates'!$S64)</f>
+        <v>90.660982047270551</v>
+      </c>
+      <c r="R33">
+        <f>R6*(1-'Learning Rates'!$S64)</f>
+        <v>156.87508074827826</v>
+      </c>
+      <c r="S33">
+        <f>S6*(1-'Learning Rates'!$S64)</f>
+        <v>9.4296496624648146E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2045</v>
       </c>
@@ -8688,8 +9531,39 @@
       <c r="H34" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="L34">
+        <v>2045</v>
+      </c>
+      <c r="M34">
+        <f>M7*(1-'Learning Rates'!$S65)</f>
+        <v>205.84331917864625</v>
+      </c>
+      <c r="N34">
+        <f>N7*(1-'Learning Rates'!$S65)</f>
+        <v>96.460210108379059</v>
+      </c>
+      <c r="O34">
+        <f>O7*(1-'Learning Rates'!$S65)</f>
+        <v>136.58306259555448</v>
+      </c>
+      <c r="P34">
+        <f>P7*(1-'Learning Rates'!$S65)</f>
+        <v>83.082072510036795</v>
+      </c>
+      <c r="Q34">
+        <f>Q7*(1-'Learning Rates'!$S65)</f>
+        <v>80.560098298443279</v>
+      </c>
+      <c r="R34">
+        <f>R7*(1-'Learning Rates'!$S65)</f>
+        <v>141.42018318889242</v>
+      </c>
+      <c r="S34">
+        <f>S7*(1-'Learning Rates'!$S65)</f>
+        <v>8.5006667490591076E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2050</v>
       </c>
@@ -8714,8 +9588,519 @@
       <c r="H35" t="s">
         <v>35</v>
       </c>
+      <c r="L35">
+        <v>2050</v>
+      </c>
+      <c r="M35">
+        <f>M8*(1-'Learning Rates'!$S66)</f>
+        <v>173.46148897555145</v>
+      </c>
+      <c r="N35">
+        <f>N8*(1-'Learning Rates'!$S66)</f>
+        <v>81.285765013206841</v>
+      </c>
+      <c r="O35">
+        <f>O8*(1-'Learning Rates'!$S66)</f>
+        <v>113.22100177278146</v>
+      </c>
+      <c r="P35">
+        <f>P8*(1-'Learning Rates'!$S66)</f>
+        <v>63.265475799752686</v>
+      </c>
+      <c r="Q35">
+        <f>Q8*(1-'Learning Rates'!$S66)</f>
+        <v>71.735443871304284</v>
+      </c>
+      <c r="R35">
+        <f>R8*(1-'Learning Rates'!$S66)</f>
+        <v>127.75651682131617</v>
+      </c>
+      <c r="S35">
+        <f>S8*(1-'Learning Rates'!$S66)</f>
+        <v>7.6793534701337596E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L37" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="M37" s="20"/>
+      <c r="N37" s="20"/>
+      <c r="O37" s="20"/>
+      <c r="P37" s="20"/>
+      <c r="Q37" s="20"/>
+      <c r="R37" s="20"/>
+      <c r="S37" s="20"/>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L38" t="s">
+        <v>0</v>
+      </c>
+      <c r="M38" t="s">
+        <v>9</v>
+      </c>
+      <c r="N38" t="s">
+        <v>8</v>
+      </c>
+      <c r="O38" t="s">
+        <v>38</v>
+      </c>
+      <c r="P38" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>3</v>
+      </c>
+      <c r="R38" t="s">
+        <v>28</v>
+      </c>
+      <c r="S38" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L39">
+        <v>2025</v>
+      </c>
+      <c r="M39">
+        <f>M12*(1-'Learning Rates'!T61)</f>
+        <v>410.81265512816464</v>
+      </c>
+      <c r="N39">
+        <f>N12*(1-'Learning Rates'!U61)</f>
+        <v>192.51086305333277</v>
+      </c>
+      <c r="O39">
+        <f>O12</f>
+        <v>316.03815554156989</v>
+      </c>
+      <c r="P39">
+        <f t="shared" ref="P39:S39" si="3">P12</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="Q39">
+        <f t="shared" si="3"/>
+        <v>140</v>
+      </c>
+      <c r="R39">
+        <f t="shared" si="3"/>
+        <v>232</v>
+      </c>
+      <c r="S39">
+        <f t="shared" si="3"/>
+        <v>0.13945355191256831</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L40">
+        <v>2030</v>
+      </c>
+      <c r="M40">
+        <f>M13*(1-'Learning Rates'!T62)</f>
+        <v>324.96144177654054</v>
+      </c>
+      <c r="N40">
+        <f>N13*(1-'Learning Rates'!U62)</f>
+        <v>152.28013751411871</v>
+      </c>
+      <c r="O40">
+        <f t="shared" ref="O40:S44" si="4">O13</f>
+        <v>245.91860721303428</v>
+      </c>
+      <c r="P40">
+        <f t="shared" si="4"/>
+        <v>192.98072521434506</v>
+      </c>
+      <c r="Q40">
+        <f t="shared" si="4"/>
+        <v>117.02093493470319</v>
+      </c>
+      <c r="R40">
+        <f t="shared" si="4"/>
+        <v>196.73488577042744</v>
+      </c>
+      <c r="S40">
+        <f t="shared" si="4"/>
+        <v>0.11825594226637715</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L41">
+        <v>2035</v>
+      </c>
+      <c r="M41">
+        <f>M14*(1-'Learning Rates'!T63)</f>
+        <v>267.09128465898857</v>
+      </c>
+      <c r="N41">
+        <f>N14*(1-'Learning Rates'!U63)</f>
+        <v>125.16161097248563</v>
+      </c>
+      <c r="O41">
+        <f t="shared" si="4"/>
+        <v>198.83055611794975</v>
+      </c>
+      <c r="P41">
+        <f t="shared" si="4"/>
+        <v>143.32930047938584</v>
+      </c>
+      <c r="Q41">
+        <f t="shared" si="4"/>
+        <v>101.63398544397586</v>
+      </c>
+      <c r="R41">
+        <f t="shared" si="4"/>
+        <v>173.34632336778333</v>
+      </c>
+      <c r="S41">
+        <f t="shared" si="4"/>
+        <v>0.10419724355440528</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L42">
+        <v>2040</v>
+      </c>
+      <c r="M42">
+        <f>M15*(1-'Learning Rates'!T64)</f>
+        <v>227.66811916903396</v>
+      </c>
+      <c r="N42">
+        <f>N15*(1-'Learning Rates'!U64)</f>
+        <v>106.68752669580289</v>
+      </c>
+      <c r="O42">
+        <f t="shared" si="4"/>
+        <v>166.72068371290732</v>
+      </c>
+      <c r="P42">
+        <f t="shared" si="4"/>
+        <v>110.40040006209912</v>
+      </c>
+      <c r="Q42">
+        <f t="shared" si="4"/>
+        <v>91.543806625799391</v>
+      </c>
+      <c r="R42">
+        <f t="shared" si="4"/>
+        <v>158.40267480159514</v>
+      </c>
+      <c r="S42">
+        <f t="shared" si="4"/>
+        <v>9.5214722558335865E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L43">
+        <v>2045</v>
+      </c>
+      <c r="M43">
+        <f>M16*(1-'Learning Rates'!T65)</f>
+        <v>194.06388550694726</v>
+      </c>
+      <c r="N43">
+        <f>N16*(1-'Learning Rates'!U65)</f>
+        <v>90.940251280161377</v>
+      </c>
+      <c r="O43">
+        <f t="shared" si="4"/>
+        <v>139.79635183040142</v>
+      </c>
+      <c r="P43">
+        <f t="shared" si="4"/>
+        <v>85.036683309736077</v>
+      </c>
+      <c r="Q43">
+        <f t="shared" si="4"/>
+        <v>82.455376466184575</v>
+      </c>
+      <c r="R43">
+        <f t="shared" si="4"/>
+        <v>144.7472718014576</v>
+      </c>
+      <c r="S43">
+        <f t="shared" si="4"/>
+        <v>8.7006556820548295E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L44">
+        <v>2050</v>
+      </c>
+      <c r="M44">
+        <f>M17*(1-'Learning Rates'!T66)</f>
+        <v>165.41969861881273</v>
+      </c>
+      <c r="N44">
+        <f>N17*(1-'Learning Rates'!U66)</f>
+        <v>77.517302715990709</v>
+      </c>
+      <c r="O44">
+        <f t="shared" si="4"/>
+        <v>117.22012859989482</v>
+      </c>
+      <c r="P44">
+        <f t="shared" si="4"/>
+        <v>65.500102393223656</v>
+      </c>
+      <c r="Q44">
+        <f t="shared" si="4"/>
+        <v>74.269241784666178</v>
+      </c>
+      <c r="R44">
+        <f t="shared" si="4"/>
+        <v>132.26905871512503</v>
+      </c>
+      <c r="S44">
+        <f t="shared" si="4"/>
+        <v>7.9505991577397572E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L46" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="M46" s="20"/>
+      <c r="N46" s="20"/>
+      <c r="O46" s="20"/>
+      <c r="P46" s="20"/>
+      <c r="Q46" s="20"/>
+      <c r="R46" s="20"/>
+      <c r="S46" s="20"/>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L47" t="s">
+        <v>0</v>
+      </c>
+      <c r="M47" t="s">
+        <v>9</v>
+      </c>
+      <c r="N47" t="s">
+        <v>8</v>
+      </c>
+      <c r="O47" t="s">
+        <v>38</v>
+      </c>
+      <c r="P47" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>3</v>
+      </c>
+      <c r="R47" t="s">
+        <v>28</v>
+      </c>
+      <c r="S47" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="L48">
+        <v>2025</v>
+      </c>
+      <c r="M48">
+        <f>M12*(1-'Learning Rates'!$V61)</f>
+        <v>446</v>
+      </c>
+      <c r="N48">
+        <f>N12*(1-'Learning Rates'!$V61)</f>
+        <v>209</v>
+      </c>
+      <c r="O48">
+        <f>O12*(1-'Learning Rates'!$V61)</f>
+        <v>316.03815554156989</v>
+      </c>
+      <c r="P48">
+        <f>P12*(1-'Learning Rates'!$V61)</f>
+        <v>269.98072031209182</v>
+      </c>
+      <c r="Q48">
+        <f>Q12*(1-'Learning Rates'!$V61)</f>
+        <v>140</v>
+      </c>
+      <c r="R48">
+        <f>R12*(1-'Learning Rates'!$V61)</f>
+        <v>232</v>
+      </c>
+      <c r="S48">
+        <f>S12*(1-'Learning Rates'!$V61)</f>
+        <v>0.13945355191256831</v>
+      </c>
+    </row>
+    <row r="49" spans="12:19" x14ac:dyDescent="0.25">
+      <c r="L49">
+        <v>2030</v>
+      </c>
+      <c r="M49">
+        <f>M13*(1-'Learning Rates'!$V62)</f>
+        <v>308.10722100201991</v>
+      </c>
+      <c r="N49">
+        <f>N13*(1-'Learning Rates'!$V62)</f>
+        <v>144.38208338435459</v>
+      </c>
+      <c r="O49">
+        <f>O13*(1-'Learning Rates'!$V62)</f>
+        <v>214.76840376307675</v>
+      </c>
+      <c r="P49">
+        <f>P13*(1-'Learning Rates'!$V62)</f>
+        <v>168.53609729263738</v>
+      </c>
+      <c r="Q49">
+        <f>Q13*(1-'Learning Rates'!$V62)</f>
+        <v>102.19803896749212</v>
+      </c>
+      <c r="R49">
+        <f>R13*(1-'Learning Rates'!$V62)</f>
+        <v>171.81472301046142</v>
+      </c>
+      <c r="S49">
+        <f>S13*(1-'Learning Rates'!$V62)</f>
+        <v>0.10327660945984019</v>
+      </c>
+    </row>
+    <row r="50" spans="12:19" x14ac:dyDescent="0.25">
+      <c r="L50">
+        <v>2035</v>
+      </c>
+      <c r="M50">
+        <f>M14*(1-'Learning Rates'!$V63)</f>
+        <v>242.0692893991982</v>
+      </c>
+      <c r="N50">
+        <f>N14*(1-'Learning Rates'!$V63)</f>
+        <v>113.43605713998298</v>
+      </c>
+      <c r="O50">
+        <f>O14*(1-'Learning Rates'!$V63)</f>
+        <v>165.98622977670854</v>
+      </c>
+      <c r="P50">
+        <f>P14*(1-'Learning Rates'!$V63)</f>
+        <v>119.65308887932289</v>
+      </c>
+      <c r="Q50">
+        <f>Q14*(1-'Learning Rates'!$V63)</f>
+        <v>84.845319504206103</v>
+      </c>
+      <c r="R50">
+        <f>R14*(1-'Learning Rates'!$V63)</f>
+        <v>144.71167421773845</v>
+      </c>
+      <c r="S50">
+        <f>S14*(1-'Learning Rates'!$V63)</f>
+        <v>8.6985159365853715E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="12:19" x14ac:dyDescent="0.25">
+      <c r="L51">
+        <v>2040</v>
+      </c>
+      <c r="M51">
+        <f>M15*(1-'Learning Rates'!$V64)</f>
+        <v>206.33941648999937</v>
+      </c>
+      <c r="N51">
+        <f>N15*(1-'Learning Rates'!$V64)</f>
+        <v>96.692686202712679</v>
+      </c>
+      <c r="O51">
+        <f>O15*(1-'Learning Rates'!$V64)</f>
+        <v>139.18050754172953</v>
+      </c>
+      <c r="P51">
+        <f>P15*(1-'Learning Rates'!$V64)</f>
+        <v>92.163631837741562</v>
+      </c>
+      <c r="Q51">
+        <f>Q15*(1-'Learning Rates'!$V64)</f>
+        <v>76.421912295062768</v>
+      </c>
+      <c r="R51">
+        <f>R15*(1-'Learning Rates'!$V64)</f>
+        <v>132.2365298886231</v>
+      </c>
+      <c r="S51">
+        <f>S15*(1-'Learning Rates'!$V64)</f>
+        <v>7.9486438730866318E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="12:19" x14ac:dyDescent="0.25">
+      <c r="L52">
+        <v>2045</v>
+      </c>
+      <c r="M52">
+        <f>M16*(1-'Learning Rates'!$V65)</f>
+        <v>175.88333862219545</v>
+      </c>
+      <c r="N52">
+        <f>N16*(1-'Learning Rates'!$V65)</f>
+        <v>82.420667650311316</v>
+      </c>
+      <c r="O52">
+        <f>O16*(1-'Learning Rates'!$V65)</f>
+        <v>116.70373925374641</v>
+      </c>
+      <c r="P52">
+        <f>P16*(1-'Learning Rates'!$V65)</f>
+        <v>70.989684537852582</v>
+      </c>
+      <c r="Q52">
+        <f>Q16*(1-'Learning Rates'!$V65)</f>
+        <v>68.834777368535214</v>
+      </c>
+      <c r="R52">
+        <f>R16*(1-'Learning Rates'!$V65)</f>
+        <v>120.83682903615555</v>
+      </c>
+      <c r="S52">
+        <f>S16*(1-'Learning Rates'!$V65)</f>
+        <v>7.2634159529929576E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="12:19" x14ac:dyDescent="0.25">
+      <c r="L53">
+        <v>2050</v>
+      </c>
+      <c r="M53">
+        <f>M17*(1-'Learning Rates'!$V66)</f>
+        <v>149.92263393547586</v>
+      </c>
+      <c r="N53">
+        <f>N17*(1-'Learning Rates'!$V66)</f>
+        <v>70.255225319539136</v>
+      </c>
+      <c r="O53">
+        <f>O17*(1-'Learning Rates'!$V66)</f>
+        <v>97.856826335562218</v>
+      </c>
+      <c r="P53">
+        <f>P17*(1-'Learning Rates'!$V66)</f>
+        <v>54.680302960024065</v>
+      </c>
+      <c r="Q53">
+        <f>Q17*(1-'Learning Rates'!$V66)</f>
+        <v>62.000889968333311</v>
+      </c>
+      <c r="R53">
+        <f>R17*(1-'Learning Rates'!$V66)</f>
+        <v>110.4198610157973</v>
+      </c>
+      <c r="S53">
+        <f>S17*(1-'Learning Rates'!$V66)</f>
+        <v>6.6372594053211498E-2</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="L1:S1"/>
+    <mergeCell ref="L10:S10"/>
+    <mergeCell ref="L19:S19"/>
+    <mergeCell ref="L28:S28"/>
+    <mergeCell ref="L37:S37"/>
+    <mergeCell ref="L46:S46"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
updated plots for tax credits
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8416BD9-4BAB-42FF-AAD8-E83D60A7E738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBE6802-D1D5-4907-8C0B-24115ECD51E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="4" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="123">
   <si>
     <t>Tech</t>
   </si>
@@ -409,6 +409,9 @@
   </si>
   <si>
     <t>DAC Hubs</t>
+  </si>
+  <si>
+    <t>Avg. Price CDR (High scenario)</t>
   </si>
 </sst>
 </file>
@@ -521,10 +524,10 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4765,24 +4768,24 @@
       <c r="E5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="P5" s="18" t="s">
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="P5" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="18"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="18"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
       <c r="Y5">
         <v>2021</v>
       </c>
@@ -5307,24 +5310,24 @@
       <c r="E14" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="H14" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="P14" s="18" t="s">
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="P14" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="18"/>
-      <c r="T14" s="18"/>
-      <c r="U14" s="18"/>
-      <c r="V14" s="18"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -5811,24 +5814,24 @@
         <f t="shared" si="14"/>
         <v>3512.6225095265308</v>
       </c>
-      <c r="H23" s="18" t="s">
+      <c r="H23" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-      <c r="P23" s="18" t="s">
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="P23" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="18"/>
-      <c r="T23" s="18"/>
-      <c r="U23" s="18"/>
-      <c r="V23" s="18"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="19"/>
+      <c r="U23" s="19"/>
+      <c r="V23" s="19"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="H24" s="13" t="s">
@@ -6227,24 +6230,24 @@
       <c r="V31" s="10"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H32" s="19" t="s">
+      <c r="H32" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19"/>
-      <c r="N32" s="19"/>
-      <c r="P32" s="19" t="s">
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+      <c r="P32" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="Q32" s="19"/>
-      <c r="R32" s="19"/>
-      <c r="S32" s="19"/>
-      <c r="T32" s="19"/>
-      <c r="U32" s="19"/>
-      <c r="V32" s="19"/>
+      <c r="Q32" s="18"/>
+      <c r="R32" s="18"/>
+      <c r="S32" s="18"/>
+      <c r="T32" s="18"/>
+      <c r="U32" s="18"/>
+      <c r="V32" s="18"/>
     </row>
     <row r="33" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H33" s="14" t="s">
@@ -6643,24 +6646,24 @@
       <c r="V40" s="10"/>
     </row>
     <row r="41" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H41" s="19" t="s">
+      <c r="H41" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="I41" s="19"/>
-      <c r="J41" s="19"/>
-      <c r="K41" s="19"/>
-      <c r="L41" s="19"/>
-      <c r="M41" s="19"/>
-      <c r="N41" s="19"/>
-      <c r="P41" s="19" t="s">
+      <c r="I41" s="18"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="18"/>
+      <c r="M41" s="18"/>
+      <c r="N41" s="18"/>
+      <c r="P41" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="Q41" s="19"/>
-      <c r="R41" s="19"/>
-      <c r="S41" s="19"/>
-      <c r="T41" s="19"/>
-      <c r="U41" s="19"/>
-      <c r="V41" s="19"/>
+      <c r="Q41" s="18"/>
+      <c r="R41" s="18"/>
+      <c r="S41" s="18"/>
+      <c r="T41" s="18"/>
+      <c r="U41" s="18"/>
+      <c r="V41" s="18"/>
     </row>
     <row r="42" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H42" s="14" t="s">
@@ -7059,24 +7062,24 @@
       <c r="V49" s="10"/>
     </row>
     <row r="50" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H50" s="19" t="s">
+      <c r="H50" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="I50" s="19"/>
-      <c r="J50" s="19"/>
-      <c r="K50" s="19"/>
-      <c r="L50" s="19"/>
-      <c r="M50" s="19"/>
-      <c r="N50" s="19"/>
-      <c r="P50" s="19" t="s">
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18"/>
+      <c r="N50" s="18"/>
+      <c r="P50" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="Q50" s="19"/>
-      <c r="R50" s="19"/>
-      <c r="S50" s="19"/>
-      <c r="T50" s="19"/>
-      <c r="U50" s="19"/>
-      <c r="V50" s="19"/>
+      <c r="Q50" s="18"/>
+      <c r="R50" s="18"/>
+      <c r="S50" s="18"/>
+      <c r="T50" s="18"/>
+      <c r="U50" s="18"/>
+      <c r="V50" s="18"/>
     </row>
     <row r="51" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H51" s="14" t="s">
@@ -7462,24 +7465,24 @@
       <c r="P58" s="13"/>
     </row>
     <row r="59" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H59" s="19" t="s">
+      <c r="H59" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="I59" s="19"/>
-      <c r="J59" s="19"/>
-      <c r="K59" s="19"/>
-      <c r="L59" s="19"/>
-      <c r="M59" s="19"/>
-      <c r="N59" s="19"/>
-      <c r="P59" s="19" t="s">
+      <c r="I59" s="18"/>
+      <c r="J59" s="18"/>
+      <c r="K59" s="18"/>
+      <c r="L59" s="18"/>
+      <c r="M59" s="18"/>
+      <c r="N59" s="18"/>
+      <c r="P59" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="Q59" s="19"/>
-      <c r="R59" s="19"/>
-      <c r="S59" s="19"/>
-      <c r="T59" s="19"/>
-      <c r="U59" s="19"/>
-      <c r="V59" s="19"/>
+      <c r="Q59" s="18"/>
+      <c r="R59" s="18"/>
+      <c r="S59" s="18"/>
+      <c r="T59" s="18"/>
+      <c r="U59" s="18"/>
+      <c r="V59" s="18"/>
     </row>
     <row r="60" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H60" s="14" t="s">
@@ -7863,6 +7866,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P23:V23"/>
     <mergeCell ref="P32:V32"/>
     <mergeCell ref="P41:V41"/>
     <mergeCell ref="P59:V59"/>
@@ -7871,12 +7880,6 @@
     <mergeCell ref="H32:N32"/>
     <mergeCell ref="H59:N59"/>
     <mergeCell ref="P50:V50"/>
-    <mergeCell ref="H14:N14"/>
-    <mergeCell ref="H23:N23"/>
-    <mergeCell ref="H5:N5"/>
-    <mergeCell ref="P5:V5"/>
-    <mergeCell ref="P14:V14"/>
-    <mergeCell ref="P23:V23"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="I52:N57">
@@ -10094,12 +10097,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="L46:S46"/>
     <mergeCell ref="L1:S1"/>
     <mergeCell ref="L10:S10"/>
     <mergeCell ref="L19:S19"/>
     <mergeCell ref="L28:S28"/>
     <mergeCell ref="L37:S37"/>
-    <mergeCell ref="L46:S46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10663,6 +10666,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8195A587-BA09-4421-98D4-BDAFBA104359}">
   <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
@@ -10711,14 +10722,14 @@
       <c r="A3">
         <v>2025</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="5">
         <v>0.05</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="5">
         <f>K3/$J3</f>
         <v>9.1538218144439369</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="5">
         <f>L3/$J3</f>
         <v>0</v>
       </c>
@@ -10726,13 +10737,13 @@
         <f>A3</f>
         <v>2025</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="5">
         <v>360.50516023732143</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="5">
         <v>3300</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="5">
         <v>0</v>
       </c>
     </row>
@@ -10740,14 +10751,14 @@
       <c r="A4">
         <v>2030</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="5">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="5">
         <f t="shared" ref="C4:C8" si="0">K4/$J4</f>
         <v>11.117978504373452</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="5">
         <f t="shared" ref="D4:D8" si="1">L4/$J4</f>
         <v>67.381687905293646</v>
       </c>
@@ -10755,13 +10766,13 @@
         <f t="shared" ref="I4:I8" si="2">A4</f>
         <v>2030</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="5">
         <v>296.81654796345282</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="5">
         <v>3300</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="5">
         <v>20000</v>
       </c>
     </row>
@@ -10769,14 +10780,14 @@
       <c r="A5">
         <v>2035</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="5">
         <v>10</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="5">
         <f t="shared" si="0"/>
         <v>14.945046646834507</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="5">
         <f t="shared" si="1"/>
         <v>158.50807049672963</v>
       </c>
@@ -10784,13 +10795,13 @@
         <f t="shared" si="2"/>
         <v>2035</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="5">
         <v>220.8089461332641</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="5">
         <v>3300</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="5">
         <f>(L4+L6)/2</f>
         <v>35000</v>
       </c>
@@ -10799,14 +10810,14 @@
       <c r="A6">
         <v>2040</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5">
         <v>0</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5">
         <f t="shared" si="1"/>
         <v>246.90690563233255</v>
       </c>
@@ -10814,13 +10825,13 @@
         <f t="shared" si="2"/>
         <v>2040</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="5">
         <v>202.50547416626196</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="5">
         <v>0</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="5">
         <v>50000</v>
       </c>
     </row>
@@ -10828,14 +10839,14 @@
       <c r="A7">
         <v>2045</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="5">
         <v>0</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="5">
         <f t="shared" si="1"/>
         <v>406.1713779405772</v>
       </c>
@@ -10843,13 +10854,13 @@
         <f t="shared" si="2"/>
         <v>2045</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="5">
         <v>184.65112037257458</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="5">
         <v>0</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="5">
         <f>(L6+L8)/2</f>
         <v>75000</v>
       </c>
@@ -10858,14 +10869,14 @@
       <c r="A8">
         <v>2050</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="5">
         <v>0</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="5">
         <f t="shared" si="1"/>
         <v>578.25596171173243</v>
       </c>
@@ -10873,13 +10884,13 @@
         <f t="shared" si="2"/>
         <v>2050</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="5">
         <v>172.93379856211703</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="5">
         <v>0</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="5">
         <v>100000</v>
       </c>
     </row>
@@ -10934,7 +10945,7 @@
         <v>40</v>
       </c>
       <c r="J13" t="s">
-        <v>53</v>
+        <v>122</v>
       </c>
       <c r="K13" t="s">
         <v>48</v>
@@ -10947,14 +10958,14 @@
       <c r="A14">
         <v>2025</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="5">
         <v>0.05</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="5">
         <f>K14/$J14</f>
         <v>9.1527704871198079</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="5">
         <f>L14/$J14</f>
         <v>0</v>
       </c>
@@ -10962,13 +10973,13 @@
         <f>A14</f>
         <v>2025</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="5">
         <v>360.54656943970235</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="5">
         <v>3300</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="5">
         <v>0</v>
       </c>
     </row>
@@ -10976,14 +10987,14 @@
       <c r="A15">
         <v>2030</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="5">
         <v>5</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="5">
         <f t="shared" ref="C15:C19" si="3">K15/$J15</f>
         <v>11.123317675046577</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="5">
         <f t="shared" ref="D15:D19" si="4">L15/$J15</f>
         <v>67.41404651543381</v>
       </c>
@@ -10991,13 +11002,13 @@
         <f t="shared" ref="I15:I19" si="5">A15</f>
         <v>2030</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="5">
         <v>296.67407660243612</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="5">
         <v>3300</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="5">
         <v>20000</v>
       </c>
     </row>
@@ -11005,14 +11016,14 @@
       <c r="A16">
         <v>2035</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="5">
         <v>10</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="5">
         <f t="shared" si="3"/>
         <v>14.849857137390348</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="5">
         <f t="shared" si="4"/>
         <v>157.49848479050368</v>
       </c>
@@ -11020,13 +11031,13 @@
         <f t="shared" si="5"/>
         <v>2035</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="5">
         <v>222.22436010451264</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="5">
         <v>3300</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="5">
         <f>(L15+L17)/2</f>
         <v>35000</v>
       </c>
@@ -11035,14 +11046,14 @@
       <c r="A17">
         <v>2040</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="5">
         <v>0</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="5">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="5">
         <f t="shared" si="4"/>
         <v>243.06758416564975</v>
       </c>
@@ -11050,13 +11061,13 @@
         <f t="shared" si="5"/>
         <v>2040</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="5">
         <v>205.70410559527826</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="5">
         <v>0</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="5">
         <v>50000</v>
       </c>
     </row>
@@ -11064,14 +11075,14 @@
       <c r="A18">
         <v>2045</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="5">
         <v>0</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="5">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="5">
         <f t="shared" si="4"/>
         <v>380.4751980809001</v>
       </c>
@@ -11079,13 +11090,13 @@
         <f t="shared" si="5"/>
         <v>2045</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="5">
         <v>197.12191590489118</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="5">
         <v>0</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="5">
         <f>(L17+L19)/2</f>
         <v>75000</v>
       </c>
@@ -11094,14 +11105,14 @@
       <c r="A19">
         <v>2050</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="5">
         <v>0</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="5">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="5">
         <f t="shared" si="4"/>
         <v>474.18677475115379</v>
       </c>
@@ -11109,13 +11120,13 @@
         <f t="shared" si="5"/>
         <v>2050</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="5">
         <v>210.88736617017318</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="5">
         <v>0</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="5">
         <v>100000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add procurement to nothing scenarios
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBE6802-D1D5-4907-8C0B-24115ECD51E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC4D50F-EBC6-497A-961B-C677FB9575FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="4" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="125">
   <si>
     <t>Tech</t>
   </si>
@@ -412,6 +412,12 @@
   </si>
   <si>
     <t>Avg. Price CDR (High scenario)</t>
+  </si>
+  <si>
+    <t>NOTHING</t>
+  </si>
+  <si>
+    <t>Avg. Price CDR (Nothing scenario)</t>
   </si>
 </sst>
 </file>
@@ -524,10 +530,10 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4768,24 +4774,24 @@
       <c r="E5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="P5" s="19" t="s">
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="P5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
       <c r="Y5">
         <v>2021</v>
       </c>
@@ -5310,24 +5316,24 @@
       <c r="E14" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="19"/>
-      <c r="P14" s="19" t="s">
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="P14" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="19"/>
-      <c r="R14" s="19"/>
-      <c r="S14" s="19"/>
-      <c r="T14" s="19"/>
-      <c r="U14" s="19"/>
-      <c r="V14" s="19"/>
+      <c r="Q14" s="18"/>
+      <c r="R14" s="18"/>
+      <c r="S14" s="18"/>
+      <c r="T14" s="18"/>
+      <c r="U14" s="18"/>
+      <c r="V14" s="18"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -5814,24 +5820,24 @@
         <f t="shared" si="14"/>
         <v>3512.6225095265308</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="P23" s="19" t="s">
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="18"/>
+      <c r="M23" s="18"/>
+      <c r="N23" s="18"/>
+      <c r="P23" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="19"/>
-      <c r="S23" s="19"/>
-      <c r="T23" s="19"/>
-      <c r="U23" s="19"/>
-      <c r="V23" s="19"/>
+      <c r="Q23" s="18"/>
+      <c r="R23" s="18"/>
+      <c r="S23" s="18"/>
+      <c r="T23" s="18"/>
+      <c r="U23" s="18"/>
+      <c r="V23" s="18"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="H24" s="13" t="s">
@@ -6230,24 +6236,24 @@
       <c r="V31" s="10"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H32" s="18" t="s">
+      <c r="H32" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="P32" s="18" t="s">
+      <c r="I32" s="19"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
+      <c r="P32" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="Q32" s="18"/>
-      <c r="R32" s="18"/>
-      <c r="S32" s="18"/>
-      <c r="T32" s="18"/>
-      <c r="U32" s="18"/>
-      <c r="V32" s="18"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="19"/>
+      <c r="S32" s="19"/>
+      <c r="T32" s="19"/>
+      <c r="U32" s="19"/>
+      <c r="V32" s="19"/>
     </row>
     <row r="33" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H33" s="14" t="s">
@@ -6646,24 +6652,24 @@
       <c r="V40" s="10"/>
     </row>
     <row r="41" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H41" s="18" t="s">
+      <c r="H41" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="I41" s="18"/>
-      <c r="J41" s="18"/>
-      <c r="K41" s="18"/>
-      <c r="L41" s="18"/>
-      <c r="M41" s="18"/>
-      <c r="N41" s="18"/>
-      <c r="P41" s="18" t="s">
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
+      <c r="N41" s="19"/>
+      <c r="P41" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="Q41" s="18"/>
-      <c r="R41" s="18"/>
-      <c r="S41" s="18"/>
-      <c r="T41" s="18"/>
-      <c r="U41" s="18"/>
-      <c r="V41" s="18"/>
+      <c r="Q41" s="19"/>
+      <c r="R41" s="19"/>
+      <c r="S41" s="19"/>
+      <c r="T41" s="19"/>
+      <c r="U41" s="19"/>
+      <c r="V41" s="19"/>
     </row>
     <row r="42" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H42" s="14" t="s">
@@ -7062,24 +7068,24 @@
       <c r="V49" s="10"/>
     </row>
     <row r="50" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H50" s="18" t="s">
+      <c r="H50" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="I50" s="18"/>
-      <c r="J50" s="18"/>
-      <c r="K50" s="18"/>
-      <c r="L50" s="18"/>
-      <c r="M50" s="18"/>
-      <c r="N50" s="18"/>
-      <c r="P50" s="18" t="s">
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
+      <c r="K50" s="19"/>
+      <c r="L50" s="19"/>
+      <c r="M50" s="19"/>
+      <c r="N50" s="19"/>
+      <c r="P50" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="Q50" s="18"/>
-      <c r="R50" s="18"/>
-      <c r="S50" s="18"/>
-      <c r="T50" s="18"/>
-      <c r="U50" s="18"/>
-      <c r="V50" s="18"/>
+      <c r="Q50" s="19"/>
+      <c r="R50" s="19"/>
+      <c r="S50" s="19"/>
+      <c r="T50" s="19"/>
+      <c r="U50" s="19"/>
+      <c r="V50" s="19"/>
     </row>
     <row r="51" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H51" s="14" t="s">
@@ -7465,24 +7471,24 @@
       <c r="P58" s="13"/>
     </row>
     <row r="59" spans="8:22" x14ac:dyDescent="0.25">
-      <c r="H59" s="18" t="s">
+      <c r="H59" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="I59" s="18"/>
-      <c r="J59" s="18"/>
-      <c r="K59" s="18"/>
-      <c r="L59" s="18"/>
-      <c r="M59" s="18"/>
-      <c r="N59" s="18"/>
-      <c r="P59" s="18" t="s">
+      <c r="I59" s="19"/>
+      <c r="J59" s="19"/>
+      <c r="K59" s="19"/>
+      <c r="L59" s="19"/>
+      <c r="M59" s="19"/>
+      <c r="N59" s="19"/>
+      <c r="P59" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="Q59" s="18"/>
-      <c r="R59" s="18"/>
-      <c r="S59" s="18"/>
-      <c r="T59" s="18"/>
-      <c r="U59" s="18"/>
-      <c r="V59" s="18"/>
+      <c r="Q59" s="19"/>
+      <c r="R59" s="19"/>
+      <c r="S59" s="19"/>
+      <c r="T59" s="19"/>
+      <c r="U59" s="19"/>
+      <c r="V59" s="19"/>
     </row>
     <row r="60" spans="8:22" x14ac:dyDescent="0.25">
       <c r="H60" s="14" t="s">
@@ -7866,12 +7872,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H14:N14"/>
-    <mergeCell ref="H23:N23"/>
-    <mergeCell ref="H5:N5"/>
-    <mergeCell ref="P5:V5"/>
-    <mergeCell ref="P14:V14"/>
-    <mergeCell ref="P23:V23"/>
     <mergeCell ref="P32:V32"/>
     <mergeCell ref="P41:V41"/>
     <mergeCell ref="P59:V59"/>
@@ -7880,6 +7880,12 @@
     <mergeCell ref="H32:N32"/>
     <mergeCell ref="H59:N59"/>
     <mergeCell ref="P50:V50"/>
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P23:V23"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="I52:N57">
@@ -10664,10 +10670,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8195A587-BA09-4421-98D4-BDAFBA104359}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="27.42578125" bestFit="1" customWidth="1"/>
@@ -11147,6 +11153,242 @@
         <v>49</v>
       </c>
     </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
+      </c>
+      <c r="I22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>44</v>
+      </c>
+      <c r="I23" t="s">
+        <v>40</v>
+      </c>
+      <c r="J23" t="s">
+        <v>124</v>
+      </c>
+      <c r="K23" t="s">
+        <v>48</v>
+      </c>
+      <c r="L23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2025</v>
+      </c>
+      <c r="B24" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="C24" s="5">
+        <f>K24/$J24</f>
+        <v>9.1497691446116427</v>
+      </c>
+      <c r="D24" s="5">
+        <f>L24/$J24</f>
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <f>A24</f>
+        <v>2025</v>
+      </c>
+      <c r="J24" s="5">
+        <v>360.6648373137798</v>
+      </c>
+      <c r="K24" s="5">
+        <v>3300</v>
+      </c>
+      <c r="L24" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2030</v>
+      </c>
+      <c r="B25" s="5">
+        <v>5</v>
+      </c>
+      <c r="C25" s="5">
+        <f t="shared" ref="C25:C29" si="6">K25/$J25</f>
+        <v>10.257766689126317</v>
+      </c>
+      <c r="D25" s="5">
+        <f t="shared" ref="D25:D29" si="7">L25/$J25</f>
+        <v>62.168282964401925</v>
+      </c>
+      <c r="I25">
+        <f t="shared" ref="I25:I29" si="8">A25</f>
+        <v>2030</v>
+      </c>
+      <c r="J25" s="5">
+        <v>321.70745348479653</v>
+      </c>
+      <c r="K25" s="5">
+        <v>3300</v>
+      </c>
+      <c r="L25" s="5">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2035</v>
+      </c>
+      <c r="B26" s="5">
+        <v>10</v>
+      </c>
+      <c r="C26" s="5">
+        <f t="shared" si="6"/>
+        <v>14.173567907117816</v>
+      </c>
+      <c r="D26" s="5">
+        <f t="shared" si="7"/>
+        <v>150.32572022700714</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="8"/>
+        <v>2035</v>
+      </c>
+      <c r="J26" s="5">
+        <v>232.82775527132975</v>
+      </c>
+      <c r="K26" s="5">
+        <v>3300</v>
+      </c>
+      <c r="L26" s="5">
+        <f>(L25+L27)/2</f>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2040</v>
+      </c>
+      <c r="B27" s="5">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="D27" s="5">
+        <f t="shared" si="7"/>
+        <v>230.33503394108612</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="8"/>
+        <v>2040</v>
+      </c>
+      <c r="J27" s="5">
+        <v>217.07509771522092</v>
+      </c>
+      <c r="K27" s="5">
+        <v>0</v>
+      </c>
+      <c r="L27" s="5">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2045</v>
+      </c>
+      <c r="B28" s="5">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="D28" s="5">
+        <f t="shared" si="7"/>
+        <v>394.18160776815387</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="8"/>
+        <v>2045</v>
+      </c>
+      <c r="J28" s="5">
+        <v>190.26762923985234</v>
+      </c>
+      <c r="K28" s="5">
+        <v>0</v>
+      </c>
+      <c r="L28" s="5">
+        <f>(L27+L29)/2</f>
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2050</v>
+      </c>
+      <c r="B29" s="5">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="D29" s="5">
+        <f t="shared" si="7"/>
+        <v>591.29305280005849</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="8"/>
+        <v>2050</v>
+      </c>
+      <c r="J29" s="5">
+        <v>169.12087758591389</v>
+      </c>
+      <c r="K29" s="5">
+        <v>0</v>
+      </c>
+      <c r="L29" s="5">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" t="s">
+        <v>43</v>
+      </c>
+      <c r="J30" t="s">
+        <v>52</v>
+      </c>
+      <c r="K30" t="s">
+        <v>50</v>
+      </c>
+      <c r="L30" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
100Mt baseline with cost decreases
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F52B6A2A-115A-4D63-B8C4-55D81385F736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95ADED34-BAFA-4EAD-B0CE-BACF1CC9882F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -487,7 +487,7 @@
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="171" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -607,18 +607,18 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="0" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -4725,35 +4725,35 @@
         <f>1-2^V3</f>
         <v>4.9999617125113915E-2</v>
       </c>
-      <c r="W2" s="25">
+      <c r="W2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="X2" s="25">
+      <c r="X2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="Y2" s="25">
+      <c r="Y2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="Z2" s="25">
+      <c r="Z2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="AA2" s="25">
+      <c r="AA2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="AB2" s="25">
+      <c r="AB2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="AC2" s="25">
+      <c r="AC2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
-      <c r="AD2" s="25">
+      <c r="AD2" s="22">
         <f t="shared" si="4"/>
         <v>2.4982512346666597E-2</v>
       </c>
@@ -5075,24 +5075,24 @@
       <c r="E5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="P5" s="23" t="s">
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="25"/>
+      <c r="P5" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" s="23"/>
-      <c r="R5" s="23"/>
-      <c r="S5" s="23"/>
-      <c r="T5" s="23"/>
-      <c r="U5" s="23"/>
-      <c r="V5" s="23"/>
+      <c r="Q5" s="25"/>
+      <c r="R5" s="25"/>
+      <c r="S5" s="25"/>
+      <c r="T5" s="25"/>
+      <c r="U5" s="25"/>
+      <c r="V5" s="25"/>
       <c r="AP5">
         <v>2021</v>
       </c>
@@ -6049,24 +6049,24 @@
       <c r="E14" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="H14" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="P14" s="23" t="s">
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="25"/>
+      <c r="N14" s="25"/>
+      <c r="P14" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="23"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="23"/>
-      <c r="T14" s="23"/>
-      <c r="U14" s="23"/>
-      <c r="V14" s="23"/>
+      <c r="Q14" s="25"/>
+      <c r="R14" s="25"/>
+      <c r="S14" s="25"/>
+      <c r="T14" s="25"/>
+      <c r="U14" s="25"/>
+      <c r="V14" s="25"/>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -6365,14 +6365,14 @@
       <c r="AA17" s="16">
         <v>3018</v>
       </c>
-      <c r="AB17" s="20">
-        <v>0</v>
+      <c r="AB17" s="16">
+        <v>3759</v>
       </c>
       <c r="AC17" s="16">
         <v>4137</v>
       </c>
-      <c r="AD17" s="20">
-        <v>0</v>
+      <c r="AD17" s="16">
+        <v>4609</v>
       </c>
       <c r="AE17" s="20">
         <v>0</v>
@@ -6889,24 +6889,24 @@
         <f t="shared" si="45"/>
         <v>3512.6225095265308</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="23"/>
-      <c r="P23" s="23" t="s">
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="25"/>
+      <c r="N23" s="25"/>
+      <c r="P23" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="Q23" s="23"/>
-      <c r="R23" s="23"/>
-      <c r="S23" s="23"/>
-      <c r="T23" s="23"/>
-      <c r="U23" s="23"/>
-      <c r="V23" s="23"/>
+      <c r="Q23" s="25"/>
+      <c r="R23" s="25"/>
+      <c r="S23" s="25"/>
+      <c r="T23" s="25"/>
+      <c r="U23" s="25"/>
+      <c r="V23" s="25"/>
     </row>
     <row r="24" spans="1:38" x14ac:dyDescent="0.25">
       <c r="H24" s="13" t="s">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="AB26" s="10">
         <f t="shared" si="54"/>
-        <v>9949</v>
+        <v>17467</v>
       </c>
       <c r="AC26" s="10">
         <f t="shared" si="54"/>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="AD26" s="10">
         <f t="shared" si="54"/>
-        <v>9949</v>
+        <v>19167</v>
       </c>
       <c r="AE26" s="10">
         <f t="shared" si="53"/>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="AB27" s="10">
         <f t="shared" si="59"/>
-        <v>9949</v>
+        <v>17467</v>
       </c>
       <c r="AC27" s="10">
         <f t="shared" si="59"/>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="AD27" s="10">
         <f t="shared" si="58"/>
-        <v>9949</v>
+        <v>19167</v>
       </c>
       <c r="AE27" s="10">
         <f t="shared" si="58"/>
@@ -7437,7 +7437,7 @@
       </c>
       <c r="AB28" s="10">
         <f t="shared" si="62"/>
-        <v>9949</v>
+        <v>17467</v>
       </c>
       <c r="AC28" s="10">
         <f t="shared" si="62"/>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="AD28" s="10">
         <f t="shared" si="61"/>
-        <v>9949</v>
+        <v>19167</v>
       </c>
       <c r="AE28" s="10">
         <f t="shared" si="61"/>
@@ -7557,7 +7557,7 @@
       </c>
       <c r="AB29" s="10">
         <f t="shared" si="65"/>
-        <v>9949</v>
+        <v>17467</v>
       </c>
       <c r="AC29" s="10">
         <f t="shared" si="65"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="AD29" s="10">
         <f t="shared" si="64"/>
-        <v>9949</v>
+        <v>19167</v>
       </c>
       <c r="AE29" s="10">
         <f t="shared" si="64"/>
@@ -7677,7 +7677,7 @@
       </c>
       <c r="AB30" s="10">
         <f t="shared" si="68"/>
-        <v>9949</v>
+        <v>17467</v>
       </c>
       <c r="AC30" s="10">
         <f t="shared" si="68"/>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="AD30" s="10">
         <f t="shared" si="67"/>
-        <v>9949</v>
+        <v>19167</v>
       </c>
       <c r="AE30" s="10">
         <f t="shared" si="67"/>
@@ -7737,24 +7737,24 @@
       <c r="V31" s="10"/>
     </row>
     <row r="32" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="H32" s="22" t="s">
+      <c r="H32" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="I32" s="22"/>
-      <c r="J32" s="22"/>
-      <c r="K32" s="22"/>
-      <c r="L32" s="22"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="22"/>
-      <c r="P32" s="22" t="s">
+      <c r="I32" s="26"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="26"/>
+      <c r="P32" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="Q32" s="22"/>
-      <c r="R32" s="22"/>
-      <c r="S32" s="22"/>
-      <c r="T32" s="22"/>
-      <c r="U32" s="22"/>
-      <c r="V32" s="22"/>
+      <c r="Q32" s="26"/>
+      <c r="R32" s="26"/>
+      <c r="S32" s="26"/>
+      <c r="T32" s="26"/>
+      <c r="U32" s="26"/>
+      <c r="V32" s="26"/>
     </row>
     <row r="33" spans="8:38" x14ac:dyDescent="0.25">
       <c r="H33" s="14" t="s">
@@ -8585,24 +8585,24 @@
       <c r="V40" s="10"/>
     </row>
     <row r="41" spans="8:38" x14ac:dyDescent="0.25">
-      <c r="H41" s="22" t="s">
+      <c r="H41" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
-      <c r="N41" s="22"/>
-      <c r="P41" s="22" t="s">
+      <c r="I41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
+      <c r="N41" s="26"/>
+      <c r="P41" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="Q41" s="22"/>
-      <c r="R41" s="22"/>
-      <c r="S41" s="22"/>
-      <c r="T41" s="22"/>
-      <c r="U41" s="22"/>
-      <c r="V41" s="22"/>
+      <c r="Q41" s="26"/>
+      <c r="R41" s="26"/>
+      <c r="S41" s="26"/>
+      <c r="T41" s="26"/>
+      <c r="U41" s="26"/>
+      <c r="V41" s="26"/>
       <c r="Y41" s="18"/>
       <c r="Z41" s="18"/>
       <c r="AA41" s="18"/>
@@ -8902,7 +8902,7 @@
       </c>
       <c r="AB44" s="10">
         <f t="shared" si="80"/>
-        <v>278.39198659252952</v>
+        <v>272.73112922434825</v>
       </c>
       <c r="AC44" s="10">
         <f t="shared" si="80"/>
@@ -8910,7 +8910,7 @@
       </c>
       <c r="AD44" s="10">
         <f t="shared" si="79"/>
-        <v>278.39198659252952</v>
+        <v>271.80813653466583</v>
       </c>
       <c r="AE44" s="10">
         <f t="shared" si="79"/>
@@ -9022,7 +9022,7 @@
       </c>
       <c r="AB45" s="10">
         <f t="shared" si="83"/>
-        <v>207.10247320513693</v>
+        <v>202.89122569129299</v>
       </c>
       <c r="AC45" s="10">
         <f t="shared" si="83"/>
@@ -9030,7 +9030,7 @@
       </c>
       <c r="AD45" s="10">
         <f t="shared" si="82"/>
-        <v>207.10247320513693</v>
+        <v>202.20458930091704</v>
       </c>
       <c r="AE45" s="10">
         <f t="shared" si="82"/>
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AB46" s="10">
         <f t="shared" si="86"/>
-        <v>189.935169167015</v>
+        <v>186.07300375408028</v>
       </c>
       <c r="AC46" s="10">
         <f t="shared" si="86"/>
@@ -9150,7 +9150,7 @@
       </c>
       <c r="AD46" s="10">
         <f t="shared" si="85"/>
-        <v>189.935169167015</v>
+        <v>185.44328457717259</v>
       </c>
       <c r="AE46" s="10">
         <f t="shared" si="85"/>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="AB47" s="10">
         <f t="shared" si="89"/>
-        <v>173.18910478463926</v>
+        <v>169.66745593292927</v>
       </c>
       <c r="AC47" s="10">
         <f t="shared" si="89"/>
@@ -9270,7 +9270,7 @@
       </c>
       <c r="AD47" s="10">
         <f t="shared" si="88"/>
-        <v>173.18910478463926</v>
+        <v>169.09325737353313</v>
       </c>
       <c r="AE47" s="10">
         <f t="shared" si="88"/>
@@ -9382,7 +9382,7 @@
       </c>
       <c r="AB48" s="10">
         <f t="shared" si="92"/>
-        <v>162.19912286234123</v>
+        <v>158.90094567338451</v>
       </c>
       <c r="AC48" s="10">
         <f t="shared" si="92"/>
@@ -9390,7 +9390,7 @@
       </c>
       <c r="AD48" s="10">
         <f t="shared" si="91"/>
-        <v>162.19912286234123</v>
+        <v>158.36318376972039</v>
       </c>
       <c r="AE48" s="10">
         <f t="shared" si="91"/>
@@ -9442,24 +9442,24 @@
       <c r="V49" s="10"/>
     </row>
     <row r="50" spans="8:38" x14ac:dyDescent="0.25">
-      <c r="H50" s="22" t="s">
+      <c r="H50" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="I50" s="22"/>
-      <c r="J50" s="22"/>
-      <c r="K50" s="22"/>
-      <c r="L50" s="22"/>
-      <c r="M50" s="22"/>
-      <c r="N50" s="22"/>
-      <c r="P50" s="22" t="s">
+      <c r="I50" s="26"/>
+      <c r="J50" s="26"/>
+      <c r="K50" s="26"/>
+      <c r="L50" s="26"/>
+      <c r="M50" s="26"/>
+      <c r="N50" s="26"/>
+      <c r="P50" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="Q50" s="22"/>
-      <c r="R50" s="22"/>
-      <c r="S50" s="22"/>
-      <c r="T50" s="22"/>
-      <c r="U50" s="22"/>
-      <c r="V50" s="22"/>
+      <c r="Q50" s="26"/>
+      <c r="R50" s="26"/>
+      <c r="S50" s="26"/>
+      <c r="T50" s="26"/>
+      <c r="U50" s="26"/>
+      <c r="V50" s="26"/>
     </row>
     <row r="51" spans="8:38" x14ac:dyDescent="0.25">
       <c r="H51" s="14" t="s">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="AB53" s="10">
         <f t="shared" si="102"/>
-        <v>18.4245613709233</v>
+        <v>24.085418739104568</v>
       </c>
       <c r="AC53" s="10">
         <f t="shared" si="102"/>
@@ -9758,7 +9758,7 @@
       </c>
       <c r="AD53" s="10">
         <f t="shared" si="101"/>
-        <v>18.4245613709233</v>
+        <v>25.008411428786985</v>
       </c>
       <c r="AE53" s="10">
         <f t="shared" si="101"/>
@@ -9870,7 +9870,7 @@
       </c>
       <c r="AB54" s="10">
         <f t="shared" si="106"/>
-        <v>13.70647292812717</v>
+        <v>17.917720441971113</v>
       </c>
       <c r="AC54" s="10">
         <f t="shared" si="106"/>
@@ -9878,7 +9878,7 @@
       </c>
       <c r="AD54" s="10">
         <f t="shared" si="105"/>
-        <v>13.70647292812717</v>
+        <v>18.604356832347065</v>
       </c>
       <c r="AE54" s="10">
         <f t="shared" si="105"/>
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AB55" s="10">
         <f t="shared" si="110"/>
-        <v>12.570304999246957</v>
+        <v>16.432470412181686</v>
       </c>
       <c r="AC55" s="10">
         <f t="shared" si="110"/>
@@ -9998,7 +9998,7 @@
       </c>
       <c r="AD55" s="10">
         <f t="shared" si="109"/>
-        <v>12.570304999246957</v>
+        <v>17.062189589089371</v>
       </c>
       <c r="AE55" s="10">
         <f t="shared" si="109"/>
@@ -10110,7 +10110,7 @@
       </c>
       <c r="AB56" s="10">
         <f t="shared" si="114"/>
-        <v>11.462015587935326</v>
+        <v>14.98366443964531</v>
       </c>
       <c r="AC56" s="10">
         <f t="shared" si="114"/>
@@ -10118,7 +10118,7 @@
       </c>
       <c r="AD56" s="10">
         <f t="shared" si="113"/>
-        <v>11.462015587935326</v>
+        <v>15.557862999041447</v>
       </c>
       <c r="AE56" s="10">
         <f t="shared" si="113"/>
@@ -10230,7 +10230,7 @@
       </c>
       <c r="AB57" s="10">
         <f t="shared" si="118"/>
-        <v>10.734675699775806</v>
+        <v>14.032852888732521</v>
       </c>
       <c r="AC57" s="10">
         <f t="shared" si="118"/>
@@ -10238,7 +10238,7 @@
       </c>
       <c r="AD57" s="10">
         <f t="shared" si="117"/>
-        <v>10.734675699775806</v>
+        <v>14.57061479239664</v>
       </c>
       <c r="AE57" s="10">
         <f t="shared" si="117"/>
@@ -10277,24 +10277,24 @@
       <c r="P58" s="13"/>
     </row>
     <row r="59" spans="8:38" x14ac:dyDescent="0.25">
-      <c r="H59" s="22" t="s">
+      <c r="H59" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
-      <c r="K59" s="22"/>
-      <c r="L59" s="22"/>
-      <c r="M59" s="22"/>
-      <c r="N59" s="22"/>
-      <c r="P59" s="22" t="s">
+      <c r="I59" s="26"/>
+      <c r="J59" s="26"/>
+      <c r="K59" s="26"/>
+      <c r="L59" s="26"/>
+      <c r="M59" s="26"/>
+      <c r="N59" s="26"/>
+      <c r="P59" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="Q59" s="22"/>
-      <c r="R59" s="22"/>
-      <c r="S59" s="22"/>
-      <c r="T59" s="22"/>
-      <c r="U59" s="22"/>
-      <c r="V59" s="22"/>
+      <c r="Q59" s="26"/>
+      <c r="R59" s="26"/>
+      <c r="S59" s="26"/>
+      <c r="T59" s="26"/>
+      <c r="U59" s="26"/>
+      <c r="V59" s="26"/>
     </row>
     <row r="60" spans="8:38" x14ac:dyDescent="0.25">
       <c r="H60" s="14" t="s">
@@ -10419,91 +10419,91 @@
       <c r="P61" s="14">
         <v>2025</v>
       </c>
-      <c r="Q61" s="26">
+      <c r="Q61" s="23">
         <f t="shared" ref="Q61:V66" si="121">Q52/Q34</f>
         <v>0</v>
       </c>
-      <c r="R61" s="26">
+      <c r="R61" s="23">
         <f t="shared" si="121"/>
         <v>2.159864871588402E-2</v>
       </c>
-      <c r="S61" s="26">
+      <c r="S61" s="23">
         <f t="shared" si="121"/>
         <v>5.1034239185863285E-2</v>
       </c>
-      <c r="T61" s="26">
+      <c r="T61" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316965E-2</v>
       </c>
-      <c r="U61" s="26">
+      <c r="U61" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316896E-2</v>
       </c>
-      <c r="V61" s="26">
+      <c r="V61" s="23">
         <f t="shared" si="121"/>
         <v>0</v>
       </c>
-      <c r="W61" s="26">
+      <c r="W61" s="23">
         <f t="shared" ref="W61:AH61" si="122">W52/W34</f>
         <v>0</v>
       </c>
-      <c r="X61" s="27">
+      <c r="X61" s="24">
         <f t="shared" si="122"/>
         <v>0</v>
       </c>
-      <c r="Y61" s="27">
+      <c r="Y61" s="24">
         <f t="shared" si="122"/>
         <v>0</v>
       </c>
-      <c r="Z61" s="27">
+      <c r="Z61" s="24">
         <f t="shared" ref="Z61:AC61" si="123">Z52/Z34</f>
         <v>6.207390220437408E-2</v>
       </c>
-      <c r="AA61" s="27">
+      <c r="AA61" s="24">
         <f t="shared" si="123"/>
         <v>6.207390220437408E-2</v>
       </c>
-      <c r="AB61" s="27">
+      <c r="AB61" s="24">
         <f t="shared" si="123"/>
         <v>6.207390220437408E-2</v>
       </c>
-      <c r="AC61" s="27">
+      <c r="AC61" s="24">
         <f t="shared" si="123"/>
         <v>6.207390220437408E-2</v>
       </c>
-      <c r="AD61" s="27">
+      <c r="AD61" s="24">
         <f t="shared" si="122"/>
         <v>6.207390220437408E-2</v>
       </c>
-      <c r="AE61" s="27">
+      <c r="AE61" s="24">
         <f t="shared" si="122"/>
         <v>0</v>
       </c>
-      <c r="AF61" s="27">
+      <c r="AF61" s="24">
         <f t="shared" si="122"/>
         <v>0</v>
       </c>
-      <c r="AG61" s="27">
+      <c r="AG61" s="24">
         <f t="shared" si="122"/>
         <v>0</v>
       </c>
-      <c r="AH61" s="27">
+      <c r="AH61" s="24">
         <f t="shared" si="122"/>
         <v>0</v>
       </c>
-      <c r="AI61" s="27">
+      <c r="AI61" s="24">
         <f t="shared" ref="AI61:AL61" si="124">AI52/AI34</f>
         <v>0</v>
       </c>
-      <c r="AJ61" s="27">
+      <c r="AJ61" s="24">
         <f t="shared" si="124"/>
         <v>0</v>
       </c>
-      <c r="AK61" s="27">
+      <c r="AK61" s="24">
         <f t="shared" si="124"/>
         <v>0</v>
       </c>
-      <c r="AL61" s="27">
+      <c r="AL61" s="24">
         <f t="shared" si="124"/>
         <v>0</v>
       </c>
@@ -10539,91 +10539,91 @@
       <c r="P62" s="14">
         <v>2030</v>
       </c>
-      <c r="Q62" s="26">
+      <c r="Q62" s="23">
         <f t="shared" si="121"/>
         <v>7.2005255799870646E-2</v>
       </c>
-      <c r="R62" s="26">
+      <c r="R62" s="23">
         <f t="shared" si="121"/>
         <v>3.7935815937008122E-2</v>
       </c>
-      <c r="S62" s="26">
+      <c r="S62" s="23">
         <f t="shared" si="121"/>
         <v>7.9415665577240849E-2</v>
       </c>
-      <c r="T62" s="26">
+      <c r="T62" s="23">
         <f t="shared" si="121"/>
         <v>7.889539208931684E-2</v>
       </c>
-      <c r="U62" s="26">
+      <c r="U62" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316979E-2</v>
       </c>
-      <c r="V62" s="26">
+      <c r="V62" s="23">
         <f t="shared" si="121"/>
         <v>0.12666875354809062</v>
       </c>
-      <c r="W62" s="26">
+      <c r="W62" s="23">
         <f t="shared" ref="W62:AH62" si="126">W53/W35</f>
         <v>6.4622457718525664E-2</v>
       </c>
-      <c r="X62" s="27">
+      <c r="X62" s="24">
         <f t="shared" si="126"/>
         <v>8.2558409986148301E-2</v>
       </c>
-      <c r="Y62" s="27">
+      <c r="Y62" s="24">
         <f t="shared" si="126"/>
         <v>0.1383767815890895</v>
       </c>
-      <c r="Z62" s="27">
+      <c r="Z62" s="24">
         <f t="shared" ref="Z62:AC62" si="127">Z53/Z35</f>
         <v>7.4447229516503746E-2</v>
       </c>
-      <c r="AA62" s="27">
+      <c r="AA62" s="24">
         <f t="shared" si="127"/>
         <v>7.8167409509664373E-2</v>
       </c>
-      <c r="AB62" s="27">
+      <c r="AB62" s="24">
         <f t="shared" si="127"/>
-        <v>6.207390220437415E-2</v>
-      </c>
-      <c r="AC62" s="27">
+        <v>8.1145808427332766E-2</v>
+      </c>
+      <c r="AC62" s="24">
         <f t="shared" si="127"/>
         <v>8.2565761170827728E-2</v>
       </c>
-      <c r="AD62" s="27">
+      <c r="AD62" s="24">
         <f t="shared" si="126"/>
-        <v>6.207390220437415E-2</v>
-      </c>
-      <c r="AE62" s="27">
+        <v>8.4255448695085167E-2</v>
+      </c>
+      <c r="AE62" s="24">
         <f t="shared" si="126"/>
         <v>0</v>
       </c>
-      <c r="AF62" s="27">
+      <c r="AF62" s="24">
         <f t="shared" si="126"/>
         <v>0</v>
       </c>
-      <c r="AG62" s="27">
+      <c r="AG62" s="24">
         <f t="shared" si="126"/>
         <v>0</v>
       </c>
-      <c r="AH62" s="27">
+      <c r="AH62" s="24">
         <f t="shared" si="126"/>
         <v>0</v>
       </c>
-      <c r="AI62" s="27">
+      <c r="AI62" s="24">
         <f t="shared" ref="AI62:AL62" si="128">AI53/AI35</f>
         <v>0</v>
       </c>
-      <c r="AJ62" s="27">
+      <c r="AJ62" s="24">
         <f t="shared" si="128"/>
         <v>0</v>
       </c>
-      <c r="AK62" s="27">
+      <c r="AK62" s="24">
         <f t="shared" si="128"/>
         <v>0</v>
       </c>
-      <c r="AL62" s="27">
+      <c r="AL62" s="24">
         <f t="shared" si="128"/>
         <v>0</v>
       </c>
@@ -10659,91 +10659,91 @@
       <c r="P63" s="14">
         <v>2035</v>
       </c>
-      <c r="Q63" s="26">
+      <c r="Q63" s="23">
         <f t="shared" si="121"/>
         <v>0.10518985801607014</v>
       </c>
-      <c r="R63" s="26">
+      <c r="R63" s="23">
         <f t="shared" si="121"/>
         <v>5.1034239185863375E-2</v>
       </c>
-      <c r="S63" s="26">
+      <c r="S63" s="23">
         <f t="shared" si="121"/>
         <v>9.8967839167066807E-2</v>
       </c>
-      <c r="T63" s="26">
+      <c r="T63" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316993E-2</v>
       </c>
-      <c r="U63" s="26">
+      <c r="U63" s="23">
         <f t="shared" si="121"/>
         <v>7.889539208931691E-2</v>
       </c>
-      <c r="V63" s="26">
+      <c r="V63" s="23">
         <f t="shared" si="121"/>
         <v>0.1651875193758317</v>
       </c>
-      <c r="W63" s="26">
+      <c r="W63" s="23">
         <f t="shared" ref="W63:AH63" si="129">W54/W36</f>
         <v>8.5203970166686849E-2</v>
       </c>
-      <c r="X63" s="27">
+      <c r="X63" s="24">
         <f t="shared" si="129"/>
         <v>0.10389919717415493</v>
       </c>
-      <c r="Y63" s="27">
+      <c r="Y63" s="24">
         <f t="shared" si="129"/>
         <v>0.16928290688878872</v>
       </c>
-      <c r="Z63" s="27">
+      <c r="Z63" s="24">
         <f t="shared" ref="Z63:AC63" si="130">Z54/Z36</f>
         <v>7.4447229516503829E-2</v>
       </c>
-      <c r="AA63" s="27">
+      <c r="AA63" s="24">
         <f t="shared" si="130"/>
         <v>7.8167409509664554E-2</v>
       </c>
-      <c r="AB63" s="27">
+      <c r="AB63" s="24">
         <f t="shared" si="130"/>
-        <v>6.2073902204374212E-2</v>
-      </c>
-      <c r="AC63" s="27">
+        <v>8.1145808427332877E-2</v>
+      </c>
+      <c r="AC63" s="24">
         <f t="shared" si="130"/>
         <v>8.2565761170827798E-2</v>
       </c>
-      <c r="AD63" s="27">
+      <c r="AD63" s="24">
         <f t="shared" si="129"/>
-        <v>6.2073902204374212E-2</v>
-      </c>
-      <c r="AE63" s="27">
+        <v>8.4255448695085194E-2</v>
+      </c>
+      <c r="AE63" s="24">
         <f t="shared" si="129"/>
         <v>0</v>
       </c>
-      <c r="AF63" s="27">
+      <c r="AF63" s="24">
         <f t="shared" si="129"/>
         <v>0</v>
       </c>
-      <c r="AG63" s="27">
+      <c r="AG63" s="24">
         <f t="shared" si="129"/>
         <v>0</v>
       </c>
-      <c r="AH63" s="27">
+      <c r="AH63" s="24">
         <f t="shared" si="129"/>
         <v>0</v>
       </c>
-      <c r="AI63" s="27">
+      <c r="AI63" s="24">
         <f t="shared" ref="AI63:AL63" si="131">AI54/AI36</f>
         <v>0</v>
       </c>
-      <c r="AJ63" s="27">
+      <c r="AJ63" s="24">
         <f t="shared" si="131"/>
         <v>0</v>
       </c>
-      <c r="AK63" s="27">
+      <c r="AK63" s="24">
         <f t="shared" si="131"/>
         <v>0</v>
       </c>
-      <c r="AL63" s="27">
+      <c r="AL63" s="24">
         <f t="shared" si="131"/>
         <v>0</v>
       </c>
@@ -10779,91 +10779,91 @@
       <c r="P64" s="14">
         <v>2040</v>
       </c>
-      <c r="Q64" s="26">
+      <c r="Q64" s="23">
         <f t="shared" si="121"/>
         <v>0.10518985801607007</v>
       </c>
-      <c r="R64" s="26">
+      <c r="R64" s="23">
         <f t="shared" si="121"/>
         <v>6.1942541927517823E-2</v>
       </c>
-      <c r="S64" s="26">
+      <c r="S64" s="23">
         <f t="shared" si="121"/>
         <v>0.11381917348346579</v>
       </c>
-      <c r="T64" s="26">
+      <c r="T64" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316882E-2</v>
       </c>
-      <c r="U64" s="26">
+      <c r="U64" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316854E-2</v>
       </c>
-      <c r="V64" s="26">
+      <c r="V64" s="23">
         <f t="shared" si="121"/>
         <v>0.16518751937583165</v>
       </c>
-      <c r="W64" s="26">
+      <c r="W64" s="23">
         <f t="shared" ref="W64:AH64" si="132">W55/W37</f>
         <v>8.5203970166686793E-2</v>
       </c>
-      <c r="X64" s="27">
+      <c r="X64" s="24">
         <f t="shared" si="132"/>
         <v>0.10389919717415487</v>
       </c>
-      <c r="Y64" s="27">
+      <c r="Y64" s="24">
         <f t="shared" si="132"/>
         <v>0.18857209957880355</v>
       </c>
-      <c r="Z64" s="27">
+      <c r="Z64" s="24">
         <f t="shared" ref="Z64:AC64" si="133">Z55/Z37</f>
         <v>7.4447229516503705E-2</v>
       </c>
-      <c r="AA64" s="27">
+      <c r="AA64" s="24">
         <f t="shared" si="133"/>
         <v>7.8167409509664498E-2</v>
       </c>
-      <c r="AB64" s="27">
+      <c r="AB64" s="24">
         <f t="shared" si="133"/>
-        <v>6.2073902204374129E-2</v>
-      </c>
-      <c r="AC64" s="27">
+        <v>8.1145808427332808E-2</v>
+      </c>
+      <c r="AC64" s="24">
         <f t="shared" si="133"/>
         <v>8.256576117082777E-2</v>
       </c>
-      <c r="AD64" s="27">
+      <c r="AD64" s="24">
         <f t="shared" si="132"/>
-        <v>6.2073902204374129E-2</v>
-      </c>
-      <c r="AE64" s="27">
+        <v>8.4255448695085125E-2</v>
+      </c>
+      <c r="AE64" s="24">
         <f t="shared" si="132"/>
         <v>0</v>
       </c>
-      <c r="AF64" s="27">
+      <c r="AF64" s="24">
         <f t="shared" si="132"/>
         <v>0</v>
       </c>
-      <c r="AG64" s="27">
+      <c r="AG64" s="24">
         <f t="shared" si="132"/>
         <v>0</v>
       </c>
-      <c r="AH64" s="27">
+      <c r="AH64" s="24">
         <f t="shared" si="132"/>
         <v>0</v>
       </c>
-      <c r="AI64" s="27">
+      <c r="AI64" s="24">
         <f t="shared" ref="AI64:AL64" si="134">AI55/AI37</f>
         <v>0</v>
       </c>
-      <c r="AJ64" s="27">
+      <c r="AJ64" s="24">
         <f t="shared" si="134"/>
         <v>0</v>
       </c>
-      <c r="AK64" s="27">
+      <c r="AK64" s="24">
         <f t="shared" si="134"/>
         <v>0</v>
       </c>
-      <c r="AL64" s="27">
+      <c r="AL64" s="24">
         <f t="shared" si="134"/>
         <v>0</v>
       </c>
@@ -10899,91 +10899,91 @@
       <c r="P65" s="14">
         <v>2045</v>
       </c>
-      <c r="Q65" s="26">
+      <c r="Q65" s="23">
         <f t="shared" si="121"/>
         <v>0.10518985801607006</v>
       </c>
-      <c r="R65" s="26">
+      <c r="R65" s="23">
         <f t="shared" si="121"/>
         <v>7.1273477648198635E-2</v>
       </c>
-      <c r="S65" s="26">
+      <c r="S65" s="23">
         <f t="shared" si="121"/>
         <v>0.12575751774983088</v>
       </c>
-      <c r="T65" s="26">
+      <c r="T65" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316924E-2</v>
       </c>
-      <c r="U65" s="26">
+      <c r="U65" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316868E-2</v>
       </c>
-      <c r="V65" s="26">
+      <c r="V65" s="23">
         <f t="shared" si="121"/>
         <v>0.16518751937583168</v>
       </c>
-      <c r="W65" s="26">
+      <c r="W65" s="23">
         <f t="shared" ref="W65:AH65" si="135">W56/W38</f>
         <v>8.5203970166686779E-2</v>
       </c>
-      <c r="X65" s="27">
+      <c r="X65" s="24">
         <f t="shared" si="135"/>
         <v>0.10389919717415484</v>
       </c>
-      <c r="Y65" s="27">
+      <c r="Y65" s="24">
         <f t="shared" si="135"/>
         <v>0.20434010167735797</v>
       </c>
-      <c r="Z65" s="27">
+      <c r="Z65" s="24">
         <f t="shared" ref="Z65:AC65" si="136">Z56/Z38</f>
         <v>7.4447229516503746E-2</v>
       </c>
-      <c r="AA65" s="27">
+      <c r="AA65" s="24">
         <f t="shared" si="136"/>
         <v>7.8167409509664457E-2</v>
       </c>
-      <c r="AB65" s="27">
+      <c r="AB65" s="24">
         <f t="shared" si="136"/>
-        <v>6.2073902204374219E-2</v>
-      </c>
-      <c r="AC65" s="27">
+        <v>8.1145808427332822E-2</v>
+      </c>
+      <c r="AC65" s="24">
         <f t="shared" si="136"/>
         <v>8.2565761170827756E-2</v>
       </c>
-      <c r="AD65" s="27">
+      <c r="AD65" s="24">
         <f t="shared" si="135"/>
-        <v>6.2073902204374219E-2</v>
-      </c>
-      <c r="AE65" s="27">
+        <v>8.4255448695085139E-2</v>
+      </c>
+      <c r="AE65" s="24">
         <f t="shared" si="135"/>
         <v>0</v>
       </c>
-      <c r="AF65" s="27">
+      <c r="AF65" s="24">
         <f t="shared" si="135"/>
         <v>0</v>
       </c>
-      <c r="AG65" s="27">
+      <c r="AG65" s="24">
         <f t="shared" si="135"/>
         <v>0</v>
       </c>
-      <c r="AH65" s="27">
+      <c r="AH65" s="24">
         <f t="shared" si="135"/>
         <v>0</v>
       </c>
-      <c r="AI65" s="27">
+      <c r="AI65" s="24">
         <f t="shared" ref="AI65:AL65" si="137">AI56/AI38</f>
         <v>0</v>
       </c>
-      <c r="AJ65" s="27">
+      <c r="AJ65" s="24">
         <f t="shared" si="137"/>
         <v>0</v>
       </c>
-      <c r="AK65" s="27">
+      <c r="AK65" s="24">
         <f t="shared" si="137"/>
         <v>0</v>
       </c>
-      <c r="AL65" s="27">
+      <c r="AL65" s="24">
         <f t="shared" si="137"/>
         <v>0</v>
       </c>
@@ -11019,103 +11019,97 @@
       <c r="P66" s="14">
         <v>2050</v>
       </c>
-      <c r="Q66" s="26">
+      <c r="Q66" s="23">
         <f t="shared" si="121"/>
         <v>0.10518985801607002</v>
       </c>
-      <c r="R66" s="26">
+      <c r="R66" s="23">
         <f t="shared" si="121"/>
         <v>7.9415665577240932E-2</v>
       </c>
-      <c r="S66" s="26">
+      <c r="S66" s="23">
         <f t="shared" si="121"/>
         <v>0.13571754371922554</v>
       </c>
-      <c r="T66" s="26">
+      <c r="T66" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316882E-2</v>
       </c>
-      <c r="U66" s="26">
+      <c r="U66" s="23">
         <f t="shared" si="121"/>
         <v>7.8895392089316993E-2</v>
       </c>
-      <c r="V66" s="26">
+      <c r="V66" s="23">
         <f t="shared" si="121"/>
         <v>0.16518751937583168</v>
       </c>
-      <c r="W66" s="26">
+      <c r="W66" s="23">
         <f t="shared" ref="W66:AH66" si="138">W57/W39</f>
         <v>8.5203970166686835E-2</v>
       </c>
-      <c r="X66" s="27">
+      <c r="X66" s="24">
         <f t="shared" si="138"/>
         <v>0.10389919717415486</v>
       </c>
-      <c r="Y66" s="27">
+      <c r="Y66" s="24">
         <f t="shared" si="138"/>
         <v>0.21704925001897787</v>
       </c>
-      <c r="Z66" s="27">
+      <c r="Z66" s="24">
         <f t="shared" ref="Z66:AC66" si="139">Z57/Z39</f>
         <v>7.4447229516503746E-2</v>
       </c>
-      <c r="AA66" s="27">
+      <c r="AA66" s="24">
         <f t="shared" si="139"/>
         <v>7.8167409509664498E-2</v>
       </c>
-      <c r="AB66" s="27">
+      <c r="AB66" s="24">
         <f t="shared" si="139"/>
-        <v>6.2073902204374233E-2</v>
-      </c>
-      <c r="AC66" s="27">
+        <v>8.1145808427332863E-2</v>
+      </c>
+      <c r="AC66" s="24">
         <f t="shared" si="139"/>
         <v>8.2565761170827853E-2</v>
       </c>
-      <c r="AD66" s="27">
+      <c r="AD66" s="24">
         <f t="shared" si="138"/>
-        <v>6.2073902204374233E-2</v>
-      </c>
-      <c r="AE66" s="27">
+        <v>8.4255448695085139E-2</v>
+      </c>
+      <c r="AE66" s="24">
         <f t="shared" si="138"/>
         <v>0</v>
       </c>
-      <c r="AF66" s="27">
+      <c r="AF66" s="24">
         <f t="shared" si="138"/>
         <v>0</v>
       </c>
-      <c r="AG66" s="27">
+      <c r="AG66" s="24">
         <f t="shared" si="138"/>
         <v>0</v>
       </c>
-      <c r="AH66" s="27">
+      <c r="AH66" s="24">
         <f t="shared" si="138"/>
         <v>0</v>
       </c>
-      <c r="AI66" s="27">
+      <c r="AI66" s="24">
         <f t="shared" ref="AI66:AL66" si="140">AI57/AI39</f>
         <v>0</v>
       </c>
-      <c r="AJ66" s="27">
+      <c r="AJ66" s="24">
         <f t="shared" si="140"/>
         <v>0</v>
       </c>
-      <c r="AK66" s="27">
+      <c r="AK66" s="24">
         <f t="shared" si="140"/>
         <v>0</v>
       </c>
-      <c r="AL66" s="27">
+      <c r="AL66" s="24">
         <f t="shared" si="140"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="H14:N14"/>
-    <mergeCell ref="H23:N23"/>
-    <mergeCell ref="H5:N5"/>
-    <mergeCell ref="P5:V5"/>
-    <mergeCell ref="P14:V14"/>
-    <mergeCell ref="P23:V23"/>
     <mergeCell ref="P32:V32"/>
     <mergeCell ref="P41:V41"/>
     <mergeCell ref="P59:V59"/>
@@ -11124,6 +11118,12 @@
     <mergeCell ref="H32:N32"/>
     <mergeCell ref="H59:N59"/>
     <mergeCell ref="P50:V50"/>
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P23:V23"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="I52:N57">
@@ -11201,16 +11201,16 @@
       <c r="G1" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="24" t="s">
+      <c r="L1" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="24"/>
-      <c r="S1" s="24"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -11626,16 +11626,16 @@
         <f>'Baseline Parameters'!G13</f>
         <v>231.99999999999997</v>
       </c>
-      <c r="L10" s="24" t="s">
+      <c r="L10" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="24"/>
-      <c r="S10" s="24"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
+      <c r="O10" s="27"/>
+      <c r="P10" s="27"/>
+      <c r="Q10" s="27"/>
+      <c r="R10" s="27"/>
+      <c r="S10" s="27"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -12059,16 +12059,16 @@
       <c r="H19" t="s">
         <v>33</v>
       </c>
-      <c r="L19" s="24" t="s">
+      <c r="L19" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="M19" s="24"/>
-      <c r="N19" s="24"/>
-      <c r="O19" s="24"/>
-      <c r="P19" s="24"/>
-      <c r="Q19" s="24"/>
-      <c r="R19" s="24"/>
-      <c r="S19" s="24"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="27"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="L20" t="s">
@@ -12465,16 +12465,16 @@
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="L28" s="24" t="s">
+      <c r="L28" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="M28" s="24"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="24"/>
-      <c r="P28" s="24"/>
-      <c r="Q28" s="24"/>
-      <c r="R28" s="24"/>
-      <c r="S28" s="24"/>
+      <c r="M28" s="27"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -12869,16 +12869,16 @@
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="L37" s="24" t="s">
+      <c r="L37" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="M37" s="24"/>
-      <c r="N37" s="24"/>
-      <c r="O37" s="24"/>
-      <c r="P37" s="24"/>
-      <c r="Q37" s="24"/>
-      <c r="R37" s="24"/>
-      <c r="S37" s="24"/>
+      <c r="M37" s="27"/>
+      <c r="N37" s="27"/>
+      <c r="O37" s="27"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="27"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="L38" t="s">
@@ -13105,16 +13105,16 @@
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="L46" s="24" t="s">
+      <c r="L46" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="M46" s="24"/>
-      <c r="N46" s="24"/>
-      <c r="O46" s="24"/>
-      <c r="P46" s="24"/>
-      <c r="Q46" s="24"/>
-      <c r="R46" s="24"/>
-      <c r="S46" s="24"/>
+      <c r="M46" s="27"/>
+      <c r="N46" s="27"/>
+      <c r="O46" s="27"/>
+      <c r="P46" s="27"/>
+      <c r="Q46" s="27"/>
+      <c r="R46" s="27"/>
+      <c r="S46" s="27"/>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="L47" t="s">

</xml_diff>

<commit_message>
get CDRIA 2050 up and running
</commit_message>
<xml_diff>
--- a/building_xml/inputs/cost_curves.xlsx
+++ b/building_xml/inputs/cost_curves.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\building_xml\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D201AA55-B4EC-4C6F-BAC6-55AE485B79E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4BB290-6440-4740-8F0A-8812C99E1014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="3120" windowWidth="28740" windowHeight="13845" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
+    <workbookView xWindow="60" yWindow="1635" windowWidth="28740" windowHeight="13845" activeTab="1" xr2:uid="{48B2FD56-5343-48F4-B77F-7F263F678783}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline Parameters" sheetId="1" r:id="rId1"/>
@@ -549,7 +549,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -565,12 +565,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -590,7 +584,7 @@
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -614,16 +608,15 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -5092,24 +5085,24 @@
       <c r="E5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="P5" s="23" t="s">
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="P5" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" s="23"/>
-      <c r="R5" s="23"/>
-      <c r="S5" s="23"/>
-      <c r="T5" s="23"/>
-      <c r="U5" s="23"/>
-      <c r="V5" s="23"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="24"/>
       <c r="AQ5">
         <v>2021</v>
       </c>
@@ -6093,24 +6086,24 @@
       <c r="E14" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="H14" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="P14" s="23" t="s">
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="M14" s="24"/>
+      <c r="N14" s="24"/>
+      <c r="P14" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="Q14" s="23"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="23"/>
-      <c r="T14" s="23"/>
-      <c r="U14" s="23"/>
-      <c r="V14" s="23"/>
+      <c r="Q14" s="24"/>
+      <c r="R14" s="24"/>
+      <c r="S14" s="24"/>
+      <c r="T14" s="24"/>
+      <c r="U14" s="24"/>
+      <c r="V14" s="24"/>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -6321,8 +6314,8 @@
       <c r="AH16" s="17">
         <v>1646.114674533992</v>
       </c>
-      <c r="AI16" s="26">
-        <v>0</v>
+      <c r="AI16" s="17">
+        <v>1646.114674533992</v>
       </c>
       <c r="AJ16" s="17">
         <v>1646.1138665824949</v>
@@ -6333,8 +6326,8 @@
       <c r="AL16" s="17">
         <v>1646.1156062384021</v>
       </c>
-      <c r="AM16" s="26">
-        <v>0</v>
+      <c r="AM16" s="17">
+        <v>1646.1156062384021</v>
       </c>
     </row>
     <row r="17" spans="1:39" x14ac:dyDescent="0.25">
@@ -6436,8 +6429,8 @@
       <c r="AH17" s="17">
         <v>5241.8056285483299</v>
       </c>
-      <c r="AI17" s="26">
-        <v>0</v>
+      <c r="AI17" s="17">
+        <v>5241.8056285483299</v>
       </c>
       <c r="AJ17" s="17">
         <v>3759.4553761544598</v>
@@ -6448,8 +6441,8 @@
       <c r="AL17" s="17">
         <v>6533.0783923066392</v>
       </c>
-      <c r="AM17" s="26">
-        <v>0</v>
+      <c r="AM17" s="17">
+        <v>6533.0783923066392</v>
       </c>
     </row>
     <row r="18" spans="1:39" x14ac:dyDescent="0.25">
@@ -6547,8 +6540,8 @@
       <c r="AH18" s="17">
         <v>14304.354015143419</v>
       </c>
-      <c r="AI18" s="26">
-        <v>0</v>
+      <c r="AI18" s="17">
+        <v>14304.354015143419</v>
       </c>
       <c r="AJ18" s="17">
         <v>9224.9095396813736</v>
@@ -6559,8 +6552,8 @@
       <c r="AL18" s="17">
         <v>22202.074115343152</v>
       </c>
-      <c r="AM18" s="26">
-        <v>0</v>
+      <c r="AM18" s="17">
+        <v>22202.074115343152</v>
       </c>
     </row>
     <row r="19" spans="1:39" x14ac:dyDescent="0.25">
@@ -6646,8 +6639,8 @@
       <c r="AH19" s="16">
         <v>0</v>
       </c>
-      <c r="AI19" s="26">
-        <v>0</v>
+      <c r="AI19" s="17">
+        <v>29472.199684563981</v>
       </c>
       <c r="AJ19" s="17">
         <v>23536.262965393158</v>
@@ -6658,8 +6651,8 @@
       <c r="AL19" s="16">
         <v>0</v>
       </c>
-      <c r="AM19" s="26">
-        <v>0</v>
+      <c r="AM19" s="17">
+        <v>56975.014646972704</v>
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.25">
@@ -6761,8 +6754,8 @@
       <c r="AH20" s="16">
         <v>0</v>
       </c>
-      <c r="AI20" s="26">
-        <v>0</v>
+      <c r="AI20" s="17">
+        <v>60683.475142986899</v>
       </c>
       <c r="AJ20" s="16">
         <v>0</v>
@@ -6773,8 +6766,8 @@
       <c r="AL20" s="16">
         <v>0</v>
       </c>
-      <c r="AM20" s="26">
-        <v>0</v>
+      <c r="AM20" s="17">
+        <v>146153.87333086965</v>
       </c>
     </row>
     <row r="21" spans="1:39" x14ac:dyDescent="0.25">
@@ -6876,8 +6869,8 @@
       <c r="AH21" s="16">
         <v>0</v>
       </c>
-      <c r="AI21" s="26">
-        <v>0</v>
+      <c r="AI21" s="17">
+        <v>124962.53985860199</v>
       </c>
       <c r="AJ21" s="16">
         <v>0</v>
@@ -6888,8 +6881,8 @@
       <c r="AL21" s="16">
         <v>0</v>
       </c>
-      <c r="AM21" s="26">
-        <v>0</v>
+      <c r="AM21" s="17">
+        <v>374916.94085709017</v>
       </c>
     </row>
     <row r="22" spans="1:39" x14ac:dyDescent="0.25">
@@ -6954,24 +6947,24 @@
         <f t="shared" si="33"/>
         <v>3512.6225095265308</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="23"/>
-      <c r="P23" s="23" t="s">
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24"/>
+      <c r="N23" s="24"/>
+      <c r="P23" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="Q23" s="23"/>
-      <c r="R23" s="23"/>
-      <c r="S23" s="23"/>
-      <c r="T23" s="23"/>
-      <c r="U23" s="23"/>
-      <c r="V23" s="23"/>
+      <c r="Q23" s="24"/>
+      <c r="R23" s="24"/>
+      <c r="S23" s="24"/>
+      <c r="T23" s="24"/>
+      <c r="U23" s="24"/>
+      <c r="V23" s="24"/>
     </row>
     <row r="24" spans="1:39" x14ac:dyDescent="0.25">
       <c r="H24" s="13" t="s">
@@ -7173,7 +7166,7 @@
       </c>
       <c r="AI25" s="10">
         <f t="shared" si="37"/>
-        <v>1719</v>
+        <v>9949.57337266996</v>
       </c>
       <c r="AJ25" s="10">
         <f t="shared" ref="AJ25:AM25" si="39">AJ4+AJ16*5</f>
@@ -7189,7 +7182,7 @@
       </c>
       <c r="AM25" s="10">
         <f t="shared" si="39"/>
-        <v>1719</v>
+        <v>9949.5780311920098</v>
       </c>
     </row>
     <row r="26" spans="1:39" x14ac:dyDescent="0.25">
@@ -7297,7 +7290,7 @@
       </c>
       <c r="AI26" s="10">
         <f t="shared" si="42"/>
-        <v>1719</v>
+        <v>36158.60151541161</v>
       </c>
       <c r="AJ26" s="10">
         <f t="shared" ref="AJ26:AM26" si="44">AJ25+AJ17*5</f>
@@ -7313,7 +7306,7 @@
       </c>
       <c r="AM26" s="10">
         <f t="shared" si="44"/>
-        <v>1719</v>
+        <v>42614.969992725208</v>
       </c>
     </row>
     <row r="27" spans="1:39" x14ac:dyDescent="0.25">
@@ -7421,7 +7414,7 @@
       </c>
       <c r="AI27" s="10">
         <f t="shared" si="47"/>
-        <v>1719</v>
+        <v>107680.3715911287</v>
       </c>
       <c r="AJ27" s="10">
         <f t="shared" ref="AJ27:AM27" si="49">AJ26+AJ18*5</f>
@@ -7437,7 +7430,7 @@
       </c>
       <c r="AM27" s="10">
         <f t="shared" si="49"/>
-        <v>1719</v>
+        <v>153625.34056944097</v>
       </c>
     </row>
     <row r="28" spans="1:39" x14ac:dyDescent="0.25">
@@ -7545,7 +7538,7 @@
       </c>
       <c r="AI28" s="10">
         <f t="shared" si="50"/>
-        <v>1719</v>
+        <v>255041.37001394859</v>
       </c>
       <c r="AJ28" s="10">
         <f t="shared" ref="AJ28:AM28" si="52">AJ27+AJ19*5</f>
@@ -7561,7 +7554,7 @@
       </c>
       <c r="AM28" s="10">
         <f t="shared" si="52"/>
-        <v>1719</v>
+        <v>438500.41380430449</v>
       </c>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
@@ -7669,7 +7662,7 @@
       </c>
       <c r="AI29" s="10">
         <f t="shared" si="53"/>
-        <v>1719</v>
+        <v>558458.74572888308</v>
       </c>
       <c r="AJ29" s="10">
         <f t="shared" ref="AJ29:AM29" si="55">AJ28+AJ20*5</f>
@@ -7685,7 +7678,7 @@
       </c>
       <c r="AM29" s="10">
         <f t="shared" si="55"/>
-        <v>1719</v>
+        <v>1169269.7804586529</v>
       </c>
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
@@ -7793,7 +7786,7 @@
       </c>
       <c r="AI30" s="10">
         <f t="shared" si="56"/>
-        <v>1719</v>
+        <v>1183271.4450218929</v>
       </c>
       <c r="AJ30" s="10">
         <f t="shared" ref="AJ30:AM30" si="58">AJ29+AJ21*5</f>
@@ -7809,7 +7802,7 @@
       </c>
       <c r="AM30" s="10">
         <f t="shared" si="58"/>
-        <v>1719</v>
+        <v>3043854.4847441036</v>
       </c>
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
@@ -7829,24 +7822,24 @@
       <c r="V31" s="10"/>
     </row>
     <row r="32" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="H32" s="24" t="s">
+      <c r="H32" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="I32" s="24"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="24"/>
-      <c r="L32" s="24"/>
-      <c r="M32" s="24"/>
-      <c r="N32" s="24"/>
-      <c r="P32" s="24" t="s">
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
+      <c r="P32" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="Q32" s="24"/>
-      <c r="R32" s="24"/>
-      <c r="S32" s="24"/>
-      <c r="T32" s="24"/>
-      <c r="U32" s="24"/>
-      <c r="V32" s="24"/>
+      <c r="Q32" s="23"/>
+      <c r="R32" s="23"/>
+      <c r="S32" s="23"/>
+      <c r="T32" s="23"/>
+      <c r="U32" s="23"/>
+      <c r="V32" s="23"/>
     </row>
     <row r="33" spans="8:39" x14ac:dyDescent="0.25">
       <c r="H33" s="14" t="s">
@@ -8704,24 +8697,24 @@
       <c r="V40" s="10"/>
     </row>
     <row r="41" spans="8:39" x14ac:dyDescent="0.25">
-      <c r="H41" s="24" t="s">
+      <c r="H41" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="I41" s="24"/>
-      <c r="J41" s="24"/>
-      <c r="K41" s="24"/>
-      <c r="L41" s="24"/>
-      <c r="M41" s="24"/>
-      <c r="N41" s="24"/>
-      <c r="P41" s="24" t="s">
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="P41" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="Q41" s="24"/>
-      <c r="R41" s="24"/>
-      <c r="S41" s="24"/>
-      <c r="T41" s="24"/>
-      <c r="U41" s="24"/>
-      <c r="V41" s="24"/>
+      <c r="Q41" s="23"/>
+      <c r="R41" s="23"/>
+      <c r="S41" s="23"/>
+      <c r="T41" s="23"/>
+      <c r="U41" s="23"/>
+      <c r="V41" s="23"/>
       <c r="Z41" s="18"/>
       <c r="AA41" s="18"/>
       <c r="AB41" s="18"/>
@@ -8932,7 +8925,7 @@
       </c>
       <c r="AI43" s="10">
         <f t="shared" si="65"/>
-        <v>360.50516023732143</v>
+        <v>338.12648693431197</v>
       </c>
       <c r="AJ43" s="10">
         <f t="shared" ref="AJ43:AM43" si="67">AJ7*AJ25^AJ$3</f>
@@ -8948,7 +8941,7 @@
       </c>
       <c r="AM43" s="10">
         <f t="shared" si="67"/>
-        <v>360.50516023732143</v>
+        <v>338.12648115580498</v>
       </c>
     </row>
     <row r="44" spans="8:39" x14ac:dyDescent="0.25">
@@ -9056,7 +9049,7 @@
       </c>
       <c r="AI44" s="10">
         <f t="shared" si="68"/>
-        <v>296.81654796345282</v>
+        <v>265.58341747860783</v>
       </c>
       <c r="AJ44" s="10">
         <f t="shared" ref="AJ44:AM44" si="70">AJ8*AJ26^AJ$3</f>
@@ -9072,7 +9065,7 @@
       </c>
       <c r="AM44" s="10">
         <f t="shared" si="70"/>
-        <v>296.81654796345282</v>
+        <v>263.9955823418797</v>
       </c>
     </row>
     <row r="45" spans="8:39" x14ac:dyDescent="0.25">
@@ -9180,7 +9173,7 @@
       </c>
       <c r="AI45" s="10">
         <f t="shared" si="71"/>
-        <v>220.80894613326407</v>
+        <v>189.85902687274336</v>
       </c>
       <c r="AJ45" s="10">
         <f t="shared" ref="AJ45:AM45" si="73">AJ9*AJ27^AJ$3</f>
@@ -9196,7 +9189,7 @@
       </c>
       <c r="AM45" s="10">
         <f t="shared" si="73"/>
-        <v>220.80894613326407</v>
+        <v>187.41240770657851</v>
       </c>
     </row>
     <row r="46" spans="8:39" x14ac:dyDescent="0.25">
@@ -9304,7 +9297,7 @@
       </c>
       <c r="AI46" s="10">
         <f t="shared" si="74"/>
-        <v>202.50547416626196</v>
+        <v>168.72640337213605</v>
       </c>
       <c r="AJ46" s="10">
         <f t="shared" ref="AJ46:AM46" si="76">AJ10*AJ28^AJ$3</f>
@@ -9320,7 +9313,7 @@
       </c>
       <c r="AM46" s="10">
         <f t="shared" si="76"/>
-        <v>202.50547416626196</v>
+        <v>165.42168179653365</v>
       </c>
     </row>
     <row r="47" spans="8:39" x14ac:dyDescent="0.25">
@@ -9428,7 +9421,7 @@
       </c>
       <c r="AI47" s="10">
         <f t="shared" si="77"/>
-        <v>184.65112037257458</v>
+        <v>149.51141149398137</v>
       </c>
       <c r="AJ47" s="10">
         <f t="shared" ref="AJ47:AM47" si="79">AJ11*AJ29^AJ$3</f>
@@ -9444,7 +9437,7 @@
       </c>
       <c r="AM47" s="10">
         <f t="shared" si="79"/>
-        <v>184.65112037257458</v>
+        <v>145.53271421311371</v>
       </c>
     </row>
     <row r="48" spans="8:39" x14ac:dyDescent="0.25">
@@ -9552,7 +9545,7 @@
       </c>
       <c r="AI48" s="10">
         <f t="shared" si="80"/>
-        <v>172.93379856211703</v>
+        <v>136.23850538396292</v>
       </c>
       <c r="AJ48" s="10">
         <f t="shared" ref="AJ48:AM48" si="82">AJ12*AJ30^AJ$3</f>
@@ -9568,7 +9561,7 @@
       </c>
       <c r="AM48" s="10">
         <f t="shared" si="82"/>
-        <v>172.93379856211703</v>
+        <v>131.62017947979558</v>
       </c>
     </row>
     <row r="49" spans="8:39" x14ac:dyDescent="0.25">
@@ -9588,24 +9581,24 @@
       <c r="V49" s="10"/>
     </row>
     <row r="50" spans="8:39" x14ac:dyDescent="0.25">
-      <c r="H50" s="24" t="s">
+      <c r="H50" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="I50" s="24"/>
-      <c r="J50" s="24"/>
-      <c r="K50" s="24"/>
-      <c r="L50" s="24"/>
-      <c r="M50" s="24"/>
-      <c r="N50" s="24"/>
-      <c r="P50" s="24" t="s">
+      <c r="I50" s="23"/>
+      <c r="J50" s="23"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
+      <c r="M50" s="23"/>
+      <c r="N50" s="23"/>
+      <c r="P50" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="Q50" s="24"/>
-      <c r="R50" s="24"/>
-      <c r="S50" s="24"/>
-      <c r="T50" s="24"/>
-      <c r="U50" s="24"/>
-      <c r="V50" s="24"/>
+      <c r="Q50" s="23"/>
+      <c r="R50" s="23"/>
+      <c r="S50" s="23"/>
+      <c r="T50" s="23"/>
+      <c r="U50" s="23"/>
+      <c r="V50" s="23"/>
     </row>
     <row r="51" spans="8:39" x14ac:dyDescent="0.25">
       <c r="H51" s="14" t="s">
@@ -9807,7 +9800,7 @@
       </c>
       <c r="AI52" s="10">
         <f t="shared" si="85"/>
-        <v>0</v>
+        <v>22.378673303009464</v>
       </c>
       <c r="AJ52" s="10">
         <f t="shared" ref="AJ52:AM52" si="87">AJ34-AJ43</f>
@@ -9823,7 +9816,7 @@
       </c>
       <c r="AM52" s="10">
         <f t="shared" si="87"/>
-        <v>0</v>
+        <v>22.378679081516452</v>
       </c>
     </row>
     <row r="53" spans="8:39" x14ac:dyDescent="0.25">
@@ -9931,7 +9924,7 @@
       </c>
       <c r="AI53" s="10">
         <f t="shared" si="90"/>
-        <v>0</v>
+        <v>31.233130484844992</v>
       </c>
       <c r="AJ53" s="10">
         <f t="shared" ref="AJ53:AM53" si="92">AJ35-AJ44</f>
@@ -9947,7 +9940,7 @@
       </c>
       <c r="AM53" s="10">
         <f t="shared" si="92"/>
-        <v>0</v>
+        <v>32.820965621573123</v>
       </c>
     </row>
     <row r="54" spans="8:39" x14ac:dyDescent="0.25">
@@ -10055,7 +10048,7 @@
       </c>
       <c r="AI54" s="10">
         <f t="shared" si="94"/>
-        <v>0</v>
+        <v>30.949919260520744</v>
       </c>
       <c r="AJ54" s="10">
         <f t="shared" ref="AJ54:AM54" si="96">AJ36-AJ45</f>
@@ -10071,7 +10064,7 @@
       </c>
       <c r="AM54" s="10">
         <f t="shared" si="96"/>
-        <v>0</v>
+        <v>33.396538426685595</v>
       </c>
     </row>
     <row r="55" spans="8:39" x14ac:dyDescent="0.25">
@@ -10179,7 +10172,7 @@
       </c>
       <c r="AI55" s="10">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>33.779070794125914</v>
       </c>
       <c r="AJ55" s="10">
         <f t="shared" ref="AJ55:AM55" si="100">AJ37-AJ46</f>
@@ -10195,7 +10188,7 @@
       </c>
       <c r="AM55" s="10">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>37.083792369728314</v>
       </c>
     </row>
     <row r="56" spans="8:39" x14ac:dyDescent="0.25">
@@ -10303,7 +10296,7 @@
       </c>
       <c r="AI56" s="10">
         <f t="shared" si="102"/>
-        <v>0</v>
+        <v>35.139708878593211</v>
       </c>
       <c r="AJ56" s="10">
         <f t="shared" ref="AJ56:AM56" si="104">AJ38-AJ47</f>
@@ -10319,7 +10312,7 @@
       </c>
       <c r="AM56" s="10">
         <f t="shared" si="104"/>
-        <v>0</v>
+        <v>39.118406159460875</v>
       </c>
     </row>
     <row r="57" spans="8:39" x14ac:dyDescent="0.25">
@@ -10427,7 +10420,7 @@
       </c>
       <c r="AI57" s="10">
         <f t="shared" si="106"/>
-        <v>0</v>
+        <v>36.695293178154117</v>
       </c>
       <c r="AJ57" s="10">
         <f t="shared" ref="AJ57:AM57" si="108">AJ39-AJ48</f>
@@ -10443,31 +10436,31 @@
       </c>
       <c r="AM57" s="10">
         <f t="shared" si="108"/>
-        <v>0</v>
+        <v>41.313619082321452</v>
       </c>
     </row>
     <row r="58" spans="8:39" x14ac:dyDescent="0.25">
       <c r="P58" s="13"/>
     </row>
     <row r="59" spans="8:39" x14ac:dyDescent="0.25">
-      <c r="H59" s="24" t="s">
+      <c r="H59" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="I59" s="24"/>
-      <c r="J59" s="24"/>
-      <c r="K59" s="24"/>
-      <c r="L59" s="24"/>
-      <c r="M59" s="24"/>
-      <c r="N59" s="24"/>
-      <c r="P59" s="24" t="s">
+      <c r="I59" s="23"/>
+      <c r="J59" s="23"/>
+      <c r="K59" s="23"/>
+      <c r="L59" s="23"/>
+      <c r="M59" s="23"/>
+      <c r="N59" s="23"/>
+      <c r="P59" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="Q59" s="24"/>
-      <c r="R59" s="24"/>
-      <c r="S59" s="24"/>
-      <c r="T59" s="24"/>
-      <c r="U59" s="24"/>
-      <c r="V59" s="24"/>
+      <c r="Q59" s="23"/>
+      <c r="R59" s="23"/>
+      <c r="S59" s="23"/>
+      <c r="T59" s="23"/>
+      <c r="U59" s="23"/>
+      <c r="V59" s="23"/>
     </row>
     <row r="60" spans="8:39" x14ac:dyDescent="0.25">
       <c r="H60" s="14" t="s">
@@ -10669,7 +10662,7 @@
       </c>
       <c r="AI61" s="21">
         <f t="shared" si="111"/>
-        <v>0</v>
+        <v>6.2075875108909752E-2</v>
       </c>
       <c r="AJ61" s="21">
         <f t="shared" ref="AJ61:AM61" si="113">AJ52/AJ34</f>
@@ -10685,7 +10678,7 @@
       </c>
       <c r="AM61" s="21">
         <f t="shared" si="113"/>
-        <v>0</v>
+        <v>6.2075891137825912E-2</v>
       </c>
     </row>
     <row r="62" spans="8:39" x14ac:dyDescent="0.25">
@@ -10793,7 +10786,7 @@
       </c>
       <c r="AI62" s="21">
         <f t="shared" si="115"/>
-        <v>0</v>
+        <v>0.1052270525317569</v>
       </c>
       <c r="AJ62" s="21">
         <f t="shared" ref="AJ62:AM62" si="117">AJ53/AJ35</f>
@@ -10809,7 +10802,7 @@
       </c>
       <c r="AM62" s="21">
         <f t="shared" si="117"/>
-        <v>0</v>
+        <v>0.11057660311316062</v>
       </c>
     </row>
     <row r="63" spans="8:39" x14ac:dyDescent="0.25">
@@ -10917,7 +10910,7 @@
       </c>
       <c r="AI63" s="21">
         <f t="shared" si="118"/>
-        <v>0</v>
+        <v>0.14016605668613463</v>
       </c>
       <c r="AJ63" s="21">
         <f t="shared" ref="AJ63:AM63" si="120">AJ54/AJ36</f>
@@ -10933,7 +10926,7 @@
       </c>
       <c r="AM63" s="21">
         <f t="shared" si="120"/>
-        <v>0</v>
+        <v>0.15124631049382342</v>
       </c>
     </row>
     <row r="64" spans="8:39" x14ac:dyDescent="0.25">
@@ -11041,7 +11034,7 @@
       </c>
       <c r="AI64" s="21">
         <f t="shared" si="121"/>
-        <v>0</v>
+        <v>0.16680571689826257</v>
       </c>
       <c r="AJ64" s="21">
         <f t="shared" ref="AJ64:AM64" si="123">AJ55/AJ37</f>
@@ -11057,7 +11050,7 @@
       </c>
       <c r="AM64" s="21">
         <f t="shared" si="123"/>
-        <v>0</v>
+        <v>0.18312488846243047</v>
       </c>
     </row>
     <row r="65" spans="8:39" x14ac:dyDescent="0.25">
@@ -11165,7 +11158,7 @@
       </c>
       <c r="AI65" s="21">
         <f t="shared" si="124"/>
-        <v>0</v>
+        <v>0.1903032530086525</v>
       </c>
       <c r="AJ65" s="21">
         <f t="shared" ref="AJ65:AM65" si="126">AJ56/AJ38</f>
@@ -11181,7 +11174,7 @@
       </c>
       <c r="AM65" s="21">
         <f t="shared" si="126"/>
-        <v>0</v>
+        <v>0.21185035910169847</v>
       </c>
     </row>
     <row r="66" spans="8:39" x14ac:dyDescent="0.25">
@@ -11289,7 +11282,7 @@
       </c>
       <c r="AI66" s="21">
         <f t="shared" si="127"/>
-        <v>0</v>
+        <v>0.21219272047027485</v>
       </c>
       <c r="AJ66" s="21">
         <f t="shared" ref="AJ66:AM66" si="129">AJ57/AJ39</f>
@@ -11305,11 +11298,17 @@
       </c>
       <c r="AM66" s="21">
         <f t="shared" si="129"/>
-        <v>0</v>
+        <v>0.23889846534239972</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="H14:N14"/>
+    <mergeCell ref="H23:N23"/>
+    <mergeCell ref="H5:N5"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P23:V23"/>
     <mergeCell ref="P32:V32"/>
     <mergeCell ref="P41:V41"/>
     <mergeCell ref="P59:V59"/>
@@ -11318,12 +11317,6 @@
     <mergeCell ref="H32:N32"/>
     <mergeCell ref="H59:N59"/>
     <mergeCell ref="P50:V50"/>
-    <mergeCell ref="H14:N14"/>
-    <mergeCell ref="H23:N23"/>
-    <mergeCell ref="H5:N5"/>
-    <mergeCell ref="P5:V5"/>
-    <mergeCell ref="P14:V14"/>
-    <mergeCell ref="P23:V23"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="I52:N57">

</xml_diff>